<commit_message>
feat: made it optionnal to render and save all plots of simulations runs
</commit_message>
<xml_diff>
--- a/test_alldata.xlsx
+++ b/test_alldata.xlsx
@@ -516,25 +516,25 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>7000</v>
+        <v>1500</v>
       </c>
       <c r="H2" t="n">
-        <v>-300</v>
+        <v>-200</v>
       </c>
       <c r="I2" t="n">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>524.6392765801286</v>
+        <v>690.0868864990008</v>
       </c>
       <c r="L2" t="n">
-        <v>5479.23</v>
+        <v>1250.59</v>
       </c>
       <c r="M2" t="n">
-        <v>-203.85</v>
+        <v>-169.19</v>
       </c>
     </row>
     <row r="3">
@@ -561,25 +561,25 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>4000</v>
+        <v>9000</v>
       </c>
       <c r="H3" t="n">
-        <v>-750</v>
+        <v>-500</v>
       </c>
       <c r="I3" t="n">
-        <v>300</v>
+        <v>850</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>337.0367045574487</v>
+        <v>886.8022335987732</v>
       </c>
       <c r="L3" t="n">
-        <v>2425.03</v>
+        <v>7737.95</v>
       </c>
       <c r="M3" t="n">
-        <v>-404.23</v>
+        <v>-422.73</v>
       </c>
     </row>
     <row r="4">
@@ -606,25 +606,25 @@
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>20000</v>
+        <v>3000</v>
       </c>
       <c r="H4" t="n">
-        <v>-500</v>
+        <v>-750</v>
       </c>
       <c r="I4" t="n">
-        <v>100</v>
+        <v>650</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>147.8003722664622</v>
+        <v>664.2800545331141</v>
       </c>
       <c r="L4" t="n">
-        <v>4314.32</v>
+        <v>2477.98</v>
       </c>
       <c r="M4" t="n">
-        <v>-46.4</v>
+        <v>-627.59</v>
       </c>
     </row>
     <row r="5">
@@ -651,25 +651,25 @@
         <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>18000</v>
+        <v>1300</v>
       </c>
       <c r="H5" t="n">
         <v>-450</v>
       </c>
       <c r="I5" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J5" t="n">
         <v>0.5</v>
       </c>
       <c r="K5" t="n">
-        <v>147.8003722664622</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L5" t="n">
-        <v>4084.64</v>
+        <v>742.2</v>
       </c>
       <c r="M5" t="n">
-        <v>-60.96</v>
+        <v>-179.68</v>
       </c>
     </row>
     <row r="6">
@@ -696,25 +696,25 @@
         <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>10000</v>
+        <v>1400</v>
       </c>
       <c r="H6" t="n">
-        <v>-550</v>
+        <v>-300</v>
       </c>
       <c r="I6" t="n">
-        <v>750</v>
+        <v>450</v>
       </c>
       <c r="J6" t="n">
         <v>0.5</v>
       </c>
       <c r="K6" t="n">
-        <v>809.5359789800231</v>
+        <v>453.1473605746647</v>
       </c>
       <c r="L6" t="n">
-        <v>8168.09</v>
+        <v>1098.21</v>
       </c>
       <c r="M6" t="n">
-        <v>-426.5</v>
+        <v>-215.3</v>
       </c>
     </row>
     <row r="7">
@@ -741,25 +741,25 @@
         <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>14000</v>
+        <v>15000</v>
       </c>
       <c r="H7" t="n">
         <v>-800</v>
       </c>
       <c r="I7" t="n">
-        <v>800</v>
+        <v>200</v>
       </c>
       <c r="J7" t="n">
         <v>0.5</v>
       </c>
       <c r="K7" t="n">
-        <v>828.2097749496145</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L7" t="n">
-        <v>11844.56</v>
+        <v>7609.94</v>
       </c>
       <c r="M7" t="n">
-        <v>-686.59</v>
+        <v>-337.52</v>
       </c>
     </row>
     <row r="8">
@@ -786,25 +786,25 @@
         <v>6</v>
       </c>
       <c r="G8" t="n">
-        <v>7000</v>
+        <v>5000</v>
       </c>
       <c r="H8" t="n">
-        <v>-350</v>
+        <v>-50</v>
       </c>
       <c r="I8" t="n">
-        <v>200</v>
+        <v>450</v>
       </c>
       <c r="J8" t="n">
         <v>0.5</v>
       </c>
       <c r="K8" t="n">
-        <v>247.317326764409</v>
+        <v>467.3858153828035</v>
       </c>
       <c r="L8" t="n">
-        <v>3762.26</v>
+        <v>3890.06</v>
       </c>
       <c r="M8" t="n">
-        <v>-131.26</v>
+        <v>-10.76</v>
       </c>
     </row>
     <row r="9">
@@ -831,25 +831,25 @@
         <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="H9" t="n">
-        <v>-750</v>
+        <v>-700</v>
       </c>
       <c r="I9" t="n">
-        <v>750</v>
+        <v>100</v>
       </c>
       <c r="J9" t="n">
         <v>0.5</v>
       </c>
       <c r="K9" t="n">
-        <v>711.9008645709257</v>
+        <v>132.1966717950337</v>
       </c>
       <c r="L9" t="n">
-        <v>1042.47</v>
+        <v>275.32</v>
       </c>
       <c r="M9" t="n">
-        <v>-685.45</v>
+        <v>-36.72</v>
       </c>
     </row>
     <row r="10">
@@ -876,25 +876,25 @@
         <v>8</v>
       </c>
       <c r="G10" t="n">
-        <v>15000</v>
+        <v>8000</v>
       </c>
       <c r="H10" t="n">
-        <v>-850</v>
+        <v>-50</v>
       </c>
       <c r="I10" t="n">
-        <v>650</v>
+        <v>600</v>
       </c>
       <c r="J10" t="n">
         <v>0.5</v>
       </c>
       <c r="K10" t="n">
-        <v>690.0868864990008</v>
+        <v>630.5379376106623</v>
       </c>
       <c r="L10" t="n">
-        <v>12183.95</v>
+        <v>6505.52</v>
       </c>
       <c r="M10" t="n">
-        <v>-682.73</v>
+        <v>-24.52</v>
       </c>
     </row>
     <row r="11">
@@ -921,25 +921,25 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>6000</v>
+        <v>1400</v>
       </c>
       <c r="H11" t="n">
-        <v>-310</v>
+        <v>-210</v>
       </c>
       <c r="I11" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="J11" t="n">
         <v>0.5</v>
       </c>
       <c r="K11" t="n">
-        <v>448.3007253924136</v>
+        <v>594.8850230776515</v>
       </c>
       <c r="L11" t="n">
-        <v>4188.41</v>
+        <v>1129.87</v>
       </c>
       <c r="M11" t="n">
-        <v>-195.96</v>
+        <v>-171.7</v>
       </c>
     </row>
     <row r="12">
@@ -966,25 +966,25 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>3000</v>
+        <v>8000</v>
       </c>
       <c r="H12" t="n">
-        <v>-850</v>
+        <v>-600</v>
       </c>
       <c r="I12" t="n">
-        <v>290</v>
+        <v>750</v>
       </c>
       <c r="J12" t="n">
         <v>0.5</v>
       </c>
       <c r="K12" t="n">
-        <v>302.9006275609877</v>
+        <v>782.0860573996538</v>
       </c>
       <c r="L12" t="n">
-        <v>1974.98</v>
+        <v>6732.04</v>
       </c>
       <c r="M12" t="n">
-        <v>-507.61</v>
+        <v>-501.94</v>
       </c>
     </row>
     <row r="13">
@@ -1011,25 +1011,25 @@
         <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>19000</v>
+        <v>2900</v>
       </c>
       <c r="H13" t="n">
-        <v>-600</v>
+        <v>-850</v>
       </c>
       <c r="I13" t="n">
-        <v>90</v>
+        <v>550</v>
       </c>
       <c r="J13" t="n">
         <v>0.5</v>
       </c>
       <c r="K13" t="n">
-        <v>147.8003722664622</v>
+        <v>560.8629784593642</v>
       </c>
       <c r="L13" t="n">
-        <v>3360.51</v>
+        <v>2323.71</v>
       </c>
       <c r="M13" t="n">
-        <v>3.48</v>
+        <v>-676.1799999999999</v>
       </c>
     </row>
     <row r="14">
@@ -1056,25 +1056,25 @@
         <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>17000</v>
+        <v>1200</v>
       </c>
       <c r="H14" t="n">
         <v>-550</v>
       </c>
       <c r="I14" t="n">
-        <v>90</v>
+        <v>190</v>
       </c>
       <c r="J14" t="n">
         <v>0.5</v>
       </c>
       <c r="K14" t="n">
-        <v>147.8003722664622</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L14" t="n">
-        <v>3019.34</v>
+        <v>796.64</v>
       </c>
       <c r="M14" t="n">
-        <v>70.86</v>
+        <v>-305.79</v>
       </c>
     </row>
     <row r="15">
@@ -1101,25 +1101,25 @@
         <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>9000</v>
+        <v>1300</v>
       </c>
       <c r="H15" t="n">
-        <v>-650</v>
+        <v>-310</v>
       </c>
       <c r="I15" t="n">
-        <v>650</v>
+        <v>350</v>
       </c>
       <c r="J15" t="n">
         <v>0.5</v>
       </c>
       <c r="K15" t="n">
-        <v>680.5240193355573</v>
+        <v>362.0354958462345</v>
       </c>
       <c r="L15" t="n">
-        <v>7485.93</v>
+        <v>1033.02</v>
       </c>
       <c r="M15" t="n">
-        <v>-528.28</v>
+        <v>-223.68</v>
       </c>
     </row>
     <row r="16">
@@ -1146,25 +1146,25 @@
         <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>13000</v>
+        <v>14000</v>
       </c>
       <c r="H16" t="n">
         <v>-900</v>
       </c>
       <c r="I16" t="n">
-        <v>700</v>
+        <v>190</v>
       </c>
       <c r="J16" t="n">
         <v>0.5</v>
       </c>
       <c r="K16" t="n">
-        <v>721.0477175625025</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L16" t="n">
-        <v>10941.3</v>
+        <v>6371.95</v>
       </c>
       <c r="M16" t="n">
-        <v>-755.16</v>
+        <v>-312.87</v>
       </c>
     </row>
     <row r="17">
@@ -1191,25 +1191,25 @@
         <v>6</v>
       </c>
       <c r="G17" t="n">
-        <v>6000</v>
+        <v>4000</v>
       </c>
       <c r="H17" t="n">
-        <v>-450</v>
+        <v>-60</v>
       </c>
       <c r="I17" t="n">
-        <v>190</v>
+        <v>350</v>
       </c>
       <c r="J17" t="n">
         <v>0.5</v>
       </c>
       <c r="K17" t="n">
-        <v>219.2233794389425</v>
+        <v>379.7060313951988</v>
       </c>
       <c r="L17" t="n">
-        <v>3042.32</v>
+        <v>2723.07</v>
       </c>
       <c r="M17" t="n">
-        <v>-138.1</v>
+        <v>-4.43</v>
       </c>
     </row>
     <row r="18">
@@ -1236,25 +1236,25 @@
         <v>7</v>
       </c>
       <c r="G18" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="H18" t="n">
-        <v>-850</v>
+        <v>-800</v>
       </c>
       <c r="I18" t="n">
-        <v>650</v>
+        <v>90</v>
       </c>
       <c r="J18" t="n">
         <v>0.5</v>
       </c>
       <c r="K18" t="n">
-        <v>644.2468865272003</v>
+        <v>93.4771630765607</v>
       </c>
       <c r="L18" t="n">
-        <v>929.6799999999999</v>
+        <v>156.34</v>
       </c>
       <c r="M18" t="n">
-        <v>-724.3099999999999</v>
+        <v>30.15</v>
       </c>
     </row>
     <row r="19">
@@ -1281,25 +1281,25 @@
         <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>14000</v>
+        <v>7000</v>
       </c>
       <c r="H19" t="n">
-        <v>-950</v>
+        <v>-60</v>
       </c>
       <c r="I19" t="n">
-        <v>550</v>
+        <v>500</v>
       </c>
       <c r="J19" t="n">
         <v>0.5</v>
       </c>
       <c r="K19" t="n">
-        <v>568.5993850006796</v>
+        <v>541.0381969548956</v>
       </c>
       <c r="L19" t="n">
-        <v>11549.54</v>
+        <v>5384.7</v>
       </c>
       <c r="M19" t="n">
-        <v>-767.12</v>
+        <v>-22.4</v>
       </c>
     </row>
     <row r="20">
@@ -1326,25 +1326,25 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>5000.980614945375</v>
+        <v>1304.308177915139</v>
       </c>
       <c r="H20" t="n">
-        <v>-300.0000050428039</v>
+        <v>-200.0000043811628</v>
       </c>
       <c r="I20" t="n">
-        <v>300.8157539533038</v>
+        <v>500.1668719689348</v>
       </c>
       <c r="J20" t="n">
         <v>0.5</v>
       </c>
       <c r="K20" t="n">
-        <v>316.996482935824</v>
+        <v>499.0314924731653</v>
       </c>
       <c r="L20" t="n">
-        <v>3533.02</v>
+        <v>1052</v>
       </c>
       <c r="M20" t="n">
-        <v>-171.47</v>
+        <v>-144.76</v>
       </c>
     </row>
     <row r="21">
@@ -1371,25 +1371,25 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>2009.708301577336</v>
+        <v>7000.864222667794</v>
       </c>
       <c r="H21" t="n">
-        <v>-750.0000146728457</v>
+        <v>-500.0000199834465</v>
       </c>
       <c r="I21" t="n">
-        <v>281.5299267767371</v>
+        <v>650.2558891142786</v>
       </c>
       <c r="J21" t="n">
         <v>0.5</v>
       </c>
       <c r="K21" t="n">
-        <v>288.1159665134826</v>
+        <v>612.9707503006996</v>
       </c>
       <c r="L21" t="n">
-        <v>1363.59</v>
+        <v>6080.12</v>
       </c>
       <c r="M21" t="n">
-        <v>-480.78</v>
+        <v>-438.39</v>
       </c>
     </row>
     <row r="22">
@@ -1416,25 +1416,25 @@
         <v>2</v>
       </c>
       <c r="G22" t="n">
-        <v>18000.71088305247</v>
+        <v>2801.425034508065</v>
       </c>
       <c r="H22" t="n">
-        <v>-500.0011110633947</v>
+        <v>-750.0000091967432</v>
       </c>
       <c r="I22" t="n">
-        <v>99.886349042757</v>
+        <v>450.6663716487579</v>
       </c>
       <c r="J22" t="n">
         <v>0.5</v>
       </c>
       <c r="K22" t="n">
-        <v>147.8003722664622</v>
+        <v>423.2358566393677</v>
       </c>
       <c r="L22" t="n">
-        <v>3856.29</v>
+        <v>2305.51</v>
       </c>
       <c r="M22" t="n">
-        <v>23.7</v>
+        <v>-639.16</v>
       </c>
     </row>
     <row r="23">
@@ -1461,25 +1461,25 @@
         <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>16000.85609850038</v>
+        <v>1189.307684908337</v>
       </c>
       <c r="H23" t="n">
-        <v>-450.000467886208</v>
+        <v>-450.0000322372096</v>
       </c>
       <c r="I23" t="n">
-        <v>99.88018186571199</v>
+        <v>199.5654131250215</v>
       </c>
       <c r="J23" t="n">
         <v>0.5</v>
       </c>
       <c r="K23" t="n">
-        <v>147.8003722664622</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L23" t="n">
-        <v>3438.72</v>
+        <v>690.1799999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>36.15</v>
+        <v>-227.71</v>
       </c>
     </row>
     <row r="24">
@@ -1506,25 +1506,25 @@
         <v>4</v>
       </c>
       <c r="G24" t="n">
-        <v>8000.779672403452</v>
+        <v>1208.908155782029</v>
       </c>
       <c r="H24" t="n">
-        <v>-550.0000199294692</v>
+        <v>-300.0000028526401</v>
       </c>
       <c r="I24" t="n">
-        <v>550.3410638478135</v>
+        <v>251.0384767784776</v>
       </c>
       <c r="J24" t="n">
         <v>0.5</v>
       </c>
       <c r="K24" t="n">
-        <v>591.2014890658488</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L24" t="n">
-        <v>6141.19</v>
+        <v>837.78</v>
       </c>
       <c r="M24" t="n">
-        <v>-415.05</v>
+        <v>-209.3</v>
       </c>
     </row>
     <row r="25">
@@ -1551,25 +1551,25 @@
         <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>12000.54380404797</v>
+        <v>13000.71582931089</v>
       </c>
       <c r="H25" t="n">
-        <v>-800.0000115029715</v>
+        <v>-800.0000257079257</v>
       </c>
       <c r="I25" t="n">
-        <v>600.49409423489</v>
+        <v>197.3517214033029</v>
       </c>
       <c r="J25" t="n">
         <v>0.5</v>
       </c>
       <c r="K25" t="n">
-        <v>640.847143078262</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L25" t="n">
-        <v>9613.32</v>
+        <v>6309.48</v>
       </c>
       <c r="M25" t="n">
-        <v>-612.9</v>
+        <v>-315.02</v>
       </c>
     </row>
     <row r="26">
@@ -1596,25 +1596,25 @@
         <v>6</v>
       </c>
       <c r="G26" t="n">
-        <v>5001.421067861686</v>
+        <v>3000.76717759145</v>
       </c>
       <c r="H26" t="n">
-        <v>-350.0000823027218</v>
+        <v>-69.99948883182378</v>
       </c>
       <c r="I26" t="n">
-        <v>198.0806574400519</v>
+        <v>250.4847358760156</v>
       </c>
       <c r="J26" t="n">
         <v>0.5</v>
       </c>
       <c r="K26" t="n">
-        <v>219.2233794389425</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L26" t="n">
-        <v>2730.27</v>
+        <v>1929</v>
       </c>
       <c r="M26" t="n">
-        <v>-113.14</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="27">
@@ -1641,25 +1641,25 @@
         <v>7</v>
       </c>
       <c r="G27" t="n">
-        <v>1027.825934216527</v>
+        <v>898.7488258803544</v>
       </c>
       <c r="H27" t="n">
-        <v>-750.0000078775685</v>
+        <v>-700.0008393549177</v>
       </c>
       <c r="I27" t="n">
-        <v>550.5431132408351</v>
+        <v>99.97387878660368</v>
       </c>
       <c r="J27" t="n">
         <v>0.5</v>
       </c>
       <c r="K27" t="n">
-        <v>545.0608411660348</v>
+        <v>93.4771630765607</v>
       </c>
       <c r="L27" t="n">
-        <v>812.37</v>
+        <v>404.37</v>
       </c>
       <c r="M27" t="n">
-        <v>-622.34</v>
+        <v>-43.67</v>
       </c>
     </row>
     <row r="28">
@@ -1686,25 +1686,25 @@
         <v>8</v>
       </c>
       <c r="G28" t="n">
-        <v>13000.50991142625</v>
+        <v>6000.389603556689</v>
       </c>
       <c r="H28" t="n">
-        <v>-850.0000115881288</v>
+        <v>-50.01026982328746</v>
       </c>
       <c r="I28" t="n">
-        <v>450.8746436698235</v>
+        <v>400.2349878943206</v>
       </c>
       <c r="J28" t="n">
         <v>0.5</v>
       </c>
       <c r="K28" t="n">
-        <v>499.0314924731653</v>
+        <v>402.0604809124811</v>
       </c>
       <c r="L28" t="n">
-        <v>9631.09</v>
+        <v>4643.85</v>
       </c>
       <c r="M28" t="n">
-        <v>-599.87</v>
+        <v>-22.56</v>
       </c>
     </row>
     <row r="29">
@@ -1731,25 +1731,25 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>4066.969812207575</v>
+        <v>1215.905750860737</v>
       </c>
       <c r="H29" t="n">
-        <v>-289.9072200861101</v>
+        <v>-189.9057312945343</v>
       </c>
       <c r="I29" t="n">
-        <v>210.0417580851682</v>
+        <v>407.0881422437045</v>
       </c>
       <c r="J29" t="n">
         <v>0.5</v>
       </c>
       <c r="K29" t="n">
-        <v>219.2233794389425</v>
+        <v>438.4467588778851</v>
       </c>
       <c r="L29" t="n">
-        <v>2352.29</v>
+        <v>914.28</v>
       </c>
       <c r="M29" t="n">
-        <v>-131.42</v>
+        <v>-107.59</v>
       </c>
     </row>
     <row r="30">
@@ -1776,25 +1776,25 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>1137.954912508312</v>
+        <v>6052.18980747446</v>
       </c>
       <c r="H30" t="n">
-        <v>-646.622220474758</v>
+        <v>-396.5908804947525</v>
       </c>
       <c r="I30" t="n">
-        <v>276.30357816535</v>
+        <v>556.6098869791433</v>
       </c>
       <c r="J30" t="n">
         <v>0.5</v>
       </c>
       <c r="K30" t="n">
-        <v>228.9713521405058</v>
+        <v>583.7646963090822</v>
       </c>
       <c r="L30" t="n">
-        <v>791.08</v>
+        <v>4828.47</v>
       </c>
       <c r="M30" t="n">
-        <v>-480.36</v>
+        <v>-293.05</v>
       </c>
     </row>
     <row r="31">
@@ -1821,25 +1821,25 @@
         <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>17055.31164396607</v>
+        <v>2706.077446484792</v>
       </c>
       <c r="H31" t="n">
-        <v>-560.1781801593111</v>
+        <v>-648.755125610872</v>
       </c>
       <c r="I31" t="n">
-        <v>110.0438196228752</v>
+        <v>361.2008634418553</v>
       </c>
       <c r="J31" t="n">
         <v>0.5</v>
       </c>
       <c r="K31" t="n">
-        <v>147.8003722664622</v>
+        <v>368.0199590525625</v>
       </c>
       <c r="L31" t="n">
-        <v>4460.13</v>
+        <v>1988.35</v>
       </c>
       <c r="M31" t="n">
-        <v>1.53</v>
+        <v>-443.21</v>
       </c>
     </row>
     <row r="32">
@@ -1866,25 +1866,25 @@
         <v>3</v>
       </c>
       <c r="G32" t="n">
-        <v>15134.25041484849</v>
+        <v>1160.039326566002</v>
       </c>
       <c r="H32" t="n">
-        <v>-534.944679259166</v>
+        <v>-343.8292530048554</v>
       </c>
       <c r="I32" t="n">
-        <v>109.5818230153575</v>
+        <v>208.245839546934</v>
       </c>
       <c r="J32" t="n">
         <v>0.5</v>
       </c>
       <c r="K32" t="n">
-        <v>147.8003722664622</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L32" t="n">
-        <v>4039.29</v>
+        <v>708.4400000000001</v>
       </c>
       <c r="M32" t="n">
-        <v>-11.13</v>
+        <v>-156.91</v>
       </c>
     </row>
     <row r="33">
@@ -1911,25 +1911,25 @@
         <v>4</v>
       </c>
       <c r="G33" t="n">
-        <v>7040.99053782306</v>
+        <v>1124.005505969476</v>
       </c>
       <c r="H33" t="n">
-        <v>-446.111740891295</v>
+        <v>-289.8944116808059</v>
       </c>
       <c r="I33" t="n">
-        <v>460.2025943329842</v>
+        <v>175.450377927311</v>
       </c>
       <c r="J33" t="n">
         <v>0.5</v>
       </c>
       <c r="K33" t="n">
-        <v>485.7215873880137</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L33" t="n">
-        <v>5453.32</v>
+        <v>613.85</v>
       </c>
       <c r="M33" t="n">
-        <v>-317.41</v>
+        <v>-55.46</v>
       </c>
     </row>
     <row r="34">
@@ -1956,25 +1956,25 @@
         <v>5</v>
       </c>
       <c r="G34" t="n">
-        <v>11027.47244606105</v>
+        <v>12037.41319374223</v>
       </c>
       <c r="H34" t="n">
-        <v>-698.0497014654941</v>
+        <v>-700.456395943226</v>
       </c>
       <c r="I34" t="n">
-        <v>507.5272610347834</v>
+        <v>204.0692418838272</v>
       </c>
       <c r="J34" t="n">
         <v>0.5</v>
       </c>
       <c r="K34" t="n">
-        <v>545.0608411660348</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L34" t="n">
-        <v>8484.549999999999</v>
+        <v>6081.08</v>
       </c>
       <c r="M34" t="n">
-        <v>-516.6</v>
+        <v>-277.75</v>
       </c>
     </row>
     <row r="35">
@@ -2001,25 +2001,25 @@
         <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>4069.37581466081</v>
+        <v>2082.220672870871</v>
       </c>
       <c r="H35" t="n">
-        <v>-247.8331829809671</v>
+        <v>-81.01585838768818</v>
       </c>
       <c r="I35" t="n">
-        <v>208.0478385112941</v>
+        <v>164.6583216603972</v>
       </c>
       <c r="J35" t="n">
         <v>0.5</v>
       </c>
       <c r="K35" t="n">
-        <v>219.2233794389425</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L35" t="n">
-        <v>2309.5</v>
+        <v>1005.55</v>
       </c>
       <c r="M35" t="n">
-        <v>-112.29</v>
+        <v>42.04</v>
       </c>
     </row>
     <row r="36">
@@ -2046,25 +2046,25 @@
         <v>7</v>
       </c>
       <c r="G36" t="n">
-        <v>971.4960597453959</v>
+        <v>993.9385688637034</v>
       </c>
       <c r="H36" t="n">
-        <v>-649.1260841247031</v>
+        <v>-786.7533576806543</v>
       </c>
       <c r="I36" t="n">
-        <v>456.3691939290837</v>
+        <v>109.5955821953368</v>
       </c>
       <c r="J36" t="n">
         <v>0.5</v>
       </c>
       <c r="K36" t="n">
-        <v>423.2358566393677</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L36" t="n">
-        <v>760.36</v>
+        <v>396.93</v>
       </c>
       <c r="M36" t="n">
-        <v>-541.36</v>
+        <v>-106.37</v>
       </c>
     </row>
     <row r="37">
@@ -2091,25 +2091,25 @@
         <v>8</v>
       </c>
       <c r="G37" t="n">
-        <v>12022.73237182239</v>
+        <v>5026.361921194472</v>
       </c>
       <c r="H37" t="n">
-        <v>-747.7937256706006</v>
+        <v>-43.22364469059899</v>
       </c>
       <c r="I37" t="n">
-        <v>362.9115495318044</v>
+        <v>305.2983670604021</v>
       </c>
       <c r="J37" t="n">
         <v>0.5</v>
       </c>
       <c r="K37" t="n">
-        <v>368.0199590525625</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L37" t="n">
-        <v>8715.49</v>
+        <v>3489.11</v>
       </c>
       <c r="M37" t="n">
-        <v>-514.11</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="38">
@@ -2136,25 +2136,25 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>3158.55769225725</v>
+        <v>1130.533538985517</v>
       </c>
       <c r="H38" t="n">
-        <v>-280.0003773655003</v>
+        <v>-180.1350561957965</v>
       </c>
       <c r="I38" t="n">
-        <v>157.7193454704069</v>
+        <v>321.8148572631171</v>
       </c>
       <c r="J38" t="n">
         <v>0.5</v>
       </c>
       <c r="K38" t="n">
-        <v>198.2950076925505</v>
+        <v>295.6007445329244</v>
       </c>
       <c r="L38" t="n">
-        <v>1484.06</v>
+        <v>839.13</v>
       </c>
       <c r="M38" t="n">
-        <v>-56.77</v>
+        <v>-100.24</v>
       </c>
     </row>
     <row r="39">
@@ -2181,25 +2181,25 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>460.2959413989289</v>
+        <v>5107.677076102673</v>
       </c>
       <c r="H39" t="n">
-        <v>-544.4938153687282</v>
+        <v>-296.3310876372636</v>
       </c>
       <c r="I39" t="n">
-        <v>273.1893209249627</v>
+        <v>473.7933811832159</v>
       </c>
       <c r="J39" t="n">
         <v>0.5</v>
       </c>
       <c r="K39" t="n">
-        <v>247.317326764409</v>
+        <v>485.7215873880137</v>
       </c>
       <c r="L39" t="n">
-        <v>342.83</v>
+        <v>4066.58</v>
       </c>
       <c r="M39" t="n">
-        <v>-366.03</v>
+        <v>-223.78</v>
       </c>
     </row>
     <row r="40">
@@ -2226,25 +2226,25 @@
         <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>16085.82406528901</v>
+        <v>2609.322537535607</v>
       </c>
       <c r="H40" t="n">
-        <v>-658.4751543260527</v>
+        <v>-548.6187504593431</v>
       </c>
       <c r="I40" t="n">
-        <v>119.6776790617071</v>
+        <v>291.8737037529374</v>
       </c>
       <c r="J40" t="n">
         <v>0.5</v>
       </c>
       <c r="K40" t="n">
-        <v>198.2950076925505</v>
+        <v>302.9006275609877</v>
       </c>
       <c r="L40" t="n">
-        <v>3761.81</v>
+        <v>1823.14</v>
       </c>
       <c r="M40" t="n">
-        <v>-32.11</v>
+        <v>-341.92</v>
       </c>
     </row>
     <row r="41">
@@ -2271,25 +2271,25 @@
         <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>14163.25881694356</v>
+        <v>1167.392084340332</v>
       </c>
       <c r="H41" t="n">
-        <v>-615.8950602152241</v>
+        <v>-244.8287801604338</v>
       </c>
       <c r="I41" t="n">
-        <v>119.5606509275572</v>
+        <v>218.0751437197306</v>
       </c>
       <c r="J41" t="n">
         <v>0.5</v>
       </c>
       <c r="K41" t="n">
-        <v>198.2950076925505</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L41" t="n">
-        <v>3889.3</v>
+        <v>715.0599999999999</v>
       </c>
       <c r="M41" t="n">
-        <v>-135.09</v>
+        <v>-114.27</v>
       </c>
     </row>
     <row r="42">
@@ -2316,25 +2316,25 @@
         <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>6107.981394672544</v>
+        <v>1068.690098825986</v>
       </c>
       <c r="H42" t="n">
-        <v>-347.6288685623148</v>
+        <v>-279.8928977742883</v>
       </c>
       <c r="I42" t="n">
-        <v>373.1755734725646</v>
+        <v>191.6469241396971</v>
       </c>
       <c r="J42" t="n">
         <v>0.5</v>
       </c>
       <c r="K42" t="n">
-        <v>412.7839753774575</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L42" t="n">
-        <v>4283.31</v>
+        <v>609.97</v>
       </c>
       <c r="M42" t="n">
-        <v>-208.36</v>
+        <v>-114.53</v>
       </c>
     </row>
     <row r="43">
@@ -2361,25 +2361,25 @@
         <v>5</v>
       </c>
       <c r="G43" t="n">
-        <v>10063.41630699886</v>
+        <v>11070.39137852842</v>
       </c>
       <c r="H43" t="n">
-        <v>-600.632976826568</v>
+        <v>-600.5669461729282</v>
       </c>
       <c r="I43" t="n">
-        <v>417.0903812258337</v>
+        <v>210.7459446405713</v>
       </c>
       <c r="J43" t="n">
         <v>0.5</v>
       </c>
       <c r="K43" t="n">
-        <v>457.9427042810117</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L43" t="n">
-        <v>7174.25</v>
+        <v>5868.62</v>
       </c>
       <c r="M43" t="n">
-        <v>-403.07</v>
+        <v>-225.67</v>
       </c>
     </row>
     <row r="44">
@@ -2406,25 +2406,25 @@
         <v>6</v>
       </c>
       <c r="G44" t="n">
-        <v>3140.782280215976</v>
+        <v>1284.080548798787</v>
       </c>
       <c r="H44" t="n">
-        <v>-151.0265724899597</v>
+        <v>-92.98530775150515</v>
       </c>
       <c r="I44" t="n">
-        <v>218.2077966926774</v>
+        <v>143.0221202862179</v>
       </c>
       <c r="J44" t="n">
         <v>0.5</v>
       </c>
       <c r="K44" t="n">
-        <v>247.317326764409</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L44" t="n">
-        <v>1802.66</v>
+        <v>557.38</v>
       </c>
       <c r="M44" t="n">
-        <v>-3.51</v>
+        <v>38.38</v>
       </c>
     </row>
     <row r="45">
@@ -2451,25 +2451,25 @@
         <v>7</v>
       </c>
       <c r="G45" t="n">
-        <v>934.8992660781208</v>
+        <v>1079.869782039313</v>
       </c>
       <c r="H45" t="n">
-        <v>-550.9622393413727</v>
+        <v>-748.7272518943183</v>
       </c>
       <c r="I45" t="n">
-        <v>369.5778370615733</v>
+        <v>120.2436971469181</v>
       </c>
       <c r="J45" t="n">
         <v>0.5</v>
       </c>
       <c r="K45" t="n">
-        <v>337.0367045574487</v>
+        <v>161.9071957960046</v>
       </c>
       <c r="L45" t="n">
-        <v>703.87</v>
+        <v>396.36</v>
       </c>
       <c r="M45" t="n">
-        <v>-402.96</v>
+        <v>-113.08</v>
       </c>
     </row>
     <row r="46">
@@ -2496,25 +2496,25 @@
         <v>8</v>
       </c>
       <c r="G46" t="n">
-        <v>11066.76121939536</v>
+        <v>4067.187634609309</v>
       </c>
       <c r="H46" t="n">
-        <v>-650.7549518827076</v>
+        <v>-35.49593171959112</v>
       </c>
       <c r="I46" t="n">
-        <v>279.0304235559867</v>
+        <v>231.7263940673957</v>
       </c>
       <c r="J46" t="n">
         <v>0.5</v>
       </c>
       <c r="K46" t="n">
-        <v>280.4314892296821</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L46" t="n">
-        <v>7193.69</v>
+        <v>2246.64</v>
       </c>
       <c r="M46" t="n">
-        <v>-391.55</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="47">
@@ -2541,25 +2541,25 @@
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>2372.875687935994</v>
+        <v>1057.869932511433</v>
       </c>
       <c r="H47" t="n">
-        <v>-270.5679035970795</v>
+        <v>-171.0166596595892</v>
       </c>
       <c r="I47" t="n">
-        <v>170.5621258140479</v>
+        <v>240.7230899192821</v>
       </c>
       <c r="J47" t="n">
         <v>0.5</v>
       </c>
       <c r="K47" t="n">
-        <v>186.9543261531214</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L47" t="n">
-        <v>1096.7</v>
+        <v>676.45</v>
       </c>
       <c r="M47" t="n">
-        <v>-74.84999999999999</v>
+        <v>-52.89</v>
       </c>
     </row>
     <row r="48">
@@ -2586,25 +2586,25 @@
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>115.2298325034198</v>
+        <v>4186.962829163704</v>
       </c>
       <c r="H48" t="n">
-        <v>-442.272384299538</v>
+        <v>-205.636211435232</v>
       </c>
       <c r="I48" t="n">
-        <v>278.3311091288366</v>
+        <v>386.5641093946796</v>
       </c>
       <c r="J48" t="n">
         <v>0.5</v>
       </c>
       <c r="K48" t="n">
-        <v>132.1966717950337</v>
+        <v>402.0604809124811</v>
       </c>
       <c r="L48" t="n">
-        <v>-92.51000000000001</v>
+        <v>3102.24</v>
       </c>
       <c r="M48" t="n">
-        <v>115.35</v>
+        <v>-123.7</v>
       </c>
     </row>
     <row r="49">
@@ -2631,25 +2631,25 @@
         <v>2</v>
       </c>
       <c r="G49" t="n">
-        <v>15036.83967238983</v>
+        <v>2513.744736426754</v>
       </c>
       <c r="H49" t="n">
-        <v>-735.2255978860537</v>
+        <v>-456.0958228412754</v>
       </c>
       <c r="I49" t="n">
-        <v>129.389569310694</v>
+        <v>232.1516344876651</v>
       </c>
       <c r="J49" t="n">
         <v>0.5</v>
       </c>
       <c r="K49" t="n">
-        <v>198.2950076925505</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L49" t="n">
-        <v>4130.93</v>
+        <v>1546.31</v>
       </c>
       <c r="M49" t="n">
-        <v>-104.72</v>
+        <v>-249.29</v>
       </c>
     </row>
     <row r="50">
@@ -2676,13 +2676,13 @@
         <v>3</v>
       </c>
       <c r="G50" t="n">
-        <v>13065.3595781167</v>
+        <v>1175.544744073035</v>
       </c>
       <c r="H50" t="n">
-        <v>-658.9534233279167</v>
+        <v>-154.2231277322383</v>
       </c>
       <c r="I50" t="n">
-        <v>129.9588476451862</v>
+        <v>228.6778005707242</v>
       </c>
       <c r="J50" t="n">
         <v>0.5</v>
@@ -2691,10 +2691,10 @@
         <v>198.2950076925505</v>
       </c>
       <c r="L50" t="n">
-        <v>3855.77</v>
+        <v>757.37</v>
       </c>
       <c r="M50" t="n">
-        <v>-85.13</v>
+        <v>-55.43</v>
       </c>
     </row>
     <row r="51">
@@ -2721,25 +2721,25 @@
         <v>4</v>
       </c>
       <c r="G51" t="n">
-        <v>5171.383724506656</v>
+        <v>1098.978136782534</v>
       </c>
       <c r="H51" t="n">
-        <v>-255.3246130681338</v>
+        <v>-273.1828405283795</v>
       </c>
       <c r="I51" t="n">
-        <v>295.5890202094424</v>
+        <v>280.9807085303825</v>
       </c>
       <c r="J51" t="n">
         <v>0.5</v>
       </c>
       <c r="K51" t="n">
-        <v>323.8143915920092</v>
+        <v>302.9006275609877</v>
       </c>
       <c r="L51" t="n">
-        <v>3897.54</v>
+        <v>771.63</v>
       </c>
       <c r="M51" t="n">
-        <v>-166.55</v>
+        <v>-124.64</v>
       </c>
     </row>
     <row r="52">
@@ -2766,25 +2766,25 @@
         <v>5</v>
       </c>
       <c r="G52" t="n">
-        <v>9113.919009922887</v>
+        <v>10094.88686563815</v>
       </c>
       <c r="H52" t="n">
-        <v>-506.5763976321757</v>
+        <v>-503.9819208368904</v>
       </c>
       <c r="I52" t="n">
-        <v>334.1184605994631</v>
+        <v>218.5307011126106</v>
       </c>
       <c r="J52" t="n">
         <v>0.5</v>
       </c>
       <c r="K52" t="n">
-        <v>373.9086523062428</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L52" t="n">
-        <v>6336.01</v>
+        <v>5432.68</v>
       </c>
       <c r="M52" t="n">
-        <v>-316.03</v>
+        <v>-199.72</v>
       </c>
     </row>
     <row r="53">
@@ -2811,25 +2811,25 @@
         <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>2275.432164715334</v>
+        <v>832.207055108518</v>
       </c>
       <c r="H53" t="n">
-        <v>-52.54948851229595</v>
+        <v>-105.9291467219446</v>
       </c>
       <c r="I53" t="n">
-        <v>228.418688756215</v>
+        <v>184.2906413067089</v>
       </c>
       <c r="J53" t="n">
         <v>0.5</v>
       </c>
       <c r="K53" t="n">
-        <v>238.320939301339</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L53" t="n">
-        <v>1374.96</v>
+        <v>497.97</v>
       </c>
       <c r="M53" t="n">
-        <v>4.56</v>
+        <v>-28.13</v>
       </c>
     </row>
     <row r="54">
@@ -2856,25 +2856,25 @@
         <v>7</v>
       </c>
       <c r="G54" t="n">
-        <v>912.2483535788879</v>
+        <v>1152.715039790412</v>
       </c>
       <c r="H54" t="n">
-        <v>-455.112557255282</v>
+        <v>-646.8723436936245</v>
       </c>
       <c r="I54" t="n">
-        <v>300.3777152812987</v>
+        <v>127.9983968826375</v>
       </c>
       <c r="J54" t="n">
         <v>0.5</v>
       </c>
       <c r="K54" t="n">
-        <v>272.5304205830174</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L54" t="n">
-        <v>714.13</v>
+        <v>403.31</v>
       </c>
       <c r="M54" t="n">
-        <v>-319.41</v>
+        <v>-106.87</v>
       </c>
     </row>
     <row r="55">
@@ -2901,25 +2901,25 @@
         <v>8</v>
       </c>
       <c r="G55" t="n">
-        <v>10116.99537088159</v>
+        <v>3218.121574605791</v>
       </c>
       <c r="H55" t="n">
-        <v>-556.6591151121702</v>
+        <v>-47.7438255070707</v>
       </c>
       <c r="I55" t="n">
-        <v>219.9820950115561</v>
+        <v>182.6313955514934</v>
       </c>
       <c r="J55" t="n">
         <v>0.5</v>
       </c>
       <c r="K55" t="n">
-        <v>247.317326764409</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L55" t="n">
-        <v>5571.6</v>
+        <v>1556.73</v>
       </c>
       <c r="M55" t="n">
-        <v>-253.93</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="56">
@@ -2946,25 +2946,25 @@
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>1687.318945380105</v>
+        <v>998.3501438604079</v>
       </c>
       <c r="H56" t="n">
-        <v>-263.5063724440953</v>
+        <v>-161.773536745861</v>
       </c>
       <c r="I56" t="n">
-        <v>241.0008531807191</v>
+        <v>200.8778781042544</v>
       </c>
       <c r="J56" t="n">
         <v>0.5</v>
       </c>
       <c r="K56" t="n">
-        <v>247.317326764409</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L56" t="n">
-        <v>1052.05</v>
+        <v>645.0599999999999</v>
       </c>
       <c r="M56" t="n">
-        <v>-127.4</v>
+        <v>-19.23</v>
       </c>
     </row>
     <row r="57">
@@ -2991,25 +2991,25 @@
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>213.517735983419</v>
+        <v>3286.955743355303</v>
       </c>
       <c r="H57" t="n">
-        <v>-346.8665445864103</v>
+        <v>-120.982535159258</v>
       </c>
       <c r="I57" t="n">
-        <v>283.7212944928282</v>
+        <v>307.6638653179967</v>
       </c>
       <c r="J57" t="n">
         <v>0.5</v>
       </c>
       <c r="K57" t="n">
-        <v>219.2233794389425</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L57" t="n">
-        <v>168.37</v>
+        <v>2264.13</v>
       </c>
       <c r="M57" t="n">
-        <v>-29.45</v>
+        <v>-34.33</v>
       </c>
     </row>
     <row r="58">
@@ -3036,13 +3036,13 @@
         <v>2</v>
       </c>
       <c r="G58" t="n">
-        <v>14016.01760135145</v>
+        <v>2418.038540018982</v>
       </c>
       <c r="H58" t="n">
-        <v>-736.2848961065521</v>
+        <v>-368.8483306491573</v>
       </c>
       <c r="I58" t="n">
-        <v>137.8015339478924</v>
+        <v>195.1721381276441</v>
       </c>
       <c r="J58" t="n">
         <v>0.5</v>
@@ -3051,10 +3051,10 @@
         <v>198.2950076925505</v>
       </c>
       <c r="L58" t="n">
-        <v>4544.18</v>
+        <v>1348.52</v>
       </c>
       <c r="M58" t="n">
-        <v>-147.49</v>
+        <v>-156.29</v>
       </c>
     </row>
     <row r="59">
@@ -3081,25 +3081,25 @@
         <v>3</v>
       </c>
       <c r="G59" t="n">
-        <v>12119.74342286268</v>
+        <v>1183.867240428984</v>
       </c>
       <c r="H59" t="n">
-        <v>-581.2349741641592</v>
+        <v>-70.43678246011369</v>
       </c>
       <c r="I59" t="n">
-        <v>137.3823234960654</v>
+        <v>236.3981070702368</v>
       </c>
       <c r="J59" t="n">
         <v>0.5</v>
       </c>
       <c r="K59" t="n">
-        <v>186.9543261531214</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L59" t="n">
-        <v>4191.32</v>
+        <v>727.9</v>
       </c>
       <c r="M59" t="n">
-        <v>-139.75</v>
+        <v>-12.56</v>
       </c>
     </row>
     <row r="60">
@@ -3126,25 +3126,25 @@
         <v>4</v>
       </c>
       <c r="G60" t="n">
-        <v>4261.317757151879</v>
+        <v>1135.279271510904</v>
       </c>
       <c r="H60" t="n">
-        <v>-172.8236358257539</v>
+        <v>-264.8042285958745</v>
       </c>
       <c r="I60" t="n">
-        <v>225.8709033974851</v>
+        <v>366.7839027508929</v>
       </c>
       <c r="J60" t="n">
         <v>0.5</v>
       </c>
       <c r="K60" t="n">
-        <v>238.320939301339</v>
+        <v>362.0354958462345</v>
       </c>
       <c r="L60" t="n">
-        <v>2553.01</v>
+        <v>899.33</v>
       </c>
       <c r="M60" t="n">
-        <v>-108.6</v>
+        <v>-180.45</v>
       </c>
     </row>
     <row r="61">
@@ -3171,25 +3171,25 @@
         <v>5</v>
       </c>
       <c r="G61" t="n">
-        <v>8185.892128376252</v>
+        <v>9100.045029561477</v>
       </c>
       <c r="H61" t="n">
-        <v>-417.7957247296845</v>
+        <v>-413.2807279650972</v>
       </c>
       <c r="I61" t="n">
-        <v>260.7199480659206</v>
+        <v>224.698266886903</v>
       </c>
       <c r="J61" t="n">
         <v>0.5</v>
       </c>
       <c r="K61" t="n">
-        <v>288.1159665134826</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L61" t="n">
-        <v>5138.31</v>
+        <v>5279.37</v>
       </c>
       <c r="M61" t="n">
-        <v>-238.99</v>
+        <v>-188.05</v>
       </c>
     </row>
     <row r="62">
@@ -3216,25 +3216,25 @@
         <v>6</v>
       </c>
       <c r="G62" t="n">
-        <v>1355.611136018573</v>
+        <v>662.4546982538516</v>
       </c>
       <c r="H62" t="n">
-        <v>-38.32750000683831</v>
+        <v>-118.0140159371381</v>
       </c>
       <c r="I62" t="n">
-        <v>238.052590850084</v>
+        <v>254.5972369373023</v>
       </c>
       <c r="J62" t="n">
         <v>0.5</v>
       </c>
       <c r="K62" t="n">
-        <v>219.2233794389425</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L62" t="n">
-        <v>834.55</v>
+        <v>435.01</v>
       </c>
       <c r="M62" t="n">
-        <v>1.59</v>
+        <v>-59.1</v>
       </c>
     </row>
     <row r="63">
@@ -3261,25 +3261,25 @@
         <v>7</v>
       </c>
       <c r="G63" t="n">
-        <v>907.4816901187377</v>
+        <v>1224.138074060255</v>
       </c>
       <c r="H63" t="n">
-        <v>-365.0348123664114</v>
+        <v>-537.5982938839538</v>
       </c>
       <c r="I63" t="n">
-        <v>251.1109354321227</v>
+        <v>135.1371831682274</v>
       </c>
       <c r="J63" t="n">
         <v>0.5</v>
       </c>
       <c r="K63" t="n">
-        <v>238.320939301339</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L63" t="n">
-        <v>636.47</v>
+        <v>503.65</v>
       </c>
       <c r="M63" t="n">
-        <v>-244.06</v>
+        <v>-105.75</v>
       </c>
     </row>
     <row r="64">
@@ -3306,25 +3306,25 @@
         <v>8</v>
       </c>
       <c r="G64" t="n">
-        <v>9192.889039411055</v>
+        <v>2536.652391493659</v>
       </c>
       <c r="H64" t="n">
-        <v>-468.2370445581951</v>
+        <v>-60.94514618867011</v>
       </c>
       <c r="I64" t="n">
-        <v>191.5522502343736</v>
+        <v>172.9768278495575</v>
       </c>
       <c r="J64" t="n">
         <v>0.5</v>
       </c>
       <c r="K64" t="n">
-        <v>247.317326764409</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L64" t="n">
-        <v>4371.85</v>
+        <v>1216.5</v>
       </c>
       <c r="M64" t="n">
-        <v>-151.8</v>
+        <v>43.74</v>
       </c>
     </row>
     <row r="65">
@@ -3351,25 +3351,25 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>1200.798551008493</v>
+        <v>993.1791832040058</v>
       </c>
       <c r="H65" t="n">
-        <v>-255.4117533000119</v>
+        <v>-154.4065812306485</v>
       </c>
       <c r="I65" t="n">
-        <v>330.5282767182362</v>
+        <v>210.0361285830471</v>
       </c>
       <c r="J65" t="n">
         <v>0.5</v>
       </c>
       <c r="K65" t="n">
-        <v>316.996482935824</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L65" t="n">
-        <v>845.95</v>
+        <v>659.71</v>
       </c>
       <c r="M65" t="n">
-        <v>-163.42</v>
+        <v>-62.42</v>
       </c>
     </row>
     <row r="66">
@@ -3396,25 +3396,25 @@
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>996.1471491217818</v>
+        <v>2406.284348716117</v>
       </c>
       <c r="H66" t="n">
-        <v>-346.4376084316518</v>
+        <v>-50.69016660104491</v>
       </c>
       <c r="I66" t="n">
-        <v>297.2395555747797</v>
+        <v>237.1218925263782</v>
       </c>
       <c r="J66" t="n">
         <v>0.5</v>
       </c>
       <c r="K66" t="n">
-        <v>238.320939301339</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L66" t="n">
-        <v>651.37</v>
+        <v>1471.51</v>
       </c>
       <c r="M66" t="n">
-        <v>-255.73</v>
+        <v>26.73</v>
       </c>
     </row>
     <row r="67">
@@ -3441,25 +3441,25 @@
         <v>2</v>
       </c>
       <c r="G67" t="n">
-        <v>13073.22901759338</v>
+        <v>2327.455219949931</v>
       </c>
       <c r="H67" t="n">
-        <v>-630.4330137870253</v>
+        <v>-288.3043737660081</v>
       </c>
       <c r="I67" t="n">
-        <v>145.1121520940531</v>
+        <v>198.4797962389901</v>
       </c>
       <c r="J67" t="n">
         <v>0.5</v>
       </c>
       <c r="K67" t="n">
-        <v>198.2950076925505</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L67" t="n">
-        <v>4716.99</v>
+        <v>1298.07</v>
       </c>
       <c r="M67" t="n">
-        <v>-107.11</v>
+        <v>-68.52</v>
       </c>
     </row>
     <row r="68">
@@ -3486,25 +3486,25 @@
         <v>3</v>
       </c>
       <c r="G68" t="n">
-        <v>11122.44472850638</v>
+        <v>1159.744266047725</v>
       </c>
       <c r="H68" t="n">
-        <v>-508.3151255679198</v>
+        <v>-6.064612996981595</v>
       </c>
       <c r="I68" t="n">
-        <v>145.0097157523312</v>
+        <v>249.3962093428171</v>
       </c>
       <c r="J68" t="n">
         <v>0.5</v>
       </c>
       <c r="K68" t="n">
-        <v>198.2950076925505</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L68" t="n">
-        <v>4133.03</v>
+        <v>771.53</v>
       </c>
       <c r="M68" t="n">
-        <v>-102.56</v>
+        <v>20.41</v>
       </c>
     </row>
     <row r="69">
@@ -3531,25 +3531,25 @@
         <v>4</v>
       </c>
       <c r="G69" t="n">
-        <v>3346.556092297176</v>
+        <v>1128.912693306465</v>
       </c>
       <c r="H69" t="n">
-        <v>-95.86494945886398</v>
+        <v>-255.7785688315163</v>
       </c>
       <c r="I69" t="n">
-        <v>180.1979801180284</v>
+        <v>380.7133605619992</v>
       </c>
       <c r="J69" t="n">
         <v>0.5</v>
       </c>
       <c r="K69" t="n">
-        <v>238.320939301339</v>
+        <v>355.9504322854629</v>
       </c>
       <c r="L69" t="n">
-        <v>1583.8</v>
+        <v>861.26</v>
       </c>
       <c r="M69" t="n">
-        <v>46.48</v>
+        <v>-201.26</v>
       </c>
     </row>
     <row r="70">
@@ -3576,25 +3576,25 @@
         <v>5</v>
       </c>
       <c r="G70" t="n">
-        <v>7264.143013969493</v>
+        <v>8116.774428492253</v>
       </c>
       <c r="H70" t="n">
-        <v>-334.573960071118</v>
+        <v>-325.6708952095324</v>
       </c>
       <c r="I70" t="n">
-        <v>203.3792613712897</v>
+        <v>232.0005501236062</v>
       </c>
       <c r="J70" t="n">
         <v>0.5</v>
       </c>
       <c r="K70" t="n">
-        <v>247.317326764409</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L70" t="n">
-        <v>3746.92</v>
+        <v>4804.78</v>
       </c>
       <c r="M70" t="n">
-        <v>-118.16</v>
+        <v>-134.16</v>
       </c>
     </row>
     <row r="71">
@@ -3621,25 +3621,25 @@
         <v>6</v>
       </c>
       <c r="G71" t="n">
-        <v>606.0869003847195</v>
+        <v>748.8512730069334</v>
       </c>
       <c r="H71" t="n">
-        <v>-58.71542804940311</v>
+        <v>-120.1777167067946</v>
       </c>
       <c r="I71" t="n">
-        <v>248.857812894495</v>
+        <v>362.2653217278067</v>
       </c>
       <c r="J71" t="n">
         <v>0.5</v>
       </c>
       <c r="K71" t="n">
-        <v>238.320939301339</v>
+        <v>316.996482935824</v>
       </c>
       <c r="L71" t="n">
-        <v>411.93</v>
+        <v>552.25</v>
       </c>
       <c r="M71" t="n">
-        <v>-17.13</v>
+        <v>-92.05</v>
       </c>
     </row>
     <row r="72">
@@ -3666,25 +3666,25 @@
         <v>7</v>
       </c>
       <c r="G72" t="n">
-        <v>906.2299029154472</v>
+        <v>1296.233269953721</v>
       </c>
       <c r="H72" t="n">
-        <v>-279.5552087834045</v>
+        <v>-429.0280025806471</v>
       </c>
       <c r="I72" t="n">
-        <v>229.3509068030974</v>
+        <v>142.7098540371872</v>
       </c>
       <c r="J72" t="n">
         <v>0.5</v>
       </c>
       <c r="K72" t="n">
-        <v>198.2950076925505</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L72" t="n">
-        <v>586.4400000000001</v>
+        <v>562.99</v>
       </c>
       <c r="M72" t="n">
-        <v>-165.55</v>
+        <v>-76.38</v>
       </c>
     </row>
     <row r="73">
@@ -3711,25 +3711,25 @@
         <v>8</v>
       </c>
       <c r="G73" t="n">
-        <v>8302.115926391029</v>
+        <v>1966.860129615384</v>
       </c>
       <c r="H73" t="n">
-        <v>-389.917986527986</v>
+        <v>-71.77840755187954</v>
       </c>
       <c r="I73" t="n">
-        <v>189.7154509068546</v>
+        <v>213.9509612713936</v>
       </c>
       <c r="J73" t="n">
         <v>0.5</v>
       </c>
       <c r="K73" t="n">
-        <v>209.0212909830231</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L73" t="n">
-        <v>4279.22</v>
+        <v>1224.56</v>
       </c>
       <c r="M73" t="n">
-        <v>-158.25</v>
+        <v>5.59</v>
       </c>
     </row>
     <row r="74">
@@ -3756,25 +3756,25 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>819.6629112941687</v>
+        <v>1044.748985230956</v>
       </c>
       <c r="H74" t="n">
-        <v>-245.1630632579705</v>
+        <v>-151.6470310596627</v>
       </c>
       <c r="I74" t="n">
-        <v>380.9123481234928</v>
+        <v>289.7138182871583</v>
       </c>
       <c r="J74" t="n">
         <v>0.5</v>
       </c>
       <c r="K74" t="n">
-        <v>349.7595177200857</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L74" t="n">
-        <v>673.61</v>
+        <v>653.41</v>
       </c>
       <c r="M74" t="n">
-        <v>-201.36</v>
+        <v>-78.31</v>
       </c>
     </row>
     <row r="75">
@@ -3801,25 +3801,25 @@
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>2175.044277632117</v>
+        <v>1472.18659001652</v>
       </c>
       <c r="H75" t="n">
-        <v>-325.5479449971012</v>
+        <v>-10.57209771085231</v>
       </c>
       <c r="I75" t="n">
-        <v>310.0774207306386</v>
+        <v>181.330136554568</v>
       </c>
       <c r="J75" t="n">
         <v>0.5</v>
       </c>
       <c r="K75" t="n">
-        <v>316.996482935824</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L75" t="n">
-        <v>1504.3</v>
+        <v>777.83</v>
       </c>
       <c r="M75" t="n">
-        <v>-201.05</v>
+        <v>73.3</v>
       </c>
     </row>
     <row r="76">
@@ -3846,25 +3846,25 @@
         <v>2</v>
       </c>
       <c r="G76" t="n">
-        <v>12138.91701008291</v>
+        <v>2238.569242824106</v>
       </c>
       <c r="H76" t="n">
-        <v>-504.0955250006974</v>
+        <v>-218.2291566366799</v>
       </c>
       <c r="I76" t="n">
-        <v>151.8736384692515</v>
+        <v>249.8878113512938</v>
       </c>
       <c r="J76" t="n">
         <v>0.5</v>
       </c>
       <c r="K76" t="n">
-        <v>198.2950076925505</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L76" t="n">
-        <v>4725.77</v>
+        <v>1429.11</v>
       </c>
       <c r="M76" t="n">
-        <v>-123.32</v>
+        <v>-91.63</v>
       </c>
     </row>
     <row r="77">
@@ -3891,25 +3891,25 @@
         <v>3</v>
       </c>
       <c r="G77" t="n">
-        <v>10153.55257873</v>
+        <v>1152.948727241017</v>
       </c>
       <c r="H77" t="n">
-        <v>-403.7211011327915</v>
+        <v>8.688363564927693</v>
       </c>
       <c r="I77" t="n">
-        <v>152.5068499700974</v>
+        <v>262.364917637115</v>
       </c>
       <c r="J77" t="n">
         <v>0.5</v>
       </c>
       <c r="K77" t="n">
-        <v>198.2950076925505</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L77" t="n">
-        <v>4030.78</v>
+        <v>828.23</v>
       </c>
       <c r="M77" t="n">
-        <v>-107.14</v>
+        <v>44.6</v>
       </c>
     </row>
     <row r="78">
@@ -3936,25 +3936,25 @@
         <v>4</v>
       </c>
       <c r="G78" t="n">
-        <v>2544.561884273234</v>
+        <v>1084.732296122622</v>
       </c>
       <c r="H78" t="n">
-        <v>-27.7762442311991</v>
+        <v>-245.6267459524598</v>
       </c>
       <c r="I78" t="n">
-        <v>177.6946588499216</v>
+        <v>348.78102327582</v>
       </c>
       <c r="J78" t="n">
         <v>0.5</v>
       </c>
       <c r="K78" t="n">
-        <v>219.2233794389425</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L78" t="n">
-        <v>1231.01</v>
+        <v>820</v>
       </c>
       <c r="M78" t="n">
-        <v>44.59</v>
+        <v>-154.26</v>
       </c>
     </row>
     <row r="79">
@@ -3981,25 +3981,25 @@
         <v>5</v>
       </c>
       <c r="G79" t="n">
-        <v>6376.96907867031</v>
+        <v>7134.743092090062</v>
       </c>
       <c r="H79" t="n">
-        <v>-257.2728031043317</v>
+        <v>-239.4170646014169</v>
       </c>
       <c r="I79" t="n">
-        <v>173.6212303165567</v>
+        <v>238.3586712963733</v>
       </c>
       <c r="J79" t="n">
         <v>0.5</v>
       </c>
       <c r="K79" t="n">
-        <v>219.2233794389425</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L79" t="n">
-        <v>2719.94</v>
+        <v>3904.17</v>
       </c>
       <c r="M79" t="n">
-        <v>-46.64</v>
+        <v>-127</v>
       </c>
     </row>
     <row r="80">
@@ -4026,25 +4026,25 @@
         <v>6</v>
       </c>
       <c r="G80" t="n">
-        <v>185.3252263528502</v>
+        <v>908.6791355539108</v>
       </c>
       <c r="H80" t="n">
-        <v>-101.5161002280638</v>
+        <v>-115.0878020411436</v>
       </c>
       <c r="I80" t="n">
-        <v>262.1998751960827</v>
+        <v>450.4378892625457</v>
       </c>
       <c r="J80" t="n">
         <v>0.5</v>
       </c>
       <c r="K80" t="n">
-        <v>209.0212909830231</v>
+        <v>423.2358566393677</v>
       </c>
       <c r="L80" t="n">
-        <v>62.39</v>
+        <v>719.52</v>
       </c>
       <c r="M80" t="n">
-        <v>48.83</v>
+        <v>-86.43000000000001</v>
       </c>
     </row>
     <row r="81">
@@ -4071,25 +4071,25 @@
         <v>7</v>
       </c>
       <c r="G81" t="n">
-        <v>934.6552588253467</v>
+        <v>1358.108250714662</v>
       </c>
       <c r="H81" t="n">
-        <v>-200.1062280751102</v>
+        <v>-319.2382399572921</v>
       </c>
       <c r="I81" t="n">
-        <v>235.2308426810073</v>
+        <v>149.3078462562578</v>
       </c>
       <c r="J81" t="n">
         <v>0.5</v>
       </c>
       <c r="K81" t="n">
-        <v>198.2950076925505</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L81" t="n">
-        <v>585.71</v>
+        <v>631.02</v>
       </c>
       <c r="M81" t="n">
-        <v>-97.47</v>
+        <v>-68.17</v>
       </c>
     </row>
     <row r="82">
@@ -4116,25 +4116,25 @@
         <v>8</v>
       </c>
       <c r="G82" t="n">
-        <v>7431.803175967705</v>
+        <v>1564.837956988934</v>
       </c>
       <c r="H82" t="n">
-        <v>-324.0482695004142</v>
+        <v>-85.78169767792772</v>
       </c>
       <c r="I82" t="n">
-        <v>204.4518077402314</v>
+        <v>263.4733400299803</v>
       </c>
       <c r="J82" t="n">
         <v>0.5</v>
       </c>
       <c r="K82" t="n">
-        <v>247.317326764409</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L82" t="n">
-        <v>3695.03</v>
+        <v>1047.61</v>
       </c>
       <c r="M82" t="n">
-        <v>-97.11</v>
+        <v>-14.59</v>
       </c>
     </row>
     <row r="83">
@@ -4161,25 +4161,25 @@
         <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>577.125090045642</v>
+        <v>1078.208718474014</v>
       </c>
       <c r="H83" t="n">
-        <v>-233.8198033269143</v>
+        <v>-144.8683067472841</v>
       </c>
       <c r="I83" t="n">
-        <v>380.0281450064591</v>
+        <v>353.6085059491093</v>
       </c>
       <c r="J83" t="n">
         <v>0.5</v>
       </c>
       <c r="K83" t="n">
-        <v>402.0604809124811</v>
+        <v>343.4570282107588</v>
       </c>
       <c r="L83" t="n">
-        <v>439.51</v>
+        <v>817.41</v>
       </c>
       <c r="M83" t="n">
-        <v>-125.87</v>
+        <v>-92.33</v>
       </c>
     </row>
     <row r="84">
@@ -4206,25 +4206,25 @@
         <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>2572.336229967408</v>
+        <v>820.0051867394229</v>
       </c>
       <c r="H84" t="n">
-        <v>-255.4256497849768</v>
+        <v>-20.15805606297685</v>
       </c>
       <c r="I84" t="n">
-        <v>316.8847722509851</v>
+        <v>164.8948691240933</v>
       </c>
       <c r="J84" t="n">
         <v>0.5</v>
       </c>
       <c r="K84" t="n">
-        <v>343.4570282107588</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L84" t="n">
-        <v>1775.71</v>
+        <v>468.03</v>
       </c>
       <c r="M84" t="n">
-        <v>-140.27</v>
+        <v>84.19</v>
       </c>
     </row>
     <row r="85">
@@ -4251,25 +4251,25 @@
         <v>2</v>
       </c>
       <c r="G85" t="n">
-        <v>11146.8736233726</v>
+        <v>2132.981549682821</v>
       </c>
       <c r="H85" t="n">
-        <v>-394.2628987792985</v>
+        <v>-166.0818774239034</v>
       </c>
       <c r="I85" t="n">
-        <v>158.8460487605178</v>
+        <v>306.9913336196968</v>
       </c>
       <c r="J85" t="n">
         <v>0.5</v>
       </c>
       <c r="K85" t="n">
-        <v>209.0212909830231</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L85" t="n">
-        <v>4760.63</v>
+        <v>1506.81</v>
       </c>
       <c r="M85" t="n">
-        <v>-77.91</v>
+        <v>-77.98</v>
       </c>
     </row>
     <row r="86">
@@ -4296,25 +4296,25 @@
         <v>3</v>
       </c>
       <c r="G86" t="n">
-        <v>9147.177315210061</v>
+        <v>1114.517605338163</v>
       </c>
       <c r="H86" t="n">
-        <v>-308.741102657087</v>
+        <v>-15.87729767817521</v>
       </c>
       <c r="I86" t="n">
-        <v>159.9469484092742</v>
+        <v>271.850679174646</v>
       </c>
       <c r="J86" t="n">
         <v>0.5</v>
       </c>
       <c r="K86" t="n">
-        <v>209.0212909830231</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L86" t="n">
-        <v>3680.9</v>
+        <v>809.83</v>
       </c>
       <c r="M86" t="n">
-        <v>12.52</v>
+        <v>16.69</v>
       </c>
     </row>
     <row r="87">
@@ -4341,25 +4341,25 @@
         <v>4</v>
       </c>
       <c r="G87" t="n">
-        <v>1928.993479968963</v>
+        <v>1040.18273543798</v>
       </c>
       <c r="H87" t="n">
-        <v>-35.45787674127823</v>
+        <v>-234.9883838617904</v>
       </c>
       <c r="I87" t="n">
-        <v>195.3632898966781</v>
+        <v>304.0285450506232</v>
       </c>
       <c r="J87" t="n">
         <v>0.5</v>
       </c>
       <c r="K87" t="n">
-        <v>209.0212909830231</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L87" t="n">
-        <v>970.41</v>
+        <v>770.47</v>
       </c>
       <c r="M87" t="n">
-        <v>-17.25</v>
+        <v>-143.31</v>
       </c>
     </row>
     <row r="88">
@@ -4386,25 +4386,25 @@
         <v>5</v>
       </c>
       <c r="G88" t="n">
-        <v>5516.709071804836</v>
+        <v>6142.689044862905</v>
       </c>
       <c r="H88" t="n">
-        <v>-196.45218379572</v>
+        <v>-163.0664908170757</v>
       </c>
       <c r="I88" t="n">
-        <v>172.7290675192446</v>
+        <v>243.7100930866707</v>
       </c>
       <c r="J88" t="n">
         <v>0.5</v>
       </c>
       <c r="K88" t="n">
-        <v>219.2233794389425</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L88" t="n">
-        <v>2404.5</v>
+        <v>3600.47</v>
       </c>
       <c r="M88" t="n">
-        <v>0.83</v>
+        <v>-33.79</v>
       </c>
     </row>
     <row r="89">
@@ -4431,25 +4431,25 @@
         <v>6</v>
       </c>
       <c r="G89" t="n">
-        <v>340.4982806958129</v>
+        <v>1038.372170982426</v>
       </c>
       <c r="H89" t="n">
-        <v>-123.7430278526353</v>
+        <v>-105.3080328740211</v>
       </c>
       <c r="I89" t="n">
-        <v>274.6278309108728</v>
+        <v>461.5581520131385</v>
       </c>
       <c r="J89" t="n">
         <v>0.5</v>
       </c>
       <c r="K89" t="n">
-        <v>228.9713521405058</v>
+        <v>453.1473605746647</v>
       </c>
       <c r="L89" t="n">
-        <v>141.67</v>
+        <v>848.97</v>
       </c>
       <c r="M89" t="n">
-        <v>10.61</v>
+        <v>-65.84999999999999</v>
       </c>
     </row>
     <row r="90">
@@ -4476,25 +4476,25 @@
         <v>7</v>
       </c>
       <c r="G90" t="n">
-        <v>994.6381355118517</v>
+        <v>1415.502936800767</v>
       </c>
       <c r="H90" t="n">
-        <v>-129.5018287891428</v>
+        <v>-221.4414572216136</v>
       </c>
       <c r="I90" t="n">
-        <v>282.4821381978824</v>
+        <v>157.0395894861972</v>
       </c>
       <c r="J90" t="n">
         <v>0.5</v>
       </c>
       <c r="K90" t="n">
-        <v>247.317326764409</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L90" t="n">
-        <v>762.6799999999999</v>
+        <v>679.4299999999999</v>
       </c>
       <c r="M90" t="n">
-        <v>-69.27</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="91">
@@ -4521,25 +4521,25 @@
         <v>8</v>
       </c>
       <c r="G91" t="n">
-        <v>6573.11668458195</v>
+        <v>1158.489278176865</v>
       </c>
       <c r="H91" t="n">
-        <v>-258.8226846325616</v>
+        <v>-96.24309220192508</v>
       </c>
       <c r="I91" t="n">
-        <v>254.1503154042929</v>
+        <v>336.3927398003949</v>
       </c>
       <c r="J91" t="n">
         <v>0.5</v>
       </c>
       <c r="K91" t="n">
-        <v>272.5304205830174</v>
+        <v>343.4570282107588</v>
       </c>
       <c r="L91" t="n">
-        <v>4134.34</v>
+        <v>816.37</v>
       </c>
       <c r="M91" t="n">
-        <v>-82.48</v>
+        <v>-33.74</v>
       </c>
     </row>
     <row r="92">
@@ -4566,25 +4566,25 @@
         <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>460.3095689412088</v>
+        <v>1115.979031089478</v>
       </c>
       <c r="H92" t="n">
-        <v>-221.8545947107568</v>
+        <v>-136.4049437320336</v>
       </c>
       <c r="I92" t="n">
-        <v>346.1048114132217</v>
+        <v>372.2454576800065</v>
       </c>
       <c r="J92" t="n">
         <v>0.5</v>
       </c>
       <c r="K92" t="n">
-        <v>337.0367045574487</v>
+        <v>355.9504322854629</v>
       </c>
       <c r="L92" t="n">
-        <v>388.09</v>
+        <v>795.8</v>
       </c>
       <c r="M92" t="n">
-        <v>-67.05</v>
+        <v>-83.95999999999999</v>
       </c>
     </row>
     <row r="93">
@@ -4611,25 +4611,25 @@
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>2183.94729429368</v>
+        <v>495.8898480051805</v>
       </c>
       <c r="H93" t="n">
-        <v>-183.9700531548368</v>
+        <v>-67.54890965713822</v>
       </c>
       <c r="I93" t="n">
-        <v>317.5527145749084</v>
+        <v>193.8315659354112</v>
       </c>
       <c r="J93" t="n">
         <v>0.5</v>
       </c>
       <c r="K93" t="n">
-        <v>330.4916794875841</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L93" t="n">
-        <v>1493.11</v>
+        <v>265.31</v>
       </c>
       <c r="M93" t="n">
-        <v>-93.54000000000001</v>
+        <v>102.69</v>
       </c>
     </row>
     <row r="94">
@@ -4656,25 +4656,25 @@
         <v>2</v>
       </c>
       <c r="G94" t="n">
-        <v>10165.89225549583</v>
+        <v>2024.150024359569</v>
       </c>
       <c r="H94" t="n">
-        <v>-277.4050981376181</v>
+        <v>-111.7974668639166</v>
       </c>
       <c r="I94" t="n">
-        <v>165.785261160814</v>
+        <v>341.4261493486725</v>
       </c>
       <c r="J94" t="n">
         <v>0.5</v>
       </c>
       <c r="K94" t="n">
-        <v>219.2233794389425</v>
+        <v>330.4916794875841</v>
       </c>
       <c r="L94" t="n">
-        <v>4110.89</v>
+        <v>1536.77</v>
       </c>
       <c r="M94" t="n">
-        <v>-37.08</v>
+        <v>-66.40000000000001</v>
       </c>
     </row>
     <row r="95">
@@ -4701,25 +4701,25 @@
         <v>3</v>
       </c>
       <c r="G95" t="n">
-        <v>8154.714818232391</v>
+        <v>1044.949757183546</v>
       </c>
       <c r="H95" t="n">
-        <v>-209.2994343332427</v>
+        <v>-68.47995774128385</v>
       </c>
       <c r="I95" t="n">
-        <v>167.4732306890452</v>
+        <v>278.0409299000953</v>
       </c>
       <c r="J95" t="n">
         <v>0.5</v>
       </c>
       <c r="K95" t="n">
-        <v>209.0212909830231</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L95" t="n">
-        <v>3652.96</v>
+        <v>735.42</v>
       </c>
       <c r="M95" t="n">
-        <v>-56.53</v>
+        <v>-23.41</v>
       </c>
     </row>
     <row r="96">
@@ -4746,13 +4746,13 @@
         <v>4</v>
       </c>
       <c r="G96" t="n">
-        <v>1453.927614960564</v>
+        <v>996.9719004176009</v>
       </c>
       <c r="H96" t="n">
-        <v>-65.89280523207239</v>
+        <v>-225.0421100900935</v>
       </c>
       <c r="I96" t="n">
-        <v>240.1228542009275</v>
+        <v>253.3360651377453</v>
       </c>
       <c r="J96" t="n">
         <v>0.5</v>
@@ -4761,10 +4761,10 @@
         <v>247.317326764409</v>
       </c>
       <c r="L96" t="n">
-        <v>917.75</v>
+        <v>716.75</v>
       </c>
       <c r="M96" t="n">
-        <v>23</v>
+        <v>-126.68</v>
       </c>
     </row>
     <row r="97">
@@ -4791,25 +4791,25 @@
         <v>5</v>
       </c>
       <c r="G97" t="n">
-        <v>4669.202403853839</v>
+        <v>5228.696575126458</v>
       </c>
       <c r="H97" t="n">
-        <v>-156.6643185222407</v>
+        <v>-86.85817722151528</v>
       </c>
       <c r="I97" t="n">
-        <v>213.7323404519297</v>
+        <v>250.5550053132966</v>
       </c>
       <c r="J97" t="n">
         <v>0.5</v>
       </c>
       <c r="K97" t="n">
-        <v>238.320939301339</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L97" t="n">
-        <v>2626.1</v>
+        <v>3425.11</v>
       </c>
       <c r="M97" t="n">
-        <v>-49.3</v>
+        <v>-14.28</v>
       </c>
     </row>
     <row r="98">
@@ -4836,25 +4836,25 @@
         <v>6</v>
       </c>
       <c r="G98" t="n">
-        <v>649.3436157154672</v>
+        <v>1085.413328886694</v>
       </c>
       <c r="H98" t="n">
-        <v>-212.0437072136316</v>
+        <v>-94.89744739066985</v>
       </c>
       <c r="I98" t="n">
-        <v>285.0304121852122</v>
+        <v>391.996397980547</v>
       </c>
       <c r="J98" t="n">
         <v>0.5</v>
       </c>
       <c r="K98" t="n">
-        <v>264.3933435900673</v>
+        <v>343.4570282107588</v>
       </c>
       <c r="L98" t="n">
-        <v>485.99</v>
+        <v>861.42</v>
       </c>
       <c r="M98" t="n">
-        <v>-114.05</v>
+        <v>-66.38</v>
       </c>
     </row>
     <row r="99">
@@ -4881,25 +4881,25 @@
         <v>7</v>
       </c>
       <c r="G99" t="n">
-        <v>1076.698074856911</v>
+        <v>1461.034509116139</v>
       </c>
       <c r="H99" t="n">
-        <v>-70.57419431577387</v>
+        <v>-128.1531932808778</v>
       </c>
       <c r="I99" t="n">
-        <v>359.219607606251</v>
+        <v>165.4152434847231</v>
       </c>
       <c r="J99" t="n">
         <v>0.5</v>
       </c>
       <c r="K99" t="n">
-        <v>355.9504322854629</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L99" t="n">
-        <v>810.5700000000001</v>
+        <v>733.85</v>
       </c>
       <c r="M99" t="n">
-        <v>-23.3</v>
+        <v>22.15</v>
       </c>
     </row>
     <row r="100">
@@ -4926,25 +4926,25 @@
         <v>8</v>
       </c>
       <c r="G100" t="n">
-        <v>5698.809582435395</v>
+        <v>750.3360501749027</v>
       </c>
       <c r="H100" t="n">
-        <v>-205.0280594781762</v>
+        <v>-103.2246130659583</v>
       </c>
       <c r="I100" t="n">
-        <v>295.9067675151588</v>
+        <v>390.0644500926164</v>
       </c>
       <c r="J100" t="n">
         <v>0.5</v>
       </c>
       <c r="K100" t="n">
-        <v>323.8143915920092</v>
+        <v>349.7595177200857</v>
       </c>
       <c r="L100" t="n">
-        <v>3863.98</v>
+        <v>522.0599999999999</v>
       </c>
       <c r="M100" t="n">
-        <v>-92.77</v>
+        <v>-55.31</v>
       </c>
     </row>
   </sheetData>
@@ -5025,7 +5025,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -5044,33 +5044,33 @@
         <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>1076.698074856911</v>
+        <v>1044.949757183546</v>
       </c>
       <c r="H2" t="n">
-        <v>-70.57419431577387</v>
+        <v>-68.47995774128385</v>
       </c>
       <c r="I2" t="n">
-        <v>359.219607606251</v>
+        <v>278.0409299000953</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>355.9504322854629</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L2" t="n">
-        <v>810.5700000000001</v>
+        <v>735.42</v>
       </c>
       <c r="M2" t="n">
-        <v>-23.3</v>
+        <v>-23.41</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -5086,36 +5086,36 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>606.0869003847195</v>
+        <v>998.3501438604079</v>
       </c>
       <c r="H3" t="n">
-        <v>-58.71542804940311</v>
+        <v>-161.773536745861</v>
       </c>
       <c r="I3" t="n">
-        <v>248.857812894495</v>
+        <v>200.8778781042544</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>238.320939301339</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L3" t="n">
-        <v>411.93</v>
+        <v>645.0599999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>-17.13</v>
+        <v>-19.23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>85</v>
+        <v>57</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -5131,31 +5131,31 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>1928.993479968963</v>
+        <v>1183.867240428984</v>
       </c>
       <c r="H4" t="n">
-        <v>-35.45787674127823</v>
+        <v>-70.43678246011369</v>
       </c>
       <c r="I4" t="n">
-        <v>195.3632898966781</v>
+        <v>236.3981070702368</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>209.0212909830231</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L4" t="n">
-        <v>970.41</v>
+        <v>727.9</v>
       </c>
       <c r="M4" t="n">
-        <v>-17.25</v>
+        <v>-12.56</v>
       </c>
     </row>
   </sheetData>
@@ -5268,31 +5268,31 @@
         <v>-21.42555</v>
       </c>
       <c r="G2" t="n">
-        <v>267</v>
+        <v>238</v>
       </c>
       <c r="H2" t="n">
-        <v>83</v>
+        <v>38</v>
       </c>
       <c r="I2" t="n">
-        <v>1203</v>
+        <v>1075</v>
       </c>
       <c r="J2" t="n">
-        <v>670</v>
+        <v>96</v>
       </c>
       <c r="K2" t="n">
-        <v>-54</v>
+        <v>-100</v>
       </c>
       <c r="L2" t="n">
-        <v>670</v>
+        <v>96</v>
       </c>
       <c r="M2" t="n">
-        <v>-4.71</v>
+        <v>-17.61</v>
       </c>
       <c r="N2" t="n">
-        <v>39.65670577452622</v>
+        <v>32.46503808274238</v>
       </c>
       <c r="O2" t="n">
-        <v>60.98474917760892</v>
+        <v>78.62363537239543</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: first version of GUI
</commit_message>
<xml_diff>
--- a/test_alldata.xlsx
+++ b/test_alldata.xlsx
@@ -516,25 +516,25 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1500</v>
+        <v>16000</v>
       </c>
       <c r="H2" t="n">
-        <v>-550</v>
+        <v>-50</v>
       </c>
       <c r="I2" t="n">
-        <v>550</v>
+        <v>100</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>528.7866871801347</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L2" t="n">
-        <v>1248.89</v>
+        <v>3434.76</v>
       </c>
       <c r="M2" t="n">
-        <v>-471.44</v>
+        <v>89.78</v>
       </c>
     </row>
     <row r="3">
@@ -561,25 +561,25 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1100</v>
+        <v>1500</v>
       </c>
       <c r="H3" t="n">
-        <v>-500</v>
+        <v>-650</v>
       </c>
       <c r="I3" t="n">
-        <v>350</v>
+        <v>750</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>323.8143915920092</v>
+        <v>733.0660072843224</v>
       </c>
       <c r="L3" t="n">
-        <v>845.49</v>
+        <v>1302.14</v>
       </c>
       <c r="M3" t="n">
-        <v>-367.92</v>
+        <v>-578.55</v>
       </c>
     </row>
     <row r="4">
@@ -606,25 +606,25 @@
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>7000</v>
+        <v>16000</v>
       </c>
       <c r="H4" t="n">
-        <v>-750</v>
+        <v>-600</v>
       </c>
       <c r="I4" t="n">
-        <v>550</v>
+        <v>850</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>572.4283803512647</v>
+        <v>869.3878716987178</v>
       </c>
       <c r="L4" t="n">
-        <v>5646.55</v>
+        <v>13774.54</v>
       </c>
       <c r="M4" t="n">
-        <v>-585.0700000000001</v>
+        <v>-515.13</v>
       </c>
     </row>
     <row r="5">
@@ -651,25 +651,25 @@
         <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>18000</v>
+        <v>9000</v>
       </c>
       <c r="H5" t="n">
         <v>-650</v>
       </c>
       <c r="I5" t="n">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="J5" t="n">
         <v>0.5</v>
       </c>
       <c r="K5" t="n">
-        <v>756.5300331798771</v>
+        <v>627.0638729490693</v>
       </c>
       <c r="L5" t="n">
-        <v>14500.46</v>
+        <v>7387.98</v>
       </c>
       <c r="M5" t="n">
-        <v>-502.42</v>
+        <v>-517.85</v>
       </c>
     </row>
     <row r="6">
@@ -696,25 +696,25 @@
         <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>17000</v>
+        <v>1500</v>
       </c>
       <c r="H6" t="n">
-        <v>-850</v>
+        <v>-50</v>
       </c>
       <c r="I6" t="n">
-        <v>300</v>
+        <v>650</v>
       </c>
       <c r="J6" t="n">
         <v>0.5</v>
       </c>
       <c r="K6" t="n">
-        <v>337.0367045574487</v>
+        <v>660.9833589751682</v>
       </c>
       <c r="L6" t="n">
-        <v>10601.77</v>
+        <v>1261.13</v>
       </c>
       <c r="M6" t="n">
-        <v>-473.43</v>
+        <v>-21.37</v>
       </c>
     </row>
     <row r="7">
@@ -741,25 +741,25 @@
         <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>20000</v>
+        <v>1100</v>
       </c>
       <c r="H7" t="n">
-        <v>-150</v>
+        <v>-600</v>
       </c>
       <c r="I7" t="n">
-        <v>650</v>
+        <v>400</v>
       </c>
       <c r="J7" t="n">
         <v>0.5</v>
       </c>
       <c r="K7" t="n">
-        <v>647.6287831840184</v>
+        <v>385.4162169477469</v>
       </c>
       <c r="L7" t="n">
-        <v>16386.09</v>
+        <v>854.63</v>
       </c>
       <c r="M7" t="n">
-        <v>-101.64</v>
+        <v>-462.13</v>
       </c>
     </row>
     <row r="8">
@@ -786,10 +786,10 @@
         <v>6</v>
       </c>
       <c r="G8" t="n">
-        <v>1400</v>
+        <v>2000</v>
       </c>
       <c r="H8" t="n">
-        <v>-750</v>
+        <v>-150</v>
       </c>
       <c r="I8" t="n">
         <v>300</v>
@@ -798,13 +798,13 @@
         <v>0.5</v>
       </c>
       <c r="K8" t="n">
-        <v>302.9006275609877</v>
+        <v>310.0286763918156</v>
       </c>
       <c r="L8" t="n">
-        <v>1003.22</v>
+        <v>1371.01</v>
       </c>
       <c r="M8" t="n">
-        <v>-485.53</v>
+        <v>-52.2</v>
       </c>
     </row>
     <row r="9">
@@ -831,25 +831,25 @@
         <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>1500</v>
+        <v>3000</v>
       </c>
       <c r="H9" t="n">
-        <v>-450</v>
+        <v>-100</v>
       </c>
       <c r="I9" t="n">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="J9" t="n">
         <v>0.5</v>
       </c>
       <c r="K9" t="n">
-        <v>699.5190354401714</v>
+        <v>804.1209618249621</v>
       </c>
       <c r="L9" t="n">
-        <v>1272.21</v>
+        <v>2634.42</v>
       </c>
       <c r="M9" t="n">
-        <v>-389.85</v>
+        <v>-74.76000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -876,25 +876,25 @@
         <v>8</v>
       </c>
       <c r="G10" t="n">
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="H10" t="n">
-        <v>-50</v>
+        <v>-700</v>
       </c>
       <c r="I10" t="n">
-        <v>750</v>
+        <v>850</v>
       </c>
       <c r="J10" t="n">
         <v>0.5</v>
       </c>
       <c r="K10" t="n">
-        <v>776.4796334496434</v>
+        <v>891.7153029597591</v>
       </c>
       <c r="L10" t="n">
-        <v>10195.16</v>
+        <v>15279.63</v>
       </c>
       <c r="M10" t="n">
-        <v>-34.95</v>
+        <v>-584.6900000000001</v>
       </c>
     </row>
     <row r="11">
@@ -921,25 +921,25 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1400</v>
+        <v>15000</v>
       </c>
       <c r="H11" t="n">
-        <v>-650</v>
+        <v>-60</v>
       </c>
       <c r="I11" t="n">
-        <v>450</v>
+        <v>90</v>
       </c>
       <c r="J11" t="n">
         <v>0.5</v>
       </c>
       <c r="K11" t="n">
-        <v>428.3661755480705</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L11" t="n">
-        <v>1174.58</v>
+        <v>2750.88</v>
       </c>
       <c r="M11" t="n">
-        <v>-570.26</v>
+        <v>63.84</v>
       </c>
     </row>
     <row r="12">
@@ -966,25 +966,25 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>1000</v>
+        <v>1400</v>
       </c>
       <c r="H12" t="n">
-        <v>-600</v>
+        <v>-750</v>
       </c>
       <c r="I12" t="n">
-        <v>250</v>
+        <v>650</v>
       </c>
       <c r="J12" t="n">
         <v>0.5</v>
       </c>
       <c r="K12" t="n">
-        <v>209.0212909830231</v>
+        <v>605.8012551219755</v>
       </c>
       <c r="L12" t="n">
-        <v>660.22</v>
+        <v>1250.44</v>
       </c>
       <c r="M12" t="n">
-        <v>-421.7</v>
+        <v>-682.08</v>
       </c>
     </row>
     <row r="13">
@@ -1011,25 +1011,25 @@
         <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>6000</v>
+        <v>15000</v>
       </c>
       <c r="H13" t="n">
-        <v>-850</v>
+        <v>-700</v>
       </c>
       <c r="I13" t="n">
-        <v>450</v>
+        <v>750</v>
       </c>
       <c r="J13" t="n">
         <v>0.5</v>
       </c>
       <c r="K13" t="n">
-        <v>418.0425819660462</v>
+        <v>801.3997324917706</v>
       </c>
       <c r="L13" t="n">
-        <v>4785.83</v>
+        <v>12234.27</v>
       </c>
       <c r="M13" t="n">
-        <v>-656.8</v>
+        <v>-554.61</v>
       </c>
     </row>
     <row r="14">
@@ -1056,25 +1056,25 @@
         <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>17000</v>
+        <v>8000</v>
       </c>
       <c r="H14" t="n">
         <v>-750</v>
       </c>
       <c r="I14" t="n">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="J14" t="n">
         <v>0.5</v>
       </c>
       <c r="K14" t="n">
-        <v>650.9931111899981</v>
+        <v>532.9018207393951</v>
       </c>
       <c r="L14" t="n">
-        <v>13234.47</v>
+        <v>6197.48</v>
       </c>
       <c r="M14" t="n">
-        <v>-556.67</v>
+        <v>-567.14</v>
       </c>
     </row>
     <row r="15">
@@ -1101,25 +1101,25 @@
         <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>16000</v>
+        <v>1400</v>
       </c>
       <c r="H15" t="n">
-        <v>-950</v>
+        <v>-60</v>
       </c>
       <c r="I15" t="n">
-        <v>290</v>
+        <v>550</v>
       </c>
       <c r="J15" t="n">
         <v>0.5</v>
       </c>
       <c r="K15" t="n">
-        <v>330.4916794875841</v>
+        <v>511.9955082862131</v>
       </c>
       <c r="L15" t="n">
-        <v>9691.530000000001</v>
+        <v>1191.94</v>
       </c>
       <c r="M15" t="n">
-        <v>-521.75</v>
+        <v>-45.79</v>
       </c>
     </row>
     <row r="16">
@@ -1146,25 +1146,25 @@
         <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>19000</v>
+        <v>1000</v>
       </c>
       <c r="H16" t="n">
-        <v>-160</v>
+        <v>-700</v>
       </c>
       <c r="I16" t="n">
-        <v>550</v>
+        <v>300</v>
       </c>
       <c r="J16" t="n">
         <v>0.5</v>
       </c>
       <c r="K16" t="n">
-        <v>591.2014890658488</v>
+        <v>302.9006275609877</v>
       </c>
       <c r="L16" t="n">
-        <v>14842.33</v>
+        <v>728.99</v>
       </c>
       <c r="M16" t="n">
-        <v>-93.29000000000001</v>
+        <v>-455.73</v>
       </c>
     </row>
     <row r="17">
@@ -1191,10 +1191,10 @@
         <v>6</v>
       </c>
       <c r="G17" t="n">
-        <v>1300</v>
+        <v>1900</v>
       </c>
       <c r="H17" t="n">
-        <v>-850</v>
+        <v>-160</v>
       </c>
       <c r="I17" t="n">
         <v>290</v>
@@ -1203,13 +1203,13 @@
         <v>0.5</v>
       </c>
       <c r="K17" t="n">
-        <v>295.6007445329244</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L17" t="n">
-        <v>937.86</v>
+        <v>1334.83</v>
       </c>
       <c r="M17" t="n">
-        <v>-563.62</v>
+        <v>-88.59</v>
       </c>
     </row>
     <row r="18">
@@ -1236,25 +1236,25 @@
         <v>7</v>
       </c>
       <c r="G18" t="n">
-        <v>1400</v>
+        <v>2900</v>
       </c>
       <c r="H18" t="n">
-        <v>-550</v>
+        <v>-110</v>
       </c>
       <c r="I18" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="J18" t="n">
         <v>0.5</v>
       </c>
       <c r="K18" t="n">
-        <v>485.7215873880137</v>
+        <v>721.0477175625025</v>
       </c>
       <c r="L18" t="n">
-        <v>1175.99</v>
+        <v>2435.11</v>
       </c>
       <c r="M18" t="n">
-        <v>-497.76</v>
+        <v>-76.88</v>
       </c>
     </row>
     <row r="19">
@@ -1281,25 +1281,25 @@
         <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>11000</v>
+        <v>17000</v>
       </c>
       <c r="H19" t="n">
-        <v>-60</v>
+        <v>-800</v>
       </c>
       <c r="I19" t="n">
-        <v>650</v>
+        <v>750</v>
       </c>
       <c r="J19" t="n">
         <v>0.5</v>
       </c>
       <c r="K19" t="n">
-        <v>690.0868864990008</v>
+        <v>787.6525764547314</v>
       </c>
       <c r="L19" t="n">
-        <v>8953.41</v>
+        <v>14349.02</v>
       </c>
       <c r="M19" t="n">
-        <v>-33.83</v>
+        <v>-663.39</v>
       </c>
     </row>
     <row r="20">
@@ -1326,25 +1326,25 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>1309.861170509832</v>
+        <v>14001.77852921273</v>
       </c>
       <c r="H20" t="n">
-        <v>-550.0000117628734</v>
+        <v>-69.99999199863345</v>
       </c>
       <c r="I20" t="n">
-        <v>351.1145283712297</v>
+        <v>99.83889423976993</v>
       </c>
       <c r="J20" t="n">
         <v>0.5</v>
       </c>
       <c r="K20" t="n">
-        <v>316.996482935824</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L20" t="n">
-        <v>1021.46</v>
+        <v>2930.37</v>
       </c>
       <c r="M20" t="n">
-        <v>-433.48</v>
+        <v>183.03</v>
       </c>
     </row>
     <row r="21">
@@ -1371,25 +1371,25 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>951.4571324201941</v>
+        <v>1310.154300581582</v>
       </c>
       <c r="H21" t="n">
-        <v>-500.000014472373</v>
+        <v>-650.0000096439097</v>
       </c>
       <c r="I21" t="n">
-        <v>169.4668957805326</v>
+        <v>550.426048659099</v>
       </c>
       <c r="J21" t="n">
         <v>0.5</v>
       </c>
       <c r="K21" t="n">
-        <v>147.8003722664622</v>
+        <v>472.0365350579011</v>
       </c>
       <c r="L21" t="n">
-        <v>459.97</v>
+        <v>1062.68</v>
       </c>
       <c r="M21" t="n">
-        <v>-158.63</v>
+        <v>-521.46</v>
       </c>
     </row>
     <row r="22">
@@ -1416,25 +1416,25 @@
         <v>2</v>
       </c>
       <c r="G22" t="n">
-        <v>5001.957430303275</v>
+        <v>14000.35243258604</v>
       </c>
       <c r="H22" t="n">
-        <v>-750.0000113163368</v>
+        <v>-600.0000186326773</v>
       </c>
       <c r="I22" t="n">
-        <v>351.2149762766293</v>
+        <v>650.382056893912</v>
       </c>
       <c r="J22" t="n">
         <v>0.5</v>
       </c>
       <c r="K22" t="n">
-        <v>373.9086523062428</v>
+        <v>686.9140564215176</v>
       </c>
       <c r="L22" t="n">
-        <v>3689.37</v>
+        <v>11463.82</v>
       </c>
       <c r="M22" t="n">
-        <v>-521.6799999999999</v>
+        <v>-478.76</v>
       </c>
     </row>
     <row r="23">
@@ -1461,25 +1461,25 @@
         <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>16000.31630670482</v>
+        <v>7001.052145694428</v>
       </c>
       <c r="H23" t="n">
-        <v>-650.0000196320225</v>
+        <v>-650.0000143552476</v>
       </c>
       <c r="I23" t="n">
-        <v>500.5829353951749</v>
+        <v>400.8530474728325</v>
       </c>
       <c r="J23" t="n">
         <v>0.5</v>
       </c>
       <c r="K23" t="n">
-        <v>553.0183546587466</v>
+        <v>428.3661755480705</v>
       </c>
       <c r="L23" t="n">
-        <v>11823.24</v>
+        <v>4783.6</v>
       </c>
       <c r="M23" t="n">
-        <v>-441.01</v>
+        <v>-407.92</v>
       </c>
     </row>
     <row r="24">
@@ -1506,25 +1506,25 @@
         <v>4</v>
       </c>
       <c r="G24" t="n">
-        <v>15000.49794579109</v>
+        <v>1301.005694904366</v>
       </c>
       <c r="H24" t="n">
-        <v>-850.0000179941949</v>
+        <v>-66.41361308858089</v>
       </c>
       <c r="I24" t="n">
-        <v>282.2697810936715</v>
+        <v>450.0447150940522</v>
       </c>
       <c r="J24" t="n">
         <v>0.5</v>
       </c>
       <c r="K24" t="n">
-        <v>337.0367045574487</v>
+        <v>423.2358566393677</v>
       </c>
       <c r="L24" t="n">
-        <v>8967.42</v>
+        <v>1043.96</v>
       </c>
       <c r="M24" t="n">
-        <v>-436.65</v>
+        <v>-59.69</v>
       </c>
     </row>
     <row r="25">
@@ -1551,25 +1551,25 @@
         <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>18000.15109334753</v>
+        <v>953.2875846635555</v>
       </c>
       <c r="H25" t="n">
-        <v>-150.0000435722097</v>
+        <v>-600.0000114576097</v>
       </c>
       <c r="I25" t="n">
-        <v>450.6047066177493</v>
+        <v>205.4458625081447</v>
       </c>
       <c r="J25" t="n">
         <v>0.5</v>
       </c>
       <c r="K25" t="n">
-        <v>472.0365350579011</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L25" t="n">
-        <v>13671.82</v>
+        <v>611.8200000000001</v>
       </c>
       <c r="M25" t="n">
-        <v>-87.18000000000001</v>
+        <v>-303.06</v>
       </c>
     </row>
     <row r="26">
@@ -1596,25 +1596,25 @@
         <v>6</v>
       </c>
       <c r="G26" t="n">
-        <v>1225.561337277732</v>
+        <v>1800.804604707089</v>
       </c>
       <c r="H26" t="n">
-        <v>-750.0000108217299</v>
+        <v>-150.0000270242403</v>
       </c>
       <c r="I26" t="n">
-        <v>284.8082402420575</v>
+        <v>280.7608868442319</v>
       </c>
       <c r="J26" t="n">
         <v>0.5</v>
       </c>
       <c r="K26" t="n">
-        <v>255.9977541431066</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L26" t="n">
-        <v>862.55</v>
+        <v>1338.59</v>
       </c>
       <c r="M26" t="n">
-        <v>-528.58</v>
+        <v>-74.62</v>
       </c>
     </row>
     <row r="27">
@@ -1641,25 +1641,25 @@
         <v>7</v>
       </c>
       <c r="G27" t="n">
-        <v>1308.014339610161</v>
+        <v>2800.266111677523</v>
       </c>
       <c r="H27" t="n">
-        <v>-450.0000150911927</v>
+        <v>-100.0000258654949</v>
       </c>
       <c r="I27" t="n">
-        <v>500.3405394971627</v>
+        <v>600.0786424741285</v>
       </c>
       <c r="J27" t="n">
         <v>0.5</v>
       </c>
       <c r="K27" t="n">
-        <v>448.3007253924136</v>
+        <v>602.1844988862963</v>
       </c>
       <c r="L27" t="n">
-        <v>1102.17</v>
+        <v>2358.24</v>
       </c>
       <c r="M27" t="n">
-        <v>-392.63</v>
+        <v>-68.84</v>
       </c>
     </row>
     <row r="28">
@@ -1686,25 +1686,25 @@
         <v>8</v>
       </c>
       <c r="G28" t="n">
-        <v>10000.23967230242</v>
+        <v>16000.31879978021</v>
       </c>
       <c r="H28" t="n">
-        <v>-50.00088892968448</v>
+        <v>-700.0000161074539</v>
       </c>
       <c r="I28" t="n">
-        <v>550.1933904039399</v>
+        <v>650.3989698248582</v>
       </c>
       <c r="J28" t="n">
         <v>0.5</v>
       </c>
       <c r="K28" t="n">
-        <v>591.2014890658488</v>
+        <v>702.6349485697167</v>
       </c>
       <c r="L28" t="n">
-        <v>7755.16</v>
+        <v>12844.9</v>
       </c>
       <c r="M28" t="n">
-        <v>-15.89</v>
+        <v>-544.24</v>
       </c>
     </row>
     <row r="29">
@@ -1731,25 +1731,25 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>1227.550021353459</v>
+        <v>13046.96148023747</v>
       </c>
       <c r="H29" t="n">
-        <v>-447.3366276080089</v>
+        <v>-79.6402725068038</v>
       </c>
       <c r="I29" t="n">
-        <v>270.8310616200254</v>
+        <v>109.9954851352551</v>
       </c>
       <c r="J29" t="n">
         <v>0.5</v>
       </c>
       <c r="K29" t="n">
-        <v>280.4314892296821</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L29" t="n">
-        <v>832.3099999999999</v>
+        <v>3148.88</v>
       </c>
       <c r="M29" t="n">
-        <v>-292.21</v>
+        <v>17.84</v>
       </c>
     </row>
     <row r="30">
@@ -1776,25 +1776,25 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>960.455888940106</v>
+        <v>1225.68608921074</v>
       </c>
       <c r="H30" t="n">
-        <v>-398.2625352704197</v>
+        <v>-547.6514396085951</v>
       </c>
       <c r="I30" t="n">
-        <v>233.6187560139707</v>
+        <v>462.6325435628922</v>
       </c>
       <c r="J30" t="n">
         <v>0.5</v>
       </c>
       <c r="K30" t="n">
-        <v>209.0212909830231</v>
+        <v>443.4011167993866</v>
       </c>
       <c r="L30" t="n">
-        <v>661.08</v>
+        <v>1017.71</v>
       </c>
       <c r="M30" t="n">
-        <v>-226.08</v>
+        <v>-439.11</v>
       </c>
     </row>
     <row r="31">
@@ -1821,25 +1821,25 @@
         <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>4063.319455222745</v>
+        <v>13032.25511269434</v>
       </c>
       <c r="H31" t="n">
-        <v>-647.7215321511085</v>
+        <v>-498.0287210202926</v>
       </c>
       <c r="I31" t="n">
-        <v>276.7132970187018</v>
+        <v>553.8675308112345</v>
       </c>
       <c r="J31" t="n">
         <v>0.5</v>
       </c>
       <c r="K31" t="n">
-        <v>295.6007445329244</v>
+        <v>591.2014890658488</v>
       </c>
       <c r="L31" t="n">
-        <v>2696.52</v>
+        <v>10044.43</v>
       </c>
       <c r="M31" t="n">
-        <v>-377.85</v>
+        <v>-363.92</v>
       </c>
     </row>
     <row r="32">
@@ -1866,25 +1866,25 @@
         <v>3</v>
       </c>
       <c r="G32" t="n">
-        <v>15027.11124671713</v>
+        <v>6057.31548080692</v>
       </c>
       <c r="H32" t="n">
-        <v>-547.6020144220137</v>
+        <v>-547.8748569533839</v>
       </c>
       <c r="I32" t="n">
-        <v>408.3801435284061</v>
+        <v>311.047839387307</v>
       </c>
       <c r="J32" t="n">
         <v>0.5</v>
       </c>
       <c r="K32" t="n">
-        <v>453.1473605746647</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L32" t="n">
-        <v>10671.2</v>
+        <v>4085.63</v>
       </c>
       <c r="M32" t="n">
-        <v>-358.76</v>
+        <v>-338.29</v>
       </c>
     </row>
     <row r="33">
@@ -1911,25 +1911,25 @@
         <v>4</v>
       </c>
       <c r="G33" t="n">
-        <v>14030.06219472345</v>
+        <v>1209.042552352751</v>
       </c>
       <c r="H33" t="n">
-        <v>-747.9220790941886</v>
+        <v>-55.73898185861684</v>
       </c>
       <c r="I33" t="n">
-        <v>275.0272814178894</v>
+        <v>368.4870223911405</v>
       </c>
       <c r="J33" t="n">
         <v>0.5</v>
       </c>
       <c r="K33" t="n">
-        <v>302.9006275609877</v>
+        <v>355.9504322854629</v>
       </c>
       <c r="L33" t="n">
-        <v>9206.110000000001</v>
+        <v>904.98</v>
       </c>
       <c r="M33" t="n">
-        <v>-451.6</v>
+        <v>-29.34</v>
       </c>
     </row>
     <row r="34">
@@ -1956,25 +1956,25 @@
         <v>5</v>
       </c>
       <c r="G34" t="n">
-        <v>17013.05278629104</v>
+        <v>941.3514482732445</v>
       </c>
       <c r="H34" t="n">
-        <v>-140.1436221297412</v>
+        <v>-499.9047126525462</v>
       </c>
       <c r="I34" t="n">
-        <v>354.2314988788998</v>
+        <v>155.2998775422665</v>
       </c>
       <c r="J34" t="n">
         <v>0.5</v>
       </c>
       <c r="K34" t="n">
-        <v>402.0604809124811</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L34" t="n">
-        <v>11586.37</v>
+        <v>374.75</v>
       </c>
       <c r="M34" t="n">
-        <v>-46.77</v>
+        <v>-100.91</v>
       </c>
     </row>
     <row r="35">
@@ -2001,25 +2001,25 @@
         <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>1163.196150517319</v>
+        <v>1710.367743176406</v>
       </c>
       <c r="H35" t="n">
-        <v>-648.0622376460287</v>
+        <v>-139.0746289883452</v>
       </c>
       <c r="I35" t="n">
-        <v>280.9474981131073</v>
+        <v>277.9596951593777</v>
       </c>
       <c r="J35" t="n">
         <v>0.5</v>
       </c>
       <c r="K35" t="n">
-        <v>255.9977541431066</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L35" t="n">
-        <v>822.71</v>
+        <v>1138.88</v>
       </c>
       <c r="M35" t="n">
-        <v>-464.65</v>
+        <v>-67.05</v>
       </c>
     </row>
     <row r="36">
@@ -2046,25 +2046,25 @@
         <v>7</v>
       </c>
       <c r="G36" t="n">
-        <v>1225.460107304382</v>
+        <v>2702.494429589704</v>
       </c>
       <c r="H36" t="n">
-        <v>-346.3656279792849</v>
+        <v>-89.82350350259199</v>
       </c>
       <c r="I36" t="n">
-        <v>425.8341753232367</v>
+        <v>503.8268420044408</v>
       </c>
       <c r="J36" t="n">
         <v>0.5</v>
       </c>
       <c r="K36" t="n">
-        <v>423.2358566393677</v>
+        <v>532.9018207393951</v>
       </c>
       <c r="L36" t="n">
-        <v>951.6</v>
+        <v>2117.78</v>
       </c>
       <c r="M36" t="n">
-        <v>-254.76</v>
+        <v>-53.02</v>
       </c>
     </row>
     <row r="37">
@@ -2091,25 +2091,25 @@
         <v>8</v>
       </c>
       <c r="G37" t="n">
-        <v>9018.149915238117</v>
+        <v>15023.11868049572</v>
       </c>
       <c r="H37" t="n">
-        <v>-40.03800260725571</v>
+        <v>-597.4204471109011</v>
       </c>
       <c r="I37" t="n">
-        <v>453.550975032902</v>
+        <v>556.5192155775079</v>
       </c>
       <c r="J37" t="n">
         <v>0.5</v>
       </c>
       <c r="K37" t="n">
-        <v>490.1983786827053</v>
+        <v>499.0314924731653</v>
       </c>
       <c r="L37" t="n">
-        <v>6637.25</v>
+        <v>12440.53</v>
       </c>
       <c r="M37" t="n">
-        <v>-7.9</v>
+        <v>-481.28</v>
       </c>
     </row>
     <row r="38">
@@ -2136,25 +2136,25 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>1154.523010984829</v>
+        <v>12157.71600259174</v>
       </c>
       <c r="H38" t="n">
-        <v>-349.9356601163787</v>
+        <v>-91.03429994640456</v>
       </c>
       <c r="I38" t="n">
-        <v>221.7498618066097</v>
+        <v>119.0525508970402</v>
       </c>
       <c r="J38" t="n">
         <v>0.5</v>
       </c>
       <c r="K38" t="n">
-        <v>219.2233794389425</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L38" t="n">
-        <v>751.36</v>
+        <v>3359.54</v>
       </c>
       <c r="M38" t="n">
-        <v>-160.77</v>
+        <v>51.83</v>
       </c>
     </row>
     <row r="39">
@@ -2181,25 +2181,25 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>1045.109912733941</v>
+        <v>1151.748523211517</v>
       </c>
       <c r="H39" t="n">
-        <v>-317.4287818727734</v>
+        <v>-450.435630989574</v>
       </c>
       <c r="I39" t="n">
-        <v>345.01543606427</v>
+        <v>386.5974240265782</v>
       </c>
       <c r="J39" t="n">
         <v>0.5</v>
       </c>
       <c r="K39" t="n">
-        <v>272.5304205830174</v>
+        <v>373.9086523062428</v>
       </c>
       <c r="L39" t="n">
-        <v>729.77</v>
+        <v>889.39</v>
       </c>
       <c r="M39" t="n">
-        <v>-204.79</v>
+        <v>-337.8</v>
       </c>
     </row>
     <row r="40">
@@ -2226,25 +2226,25 @@
         <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>3180.456085294249</v>
+        <v>12059.60463998207</v>
       </c>
       <c r="H40" t="n">
-        <v>-549.8405478229099</v>
+        <v>-399.6250655386197</v>
       </c>
       <c r="I40" t="n">
-        <v>209.6086236274533</v>
+        <v>463.269304455952</v>
       </c>
       <c r="J40" t="n">
         <v>0.5</v>
       </c>
       <c r="K40" t="n">
-        <v>238.320939301339</v>
+        <v>503.3899288706676</v>
       </c>
       <c r="L40" t="n">
-        <v>1809.59</v>
+        <v>9146.33</v>
       </c>
       <c r="M40" t="n">
-        <v>-241.36</v>
+        <v>-276.75</v>
       </c>
     </row>
     <row r="41">
@@ -2271,25 +2271,25 @@
         <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>14055.81913903972</v>
+        <v>5148.592042699991</v>
       </c>
       <c r="H41" t="n">
-        <v>-450.7863771590958</v>
+        <v>-452.2891667264399</v>
       </c>
       <c r="I41" t="n">
-        <v>322.4213773961978</v>
+        <v>232.7159793568155</v>
       </c>
       <c r="J41" t="n">
         <v>0.5</v>
       </c>
       <c r="K41" t="n">
-        <v>349.7595177200857</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L41" t="n">
-        <v>9444.049999999999</v>
+        <v>3070.31</v>
       </c>
       <c r="M41" t="n">
-        <v>-251.32</v>
+        <v>-228.29</v>
       </c>
     </row>
     <row r="42">
@@ -2316,25 +2316,25 @@
         <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>13056.72141139878</v>
+        <v>1130.299444159703</v>
       </c>
       <c r="H42" t="n">
-        <v>-650.1735395818637</v>
+        <v>-44.17968695509059</v>
       </c>
       <c r="I42" t="n">
-        <v>267.0621900221702</v>
+        <v>301.6671373490805</v>
       </c>
       <c r="J42" t="n">
         <v>0.5</v>
       </c>
       <c r="K42" t="n">
-        <v>316.996482935824</v>
+        <v>295.6007445329244</v>
       </c>
       <c r="L42" t="n">
-        <v>7874.82</v>
+        <v>825.42</v>
       </c>
       <c r="M42" t="n">
-        <v>-356.05</v>
+        <v>-1.91</v>
       </c>
     </row>
     <row r="43">
@@ -2361,25 +2361,25 @@
         <v>5</v>
       </c>
       <c r="G43" t="n">
-        <v>16035.16935401186</v>
+        <v>973.6358608025605</v>
       </c>
       <c r="H43" t="n">
-        <v>-130.3838050195878</v>
+        <v>-407.9523685995779</v>
       </c>
       <c r="I43" t="n">
-        <v>272.5379287260595</v>
+        <v>222.4545536729751</v>
       </c>
       <c r="J43" t="n">
         <v>0.5</v>
       </c>
       <c r="K43" t="n">
-        <v>316.996482935824</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L43" t="n">
-        <v>9673.27</v>
+        <v>664.16</v>
       </c>
       <c r="M43" t="n">
-        <v>-26.87</v>
+        <v>-234.04</v>
       </c>
     </row>
     <row r="44">
@@ -2406,25 +2406,25 @@
         <v>6</v>
       </c>
       <c r="G44" t="n">
-        <v>1113.833799275448</v>
+        <v>1615.421225981708</v>
       </c>
       <c r="H44" t="n">
-        <v>-547.6974132552073</v>
+        <v>-128.9112897928376</v>
       </c>
       <c r="I44" t="n">
-        <v>283.6714889449319</v>
+        <v>280.8506807929207</v>
       </c>
       <c r="J44" t="n">
         <v>0.5</v>
       </c>
       <c r="K44" t="n">
-        <v>264.3933435900673</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L44" t="n">
-        <v>800.4400000000001</v>
+        <v>1142.16</v>
       </c>
       <c r="M44" t="n">
-        <v>-361.95</v>
+        <v>-54.18</v>
       </c>
     </row>
     <row r="45">
@@ -2451,25 +2451,25 @@
         <v>7</v>
       </c>
       <c r="G45" t="n">
-        <v>1144.51154043352</v>
+        <v>2603.303689510175</v>
       </c>
       <c r="H45" t="n">
-        <v>-247.9265596112077</v>
+        <v>-79.9676996839266</v>
       </c>
       <c r="I45" t="n">
-        <v>352.6100672995741</v>
+        <v>415.2910762703204</v>
       </c>
       <c r="J45" t="n">
         <v>0.5</v>
       </c>
       <c r="K45" t="n">
-        <v>368.0199590525625</v>
+        <v>423.2358566393677</v>
       </c>
       <c r="L45" t="n">
-        <v>853.09</v>
+        <v>2016.66</v>
       </c>
       <c r="M45" t="n">
-        <v>-137.49</v>
+        <v>-29.86</v>
       </c>
     </row>
     <row r="46">
@@ -2496,25 +2496,25 @@
         <v>8</v>
       </c>
       <c r="G46" t="n">
-        <v>8053.466405593171</v>
+        <v>14051.78181473025</v>
       </c>
       <c r="H46" t="n">
-        <v>-40.63759875156118</v>
+        <v>-499.5528525781684</v>
       </c>
       <c r="I46" t="n">
-        <v>362.6224547489066</v>
+        <v>465.0331521314256</v>
       </c>
       <c r="J46" t="n">
         <v>0.5</v>
       </c>
       <c r="K46" t="n">
-        <v>385.4162169477469</v>
+        <v>503.3899288706676</v>
       </c>
       <c r="L46" t="n">
-        <v>5862.93</v>
+        <v>10609.8</v>
       </c>
       <c r="M46" t="n">
-        <v>-12.12</v>
+        <v>-354.3</v>
       </c>
     </row>
     <row r="47">
@@ -2541,13 +2541,13 @@
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>1104.555359467327</v>
+        <v>11062.35219511693</v>
       </c>
       <c r="H47" t="n">
-        <v>-260.07795319536</v>
+        <v>-97.85995401436402</v>
       </c>
       <c r="I47" t="n">
-        <v>196.6834362350917</v>
+        <v>129.7669178687061</v>
       </c>
       <c r="J47" t="n">
         <v>0.5</v>
@@ -2556,10 +2556,10 @@
         <v>198.2950076925505</v>
       </c>
       <c r="L47" t="n">
-        <v>601.98</v>
+        <v>3406.75</v>
       </c>
       <c r="M47" t="n">
-        <v>-92.34999999999999</v>
+        <v>87.73</v>
       </c>
     </row>
     <row r="48">
@@ -2586,25 +2586,25 @@
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>1085.055776571833</v>
+        <v>1080.220775636587</v>
       </c>
       <c r="H48" t="n">
-        <v>-227.1303304001195</v>
+        <v>-356.4689200906026</v>
       </c>
       <c r="I48" t="n">
-        <v>425.0951550908626</v>
+        <v>312.4226597556309</v>
       </c>
       <c r="J48" t="n">
         <v>0.5</v>
       </c>
       <c r="K48" t="n">
-        <v>412.7839753774575</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L48" t="n">
-        <v>853.04</v>
+        <v>780.09</v>
       </c>
       <c r="M48" t="n">
-        <v>-168.79</v>
+        <v>-249.87</v>
       </c>
     </row>
     <row r="49">
@@ -2631,25 +2631,25 @@
         <v>2</v>
       </c>
       <c r="G49" t="n">
-        <v>2372.330164877648</v>
+        <v>11093.00372454842</v>
       </c>
       <c r="H49" t="n">
-        <v>-457.9429669195246</v>
+        <v>-307.8451620964086</v>
       </c>
       <c r="I49" t="n">
-        <v>172.4489881267005</v>
+        <v>377.7097208463673</v>
       </c>
       <c r="J49" t="n">
         <v>0.5</v>
       </c>
       <c r="K49" t="n">
-        <v>186.9543261531214</v>
+        <v>412.7839753774575</v>
       </c>
       <c r="L49" t="n">
-        <v>1170.55</v>
+        <v>8021.33</v>
       </c>
       <c r="M49" t="n">
-        <v>-183.32</v>
+        <v>-195.07</v>
       </c>
     </row>
     <row r="50">
@@ -2676,25 +2676,25 @@
         <v>3</v>
       </c>
       <c r="G50" t="n">
-        <v>13088.2352115802</v>
+        <v>4262.062593572969</v>
       </c>
       <c r="H50" t="n">
-        <v>-358.7078756822841</v>
+        <v>-359.9502941912115</v>
       </c>
       <c r="I50" t="n">
-        <v>248.6002399424358</v>
+        <v>178.1105325099239</v>
       </c>
       <c r="J50" t="n">
         <v>0.5</v>
       </c>
       <c r="K50" t="n">
-        <v>288.1159665134826</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L50" t="n">
-        <v>7483.59</v>
+        <v>2066.8</v>
       </c>
       <c r="M50" t="n">
-        <v>-158.58</v>
+        <v>-97.02</v>
       </c>
     </row>
     <row r="51">
@@ -2721,25 +2721,25 @@
         <v>4</v>
       </c>
       <c r="G51" t="n">
-        <v>12073.34834162148</v>
+        <v>1051.477175150365</v>
       </c>
       <c r="H51" t="n">
-        <v>-551.4040351991001</v>
+        <v>-36.66069417959777</v>
       </c>
       <c r="I51" t="n">
-        <v>261.9867310162433</v>
+        <v>237.2892518259536</v>
       </c>
       <c r="J51" t="n">
         <v>0.5</v>
       </c>
       <c r="K51" t="n">
-        <v>302.9006275609877</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L51" t="n">
-        <v>7262.46</v>
+        <v>754.51</v>
       </c>
       <c r="M51" t="n">
-        <v>-283.9</v>
+        <v>26.21</v>
       </c>
     </row>
     <row r="52">
@@ -2766,25 +2766,25 @@
         <v>5</v>
       </c>
       <c r="G52" t="n">
-        <v>15070.83908320256</v>
+        <v>1082.535800751018</v>
       </c>
       <c r="H52" t="n">
-        <v>-123.4463708474557</v>
+        <v>-339.8372708751267</v>
       </c>
       <c r="I52" t="n">
-        <v>201.4511912863043</v>
+        <v>332.3615686700963</v>
       </c>
       <c r="J52" t="n">
         <v>0.5</v>
       </c>
       <c r="K52" t="n">
-        <v>247.317326764409</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L52" t="n">
-        <v>7613.07</v>
+        <v>831.49</v>
       </c>
       <c r="M52" t="n">
-        <v>18.69</v>
+        <v>-259.78</v>
       </c>
     </row>
     <row r="53">
@@ -2811,25 +2811,25 @@
         <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>1073.285828178853</v>
+        <v>1530.627057091059</v>
       </c>
       <c r="H53" t="n">
-        <v>-450.0308590386856</v>
+        <v>-118.9626789158286</v>
       </c>
       <c r="I53" t="n">
-        <v>287.8873572447072</v>
+        <v>278.6408443395536</v>
       </c>
       <c r="J53" t="n">
         <v>0.5</v>
       </c>
       <c r="K53" t="n">
-        <v>295.6007445329244</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L53" t="n">
-        <v>730.36</v>
+        <v>1031.05</v>
       </c>
       <c r="M53" t="n">
-        <v>-265.31</v>
+        <v>-36.6</v>
       </c>
     </row>
     <row r="54">
@@ -2856,25 +2856,25 @@
         <v>7</v>
       </c>
       <c r="G54" t="n">
-        <v>1073.538130532755</v>
+        <v>2504.954258586067</v>
       </c>
       <c r="H54" t="n">
-        <v>-158.5172101700599</v>
+        <v>-71.14259769750032</v>
       </c>
       <c r="I54" t="n">
-        <v>275.1516987530632</v>
+        <v>329.923315526312</v>
       </c>
       <c r="J54" t="n">
         <v>0.5</v>
       </c>
       <c r="K54" t="n">
-        <v>280.4314892296821</v>
+        <v>330.4916794875841</v>
       </c>
       <c r="L54" t="n">
-        <v>503.27</v>
+        <v>1789.14</v>
       </c>
       <c r="M54" t="n">
-        <v>-25.86</v>
+        <v>-32.56</v>
       </c>
     </row>
     <row r="55">
@@ -2901,25 +2901,25 @@
         <v>8</v>
       </c>
       <c r="G55" t="n">
-        <v>7122.128440392031</v>
+        <v>13068.86876026682</v>
       </c>
       <c r="H55" t="n">
-        <v>-48.57475780547482</v>
+        <v>-404.4518066335505</v>
       </c>
       <c r="I55" t="n">
-        <v>282.6858380767918</v>
+        <v>393.9962950688081</v>
       </c>
       <c r="J55" t="n">
         <v>0.5</v>
       </c>
       <c r="K55" t="n">
-        <v>323.8143915920092</v>
+        <v>418.0425819660462</v>
       </c>
       <c r="L55" t="n">
-        <v>4375.89</v>
+        <v>9610.18</v>
       </c>
       <c r="M55" t="n">
-        <v>38.18</v>
+        <v>-261.78</v>
       </c>
     </row>
     <row r="56">
@@ -2946,25 +2946,25 @@
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>1074.108222998502</v>
+        <v>9996.390145223857</v>
       </c>
       <c r="H56" t="n">
-        <v>-182.8690306611674</v>
+        <v>-105.9514926791</v>
       </c>
       <c r="I56" t="n">
-        <v>237.1857520765411</v>
+        <v>137.9681270943666</v>
       </c>
       <c r="J56" t="n">
         <v>0.5</v>
       </c>
       <c r="K56" t="n">
-        <v>186.9543261531214</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L56" t="n">
-        <v>754.54</v>
+        <v>4931.19</v>
       </c>
       <c r="M56" t="n">
-        <v>-108.83</v>
+        <v>22.97</v>
       </c>
     </row>
     <row r="57">
@@ -2991,25 +2991,25 @@
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>1101.53298304133</v>
+        <v>1022.722065201188</v>
       </c>
       <c r="H57" t="n">
-        <v>-136.8210435496686</v>
+        <v>-267.4711429832689</v>
       </c>
       <c r="I57" t="n">
-        <v>464.1424585748017</v>
+        <v>250.4409275158184</v>
       </c>
       <c r="J57" t="n">
         <v>0.5</v>
       </c>
       <c r="K57" t="n">
-        <v>453.1473605746647</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L57" t="n">
-        <v>883.95</v>
+        <v>632.09</v>
       </c>
       <c r="M57" t="n">
-        <v>-96.20999999999999</v>
+        <v>-137</v>
       </c>
     </row>
     <row r="58">
@@ -3036,25 +3036,25 @@
         <v>2</v>
       </c>
       <c r="G58" t="n">
-        <v>1681.461091782936</v>
+        <v>10121.10607008271</v>
       </c>
       <c r="H58" t="n">
-        <v>-375.0243058337589</v>
+        <v>-223.2198127021985</v>
       </c>
       <c r="I58" t="n">
-        <v>183.6696978869083</v>
+        <v>300.0645920555126</v>
       </c>
       <c r="J58" t="n">
         <v>0.5</v>
       </c>
       <c r="K58" t="n">
-        <v>247.317326764409</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L58" t="n">
-        <v>995.08</v>
+        <v>6513.56</v>
       </c>
       <c r="M58" t="n">
-        <v>-162.29</v>
+        <v>-94.44</v>
       </c>
     </row>
     <row r="59">
@@ -3081,25 +3081,25 @@
         <v>3</v>
       </c>
       <c r="G59" t="n">
-        <v>12115.49336681519</v>
+        <v>3426.43879921457</v>
       </c>
       <c r="H59" t="n">
-        <v>-275.9620712495983</v>
+        <v>-275.7743828486982</v>
       </c>
       <c r="I59" t="n">
-        <v>196.0554522863893</v>
+        <v>164.2584156044719</v>
       </c>
       <c r="J59" t="n">
         <v>0.5</v>
       </c>
       <c r="K59" t="n">
-        <v>238.320939301339</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L59" t="n">
-        <v>5847.92</v>
+        <v>1470.49</v>
       </c>
       <c r="M59" t="n">
-        <v>-54.94</v>
+        <v>-41.93</v>
       </c>
     </row>
     <row r="60">
@@ -3126,25 +3126,25 @@
         <v>4</v>
       </c>
       <c r="G60" t="n">
-        <v>11112.47526625858</v>
+        <v>993.3631107615867</v>
       </c>
       <c r="H60" t="n">
-        <v>-458.3043419532548</v>
+        <v>-41.72220254210079</v>
       </c>
       <c r="I60" t="n">
-        <v>255.6182991156836</v>
+        <v>201.9241925846892</v>
       </c>
       <c r="J60" t="n">
         <v>0.5</v>
       </c>
       <c r="K60" t="n">
-        <v>302.9006275609877</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L60" t="n">
-        <v>6346.32</v>
+        <v>694.13</v>
       </c>
       <c r="M60" t="n">
-        <v>-200.13</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="61">
@@ -3171,25 +3171,25 @@
         <v>5</v>
       </c>
       <c r="G61" t="n">
-        <v>14127.9838263161</v>
+        <v>1124.813799302195</v>
       </c>
       <c r="H61" t="n">
-        <v>-119.2958594171674</v>
+        <v>-252.995658034761</v>
       </c>
       <c r="I61" t="n">
-        <v>155.5777705450787</v>
+        <v>420.782424249975</v>
       </c>
       <c r="J61" t="n">
         <v>0.5</v>
       </c>
       <c r="K61" t="n">
-        <v>198.2950076925505</v>
+        <v>396.590015385101</v>
       </c>
       <c r="L61" t="n">
-        <v>5977.47</v>
+        <v>873.2</v>
       </c>
       <c r="M61" t="n">
-        <v>30.52</v>
+        <v>-189.46</v>
       </c>
     </row>
     <row r="62">
@@ -3216,25 +3216,25 @@
         <v>6</v>
       </c>
       <c r="G62" t="n">
-        <v>1037.784100476797</v>
+        <v>1439.839316828994</v>
       </c>
       <c r="H62" t="n">
-        <v>-357.6407070844916</v>
+        <v>-109.8471544405085</v>
       </c>
       <c r="I62" t="n">
-        <v>291.8748261874923</v>
+        <v>278.1746967412088</v>
       </c>
       <c r="J62" t="n">
         <v>0.5</v>
       </c>
       <c r="K62" t="n">
-        <v>288.1159665134826</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L62" t="n">
-        <v>756.02</v>
+        <v>1040.09</v>
       </c>
       <c r="M62" t="n">
-        <v>-223.01</v>
+        <v>-47.53</v>
       </c>
     </row>
     <row r="63">
@@ -3261,25 +3261,25 @@
         <v>7</v>
       </c>
       <c r="G63" t="n">
-        <v>1010.956020702704</v>
+        <v>2399.768567013934</v>
       </c>
       <c r="H63" t="n">
-        <v>-82.13157103119752</v>
+        <v>-65.49094404203781</v>
       </c>
       <c r="I63" t="n">
-        <v>200.7828073749423</v>
+        <v>255.9470890103535</v>
       </c>
       <c r="J63" t="n">
         <v>0.5</v>
       </c>
       <c r="K63" t="n">
-        <v>161.9071957960046</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L63" t="n">
-        <v>635.52</v>
+        <v>1498.9</v>
       </c>
       <c r="M63" t="n">
-        <v>-19.7</v>
+        <v>11.02</v>
       </c>
     </row>
     <row r="64">
@@ -3306,25 +3306,25 @@
         <v>8</v>
       </c>
       <c r="G64" t="n">
-        <v>6204.204908863602</v>
+        <v>12101.89071253337</v>
       </c>
       <c r="H64" t="n">
-        <v>-56.63556251718467</v>
+        <v>-317.0210794880514</v>
       </c>
       <c r="I64" t="n">
-        <v>221.3745205486637</v>
+        <v>319.3796326336638</v>
       </c>
       <c r="J64" t="n">
         <v>0.5</v>
       </c>
       <c r="K64" t="n">
-        <v>255.9977541431066</v>
+        <v>362.0354958462345</v>
       </c>
       <c r="L64" t="n">
-        <v>3241.8</v>
+        <v>7695.53</v>
       </c>
       <c r="M64" t="n">
-        <v>39.08</v>
+        <v>-154.48</v>
       </c>
     </row>
     <row r="65">
@@ -3351,25 +3351,25 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>1108.621345979138</v>
+        <v>8976.577863166549</v>
       </c>
       <c r="H65" t="n">
-        <v>-118.7694023144646</v>
+        <v>-115.4865786618157</v>
       </c>
       <c r="I65" t="n">
-        <v>327.1329365148243</v>
+        <v>145.645574899756</v>
       </c>
       <c r="J65" t="n">
         <v>0.5</v>
       </c>
       <c r="K65" t="n">
-        <v>323.8143915920092</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L65" t="n">
-        <v>838.98</v>
+        <v>3403.06</v>
       </c>
       <c r="M65" t="n">
-        <v>-47.19</v>
+        <v>33.84</v>
       </c>
     </row>
     <row r="66">
@@ -3396,25 +3396,25 @@
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>1068.877882332997</v>
+        <v>985.6631684384834</v>
       </c>
       <c r="H66" t="n">
-        <v>-51.60805737688763</v>
+        <v>-184.135283405567</v>
       </c>
       <c r="I66" t="n">
-        <v>385.0543431830129</v>
+        <v>219.0252115834215</v>
       </c>
       <c r="J66" t="n">
         <v>0.5</v>
       </c>
       <c r="K66" t="n">
-        <v>349.7595177200857</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L66" t="n">
-        <v>841.63</v>
+        <v>608.89</v>
       </c>
       <c r="M66" t="n">
-        <v>-25.66</v>
+        <v>-73.64</v>
       </c>
     </row>
     <row r="67">
@@ -3441,25 +3441,25 @@
         <v>2</v>
       </c>
       <c r="G67" t="n">
-        <v>1182.774792802041</v>
+        <v>9149.911154774773</v>
       </c>
       <c r="H67" t="n">
-        <v>-297.4018750391295</v>
+        <v>-147.9386034386221</v>
       </c>
       <c r="I67" t="n">
-        <v>255.7242910234097</v>
+        <v>235.3122205840817</v>
       </c>
       <c r="J67" t="n">
         <v>0.5</v>
       </c>
       <c r="K67" t="n">
-        <v>238.320939301339</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L67" t="n">
-        <v>817.26</v>
+        <v>5201.34</v>
       </c>
       <c r="M67" t="n">
-        <v>-184.8</v>
+        <v>-43.07</v>
       </c>
     </row>
     <row r="68">
@@ -3486,13 +3486,13 @@
         <v>3</v>
       </c>
       <c r="G68" t="n">
-        <v>11167.34380889362</v>
+        <v>2639.652859927551</v>
       </c>
       <c r="H68" t="n">
-        <v>-204.9918995505813</v>
+        <v>-211.2618638835868</v>
       </c>
       <c r="I68" t="n">
-        <v>166.8885707974329</v>
+        <v>209.3129769283018</v>
       </c>
       <c r="J68" t="n">
         <v>0.5</v>
@@ -3501,10 +3501,10 @@
         <v>219.2233794389425</v>
       </c>
       <c r="L68" t="n">
-        <v>4741.33</v>
+        <v>1550.48</v>
       </c>
       <c r="M68" t="n">
-        <v>15.99</v>
+        <v>-52.06</v>
       </c>
     </row>
     <row r="69">
@@ -3531,25 +3531,25 @@
         <v>4</v>
       </c>
       <c r="G69" t="n">
-        <v>10148.15556186103</v>
+        <v>960.4411204732279</v>
       </c>
       <c r="H69" t="n">
-        <v>-371.316410817029</v>
+        <v>-51.86419713639165</v>
       </c>
       <c r="I69" t="n">
-        <v>250.409722582026</v>
+        <v>203.0476679464295</v>
       </c>
       <c r="J69" t="n">
         <v>0.5</v>
       </c>
       <c r="K69" t="n">
-        <v>280.4314892296821</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L69" t="n">
-        <v>6167.11</v>
+        <v>589.6799999999999</v>
       </c>
       <c r="M69" t="n">
-        <v>-177.74</v>
+        <v>38.94</v>
       </c>
     </row>
     <row r="70">
@@ -3576,25 +3576,25 @@
         <v>5</v>
       </c>
       <c r="G70" t="n">
-        <v>13268.63448874786</v>
+        <v>1123.250489118219</v>
       </c>
       <c r="H70" t="n">
-        <v>-124.0242494463683</v>
+        <v>-160.418552219151</v>
       </c>
       <c r="I70" t="n">
-        <v>146.9211186182353</v>
+        <v>449.2914158082303</v>
       </c>
       <c r="J70" t="n">
         <v>0.5</v>
       </c>
       <c r="K70" t="n">
-        <v>198.2950076925505</v>
+        <v>433.4357742066306</v>
       </c>
       <c r="L70" t="n">
-        <v>5021.36</v>
+        <v>904.8</v>
       </c>
       <c r="M70" t="n">
-        <v>85.08</v>
+        <v>-108.86</v>
       </c>
     </row>
     <row r="71">
@@ -3621,25 +3621,25 @@
         <v>6</v>
       </c>
       <c r="G71" t="n">
-        <v>1022.280511830806</v>
+        <v>1348.379432507424</v>
       </c>
       <c r="H71" t="n">
-        <v>-271.8481214526447</v>
+        <v>-102.4924644161888</v>
       </c>
       <c r="I71" t="n">
-        <v>289.9403495216851</v>
+        <v>273.8692346923003</v>
       </c>
       <c r="J71" t="n">
         <v>0.5</v>
       </c>
       <c r="K71" t="n">
-        <v>255.9977541431066</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L71" t="n">
-        <v>757.41</v>
+        <v>953.24</v>
       </c>
       <c r="M71" t="n">
-        <v>-184.18</v>
+        <v>-34.11</v>
       </c>
     </row>
     <row r="72">
@@ -3666,25 +3666,25 @@
         <v>7</v>
       </c>
       <c r="G72" t="n">
-        <v>1115.876171313298</v>
+        <v>2298.711745538368</v>
       </c>
       <c r="H72" t="n">
-        <v>-42.54978909609345</v>
+        <v>-59.46157063534964</v>
       </c>
       <c r="I72" t="n">
-        <v>169.9433866644938</v>
+        <v>206.4054375177427</v>
       </c>
       <c r="J72" t="n">
         <v>0.5</v>
       </c>
       <c r="K72" t="n">
-        <v>198.2950076925505</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L72" t="n">
-        <v>546.01</v>
+        <v>1307</v>
       </c>
       <c r="M72" t="n">
-        <v>86.8</v>
+        <v>8.470000000000001</v>
       </c>
     </row>
     <row r="73">
@@ -3711,25 +3711,25 @@
         <v>8</v>
       </c>
       <c r="G73" t="n">
-        <v>5417.412109254704</v>
+        <v>11129.88535990703</v>
       </c>
       <c r="H73" t="n">
-        <v>-70.91637680465966</v>
+        <v>-237.7948422627874</v>
       </c>
       <c r="I73" t="n">
-        <v>179.7678598358075</v>
+        <v>256.0709530494113</v>
       </c>
       <c r="J73" t="n">
         <v>0.5</v>
       </c>
       <c r="K73" t="n">
-        <v>238.320939301339</v>
+        <v>302.9006275609877</v>
       </c>
       <c r="L73" t="n">
-        <v>2419.85</v>
+        <v>6301.24</v>
       </c>
       <c r="M73" t="n">
-        <v>70.17</v>
+        <v>-90.41</v>
       </c>
     </row>
     <row r="74">
@@ -3756,25 +3756,25 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>1100.319873146858</v>
+        <v>7730.354834235022</v>
       </c>
       <c r="H74" t="n">
-        <v>-52.63483648668915</v>
+        <v>-122.0583799601923</v>
       </c>
       <c r="I74" t="n">
-        <v>429.4233774025605</v>
+        <v>153.4729769766308</v>
       </c>
       <c r="J74" t="n">
         <v>0.5</v>
       </c>
       <c r="K74" t="n">
-        <v>438.4467588778851</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L74" t="n">
-        <v>853.9400000000001</v>
+        <v>2891.78</v>
       </c>
       <c r="M74" t="n">
-        <v>-4.43</v>
+        <v>-9.220000000000001</v>
       </c>
     </row>
     <row r="75">
@@ -3801,25 +3801,25 @@
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>1000.162851667229</v>
+        <v>998.9898372717624</v>
       </c>
       <c r="H75" t="n">
-        <v>19.26187403085362</v>
+        <v>-113.84404005753</v>
       </c>
       <c r="I75" t="n">
-        <v>262.291324706099</v>
+        <v>228.1353713444672</v>
       </c>
       <c r="J75" t="n">
         <v>0.5</v>
       </c>
       <c r="K75" t="n">
-        <v>264.3933435900673</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L75" t="n">
-        <v>750.79</v>
+        <v>685.05</v>
       </c>
       <c r="M75" t="n">
-        <v>33.39</v>
+        <v>-14.91</v>
       </c>
     </row>
     <row r="76">
@@ -3846,25 +3846,25 @@
         <v>2</v>
       </c>
       <c r="G76" t="n">
-        <v>794.7412488860888</v>
+        <v>8172.739780454887</v>
       </c>
       <c r="H76" t="n">
-        <v>-221.4905756579097</v>
+        <v>-91.71072173097019</v>
       </c>
       <c r="I76" t="n">
-        <v>303.366682616218</v>
+        <v>187.047220298663</v>
       </c>
       <c r="J76" t="n">
         <v>0.5</v>
       </c>
       <c r="K76" t="n">
-        <v>316.996482935824</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L76" t="n">
-        <v>527.3099999999999</v>
+        <v>3968.2</v>
       </c>
       <c r="M76" t="n">
-        <v>-112.65</v>
+        <v>22.93</v>
       </c>
     </row>
     <row r="77">
@@ -3891,25 +3891,25 @@
         <v>3</v>
       </c>
       <c r="G77" t="n">
-        <v>10209.58714905999</v>
+        <v>1896.934847896233</v>
       </c>
       <c r="H77" t="n">
-        <v>-160.2118737038618</v>
+        <v>-167.0502441092096</v>
       </c>
       <c r="I77" t="n">
-        <v>173.7152249715903</v>
+        <v>297.691882611655</v>
       </c>
       <c r="J77" t="n">
         <v>0.5</v>
       </c>
       <c r="K77" t="n">
-        <v>209.0212909830231</v>
+        <v>310.0286763918156</v>
       </c>
       <c r="L77" t="n">
-        <v>4096.85</v>
+        <v>1371.88</v>
       </c>
       <c r="M77" t="n">
-        <v>4.55</v>
+        <v>-79.87</v>
       </c>
     </row>
     <row r="78">
@@ -3936,25 +3936,25 @@
         <v>4</v>
       </c>
       <c r="G78" t="n">
-        <v>9185.863217613607</v>
+        <v>948.4279449243487</v>
       </c>
       <c r="H78" t="n">
-        <v>-293.9280276816599</v>
+        <v>-62.11783961966383</v>
       </c>
       <c r="I78" t="n">
-        <v>244.9531663939825</v>
+        <v>236.0572052879782</v>
       </c>
       <c r="J78" t="n">
         <v>0.5</v>
       </c>
       <c r="K78" t="n">
-        <v>272.5304205830174</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L78" t="n">
-        <v>5523.29</v>
+        <v>615.36</v>
       </c>
       <c r="M78" t="n">
-        <v>-109.9</v>
+        <v>-35.51</v>
       </c>
     </row>
     <row r="79">
@@ -3981,25 +3981,25 @@
         <v>5</v>
       </c>
       <c r="G79" t="n">
-        <v>12488.60743468215</v>
+        <v>1093.077259066999</v>
       </c>
       <c r="H79" t="n">
-        <v>-132.8454423531026</v>
+        <v>-74.78251139051456</v>
       </c>
       <c r="I79" t="n">
-        <v>178.626118599424</v>
+        <v>383.6775482803339</v>
       </c>
       <c r="J79" t="n">
         <v>0.5</v>
       </c>
       <c r="K79" t="n">
-        <v>219.2233794389425</v>
+        <v>373.9086523062428</v>
       </c>
       <c r="L79" t="n">
-        <v>5880.41</v>
+        <v>849.54</v>
       </c>
       <c r="M79" t="n">
-        <v>64.34999999999999</v>
+        <v>-32.13</v>
       </c>
     </row>
     <row r="80">
@@ -4026,13 +4026,13 @@
         <v>6</v>
       </c>
       <c r="G80" t="n">
-        <v>1003.008450918537</v>
+        <v>1263.461006849141</v>
       </c>
       <c r="H80" t="n">
-        <v>-189.9751250500088</v>
+        <v>-94.03020225474324</v>
       </c>
       <c r="I80" t="n">
-        <v>288.1554011826607</v>
+        <v>281.7508111423556</v>
       </c>
       <c r="J80" t="n">
         <v>0.5</v>
@@ -4041,10 +4041,10 @@
         <v>255.9977541431066</v>
       </c>
       <c r="L80" t="n">
-        <v>564.62</v>
+        <v>923.4</v>
       </c>
       <c r="M80" t="n">
-        <v>-96.88</v>
+        <v>-39.42</v>
       </c>
     </row>
     <row r="81">
@@ -4071,25 +4071,25 @@
         <v>7</v>
       </c>
       <c r="G81" t="n">
-        <v>1181.065570236721</v>
+        <v>2215.082600809384</v>
       </c>
       <c r="H81" t="n">
-        <v>-21.32054770082142</v>
+        <v>-65.1736090109699</v>
       </c>
       <c r="I81" t="n">
-        <v>282.728399787752</v>
+        <v>180.9651670332532</v>
       </c>
       <c r="J81" t="n">
         <v>0.5</v>
       </c>
       <c r="K81" t="n">
-        <v>288.1159665134826</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L81" t="n">
-        <v>834.77</v>
+        <v>2119.21</v>
       </c>
       <c r="M81" t="n">
-        <v>21.28</v>
+        <v>42.23</v>
       </c>
     </row>
     <row r="82">
@@ -4116,25 +4116,25 @@
         <v>8</v>
       </c>
       <c r="G82" t="n">
-        <v>4728.947171287716</v>
+        <v>10174.60141269085</v>
       </c>
       <c r="H82" t="n">
-        <v>-84.62495419669982</v>
+        <v>-172.2389656368968</v>
       </c>
       <c r="I82" t="n">
-        <v>166.4095734236816</v>
+        <v>202.5363641500476</v>
       </c>
       <c r="J82" t="n">
         <v>0.5</v>
       </c>
       <c r="K82" t="n">
-        <v>209.0212909830231</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L82" t="n">
-        <v>1908.02</v>
+        <v>5073.2</v>
       </c>
       <c r="M82" t="n">
-        <v>58.01</v>
+        <v>-22.98</v>
       </c>
     </row>
     <row r="83">
@@ -4161,25 +4161,25 @@
         <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>1029.744499026845</v>
+        <v>6679.742734420605</v>
       </c>
       <c r="H83" t="n">
-        <v>-4.205286051695907</v>
+        <v>-129.4365454467413</v>
       </c>
       <c r="I83" t="n">
-        <v>394.8481485095107</v>
+        <v>162.4082351183447</v>
       </c>
       <c r="J83" t="n">
         <v>0.5</v>
       </c>
       <c r="K83" t="n">
-        <v>362.0354958462345</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L83" t="n">
-        <v>782.15</v>
+        <v>2453.43</v>
       </c>
       <c r="M83" t="n">
-        <v>19.22</v>
+        <v>50.84</v>
       </c>
     </row>
     <row r="84">
@@ -4206,25 +4206,25 @@
         <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>886.2219016529375</v>
+        <v>1049.577375560766</v>
       </c>
       <c r="H84" t="n">
-        <v>56.74687577859731</v>
+        <v>-57.93580190153996</v>
       </c>
       <c r="I84" t="n">
-        <v>135.6061128129603</v>
+        <v>289.1746264512425</v>
       </c>
       <c r="J84" t="n">
         <v>0.5</v>
       </c>
       <c r="K84" t="n">
-        <v>198.2950076925505</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L84" t="n">
-        <v>401.59</v>
+        <v>715.24</v>
       </c>
       <c r="M84" t="n">
-        <v>102.75</v>
+        <v>-8.17</v>
       </c>
     </row>
     <row r="85">
@@ -4251,25 +4251,25 @@
         <v>2</v>
       </c>
       <c r="G85" t="n">
-        <v>549.2373016955273</v>
+        <v>7201.578965891139</v>
       </c>
       <c r="H85" t="n">
-        <v>-141.1787001622592</v>
+        <v>-54.85534803329845</v>
       </c>
       <c r="I85" t="n">
-        <v>360.8110339817266</v>
+        <v>167.0509018539257</v>
       </c>
       <c r="J85" t="n">
         <v>0.5</v>
       </c>
       <c r="K85" t="n">
-        <v>368.0199590525625</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L85" t="n">
-        <v>360.23</v>
+        <v>3304.93</v>
       </c>
       <c r="M85" t="n">
-        <v>-60.59</v>
+        <v>43.72</v>
       </c>
     </row>
     <row r="86">
@@ -4296,25 +4296,25 @@
         <v>3</v>
       </c>
       <c r="G86" t="n">
-        <v>9320.89630037596</v>
+        <v>1153.655780451532</v>
       </c>
       <c r="H86" t="n">
-        <v>-154.001901766165</v>
+        <v>-123.5487997657273</v>
       </c>
       <c r="I86" t="n">
-        <v>208.8952693873649</v>
+        <v>383.1039828470152</v>
       </c>
       <c r="J86" t="n">
         <v>0.5</v>
       </c>
       <c r="K86" t="n">
-        <v>255.9977541431066</v>
+        <v>396.590015385101</v>
       </c>
       <c r="L86" t="n">
-        <v>4653.16</v>
+        <v>863.78</v>
       </c>
       <c r="M86" t="n">
-        <v>-7.06</v>
+        <v>-66.92</v>
       </c>
     </row>
     <row r="87">
@@ -4341,25 +4341,25 @@
         <v>4</v>
       </c>
       <c r="G87" t="n">
-        <v>8214.700892530696</v>
+        <v>964.9520007103177</v>
       </c>
       <c r="H87" t="n">
-        <v>-220.5503468099015</v>
+        <v>-73.92988867493112</v>
       </c>
       <c r="I87" t="n">
-        <v>242.8832267190845</v>
+        <v>269.3653491052601</v>
       </c>
       <c r="J87" t="n">
         <v>0.5</v>
       </c>
       <c r="K87" t="n">
-        <v>255.9977541431066</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L87" t="n">
-        <v>5169.95</v>
+        <v>608.14</v>
       </c>
       <c r="M87" t="n">
-        <v>-102.07</v>
+        <v>4.17</v>
       </c>
     </row>
     <row r="88">
@@ -4386,25 +4386,25 @@
         <v>5</v>
       </c>
       <c r="G88" t="n">
-        <v>11805.39278822713</v>
+        <v>1030.199254376652</v>
       </c>
       <c r="H88" t="n">
-        <v>-146.0584740308419</v>
+        <v>-2.941570257932085</v>
       </c>
       <c r="I88" t="n">
-        <v>224.3709709143997</v>
+        <v>267.4905745735769</v>
       </c>
       <c r="J88" t="n">
         <v>0.5</v>
       </c>
       <c r="K88" t="n">
-        <v>255.9977541431066</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L88" t="n">
-        <v>6894.62</v>
+        <v>710.48</v>
       </c>
       <c r="M88" t="n">
-        <v>-35.8</v>
+        <v>60.12</v>
       </c>
     </row>
     <row r="89">
@@ -4431,25 +4431,25 @@
         <v>6</v>
       </c>
       <c r="G89" t="n">
-        <v>983.0638262370773</v>
+        <v>1178.906678393879</v>
       </c>
       <c r="H89" t="n">
-        <v>-112.3743091161412</v>
+        <v>-86.98887644845881</v>
       </c>
       <c r="I89" t="n">
-        <v>293.755031938959</v>
+        <v>287.2148691201639</v>
       </c>
       <c r="J89" t="n">
         <v>0.5</v>
       </c>
       <c r="K89" t="n">
-        <v>302.9006275609877</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L89" t="n">
-        <v>709.05</v>
+        <v>839.86</v>
       </c>
       <c r="M89" t="n">
-        <v>-6.6</v>
+        <v>-37.15</v>
       </c>
     </row>
     <row r="90">
@@ -4476,25 +4476,25 @@
         <v>7</v>
       </c>
       <c r="G90" t="n">
-        <v>1236.590228693857</v>
+        <v>2142.515168320037</v>
       </c>
       <c r="H90" t="n">
-        <v>-57.44002660882258</v>
+        <v>-72.89604847396375</v>
       </c>
       <c r="I90" t="n">
-        <v>336.7586676284949</v>
+        <v>192.3066843837999</v>
       </c>
       <c r="J90" t="n">
         <v>0.5</v>
       </c>
       <c r="K90" t="n">
-        <v>323.8143915920092</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L90" t="n">
-        <v>927.83</v>
+        <v>1270.99</v>
       </c>
       <c r="M90" t="n">
-        <v>-15.01</v>
+        <v>-16.25</v>
       </c>
     </row>
     <row r="91">
@@ -4521,13 +4521,13 @@
         <v>8</v>
       </c>
       <c r="G91" t="n">
-        <v>4174.837979324144</v>
+        <v>9231.427182341828</v>
       </c>
       <c r="H91" t="n">
-        <v>-99.20002362970672</v>
+        <v>-120.7163624288772</v>
       </c>
       <c r="I91" t="n">
-        <v>170.1730697702876</v>
+        <v>168.7009603379393</v>
       </c>
       <c r="J91" t="n">
         <v>0.5</v>
@@ -4536,10 +4536,10 @@
         <v>209.0212909830231</v>
       </c>
       <c r="L91" t="n">
-        <v>1813.89</v>
+        <v>4226.75</v>
       </c>
       <c r="M91" t="n">
-        <v>56.99</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="92">
@@ -4566,25 +4566,25 @@
         <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>941.3311469807156</v>
+        <v>5617.332938579431</v>
       </c>
       <c r="H92" t="n">
-        <v>4.167713084948893</v>
+        <v>-133.8292902717329</v>
       </c>
       <c r="I92" t="n">
-        <v>261.9403372599812</v>
+        <v>172.2454659385792</v>
       </c>
       <c r="J92" t="n">
         <v>0.5</v>
       </c>
       <c r="K92" t="n">
-        <v>264.3933435900673</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L92" t="n">
-        <v>642.01</v>
+        <v>2773.91</v>
       </c>
       <c r="M92" t="n">
-        <v>40.38</v>
+        <v>-26.23</v>
       </c>
     </row>
     <row r="93">
@@ -4611,25 +4611,25 @@
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>843.019847229792</v>
+        <v>1103.836964676151</v>
       </c>
       <c r="H93" t="n">
-        <v>37.97782453582677</v>
+        <v>-39.54127393015071</v>
       </c>
       <c r="I93" t="n">
-        <v>106.3259955017865</v>
+        <v>394.4287036971203</v>
       </c>
       <c r="J93" t="n">
         <v>0.5</v>
       </c>
       <c r="K93" t="n">
-        <v>114.4856760702529</v>
+        <v>385.4162169477469</v>
       </c>
       <c r="L93" t="n">
-        <v>46.13</v>
+        <v>889.25</v>
       </c>
       <c r="M93" t="n">
-        <v>79.58</v>
+        <v>-1.17</v>
       </c>
     </row>
     <row r="94">
@@ -4656,25 +4656,25 @@
         <v>2</v>
       </c>
       <c r="G94" t="n">
-        <v>562.2679543294247</v>
+        <v>6354.804093327559</v>
       </c>
       <c r="H94" t="n">
-        <v>-71.4736504712365</v>
+        <v>-57.58146918787546</v>
       </c>
       <c r="I94" t="n">
-        <v>334.3798651198496</v>
+        <v>179.6504578397151</v>
       </c>
       <c r="J94" t="n">
         <v>0.5</v>
       </c>
       <c r="K94" t="n">
-        <v>330.4916794875841</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L94" t="n">
-        <v>363.71</v>
+        <v>3110.14</v>
       </c>
       <c r="M94" t="n">
-        <v>0.5</v>
+        <v>45.01</v>
       </c>
     </row>
     <row r="95">
@@ -4701,25 +4701,25 @@
         <v>3</v>
       </c>
       <c r="G95" t="n">
-        <v>8464.907671172601</v>
+        <v>534.6759451121488</v>
       </c>
       <c r="H95" t="n">
-        <v>-157.5390190014762</v>
+        <v>-68.07543078208008</v>
       </c>
       <c r="I95" t="n">
-        <v>268.390225501604</v>
+        <v>384.0260855502955</v>
       </c>
       <c r="J95" t="n">
         <v>0.5</v>
       </c>
       <c r="K95" t="n">
-        <v>302.9006275609877</v>
+        <v>362.0354958462345</v>
       </c>
       <c r="L95" t="n">
-        <v>5194.51</v>
+        <v>312.64</v>
       </c>
       <c r="M95" t="n">
-        <v>-36.29</v>
+        <v>-15.99</v>
       </c>
     </row>
     <row r="96">
@@ -4746,25 +4746,25 @@
         <v>4</v>
       </c>
       <c r="G96" t="n">
-        <v>7224.10123059694</v>
+        <v>1003.192647082326</v>
       </c>
       <c r="H96" t="n">
-        <v>-160.6177910207787</v>
+        <v>-74.14173786160116</v>
       </c>
       <c r="I96" t="n">
-        <v>243.1781909370315</v>
+        <v>339.6836054628201</v>
       </c>
       <c r="J96" t="n">
         <v>0.5</v>
       </c>
       <c r="K96" t="n">
-        <v>255.9977541431066</v>
+        <v>302.9006275609877</v>
       </c>
       <c r="L96" t="n">
-        <v>4295.18</v>
+        <v>719.4400000000001</v>
       </c>
       <c r="M96" t="n">
-        <v>-47.69</v>
+        <v>-36.26</v>
       </c>
     </row>
     <row r="97">
@@ -4791,25 +4791,25 @@
         <v>5</v>
       </c>
       <c r="G97" t="n">
-        <v>11069.57006895396</v>
+        <v>934.7345346945779</v>
       </c>
       <c r="H97" t="n">
-        <v>-157.911232219275</v>
+        <v>39.55032836788105</v>
       </c>
       <c r="I97" t="n">
-        <v>270.0631741762186</v>
+        <v>132.5800471057387</v>
       </c>
       <c r="J97" t="n">
         <v>0.5</v>
       </c>
       <c r="K97" t="n">
-        <v>302.9006275609877</v>
+        <v>132.1966717950337</v>
       </c>
       <c r="L97" t="n">
-        <v>6825.09</v>
+        <v>382.42</v>
       </c>
       <c r="M97" t="n">
-        <v>-52.21</v>
+        <v>99.52</v>
       </c>
     </row>
     <row r="98">
@@ -4836,25 +4836,25 @@
         <v>6</v>
       </c>
       <c r="G98" t="n">
-        <v>1056.147859408361</v>
+        <v>1104.430089366956</v>
       </c>
       <c r="H98" t="n">
-        <v>-49.01982932370842</v>
+        <v>-79.16947248308036</v>
       </c>
       <c r="I98" t="n">
-        <v>302.3897176540909</v>
+        <v>298.0322256331597</v>
       </c>
       <c r="J98" t="n">
         <v>0.5</v>
       </c>
       <c r="K98" t="n">
-        <v>198.2950076925505</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L98" t="n">
-        <v>655.91</v>
+        <v>755.75</v>
       </c>
       <c r="M98" t="n">
-        <v>30.35</v>
+        <v>-22.24</v>
       </c>
     </row>
     <row r="99">
@@ -4881,25 +4881,25 @@
         <v>7</v>
       </c>
       <c r="G99" t="n">
-        <v>1226.350551350044</v>
+        <v>2051.034839792969</v>
       </c>
       <c r="H99" t="n">
-        <v>-94.44584652112869</v>
+        <v>-83.93418281636359</v>
       </c>
       <c r="I99" t="n">
-        <v>354.3925417227343</v>
+        <v>215.2141360603577</v>
       </c>
       <c r="J99" t="n">
         <v>0.5</v>
       </c>
       <c r="K99" t="n">
-        <v>337.0367045574487</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L99" t="n">
-        <v>949.85</v>
+        <v>1166.53</v>
       </c>
       <c r="M99" t="n">
-        <v>-65.70999999999999</v>
+        <v>24.82</v>
       </c>
     </row>
     <row r="100">
@@ -4926,25 +4926,25 @@
         <v>8</v>
       </c>
       <c r="G100" t="n">
-        <v>3708.675325906923</v>
+        <v>8266.264942713562</v>
       </c>
       <c r="H100" t="n">
-        <v>-112.641107412126</v>
+        <v>-95.37308012207575</v>
       </c>
       <c r="I100" t="n">
-        <v>197.9729531418009</v>
+        <v>165.382614517106</v>
       </c>
       <c r="J100" t="n">
         <v>0.5</v>
       </c>
       <c r="K100" t="n">
-        <v>219.2233794389425</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L100" t="n">
-        <v>1961.89</v>
+        <v>3748.71</v>
       </c>
       <c r="M100" t="n">
-        <v>15.82</v>
+        <v>67.92</v>
       </c>
     </row>
   </sheetData>
@@ -5025,7 +5025,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>52</v>
+        <v>96</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -5041,36 +5041,36 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G2" t="n">
-        <v>1073.538130532755</v>
+        <v>1104.430089366956</v>
       </c>
       <c r="H2" t="n">
-        <v>-158.5172101700599</v>
+        <v>-79.16947248308036</v>
       </c>
       <c r="I2" t="n">
-        <v>275.1516987530632</v>
+        <v>298.0322256331597</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>280.4314892296821</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L2" t="n">
-        <v>503.27</v>
+        <v>755.75</v>
       </c>
       <c r="M2" t="n">
-        <v>-25.86</v>
+        <v>-22.24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -5086,36 +5086,36 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1068.877882332997</v>
+        <v>998.9898372717624</v>
       </c>
       <c r="H3" t="n">
-        <v>-51.60805737688763</v>
+        <v>-113.84404005753</v>
       </c>
       <c r="I3" t="n">
-        <v>385.0543431830129</v>
+        <v>228.1353713444672</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>349.7595177200857</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L3" t="n">
-        <v>841.63</v>
+        <v>685.05</v>
       </c>
       <c r="M3" t="n">
-        <v>-25.66</v>
+        <v>-14.91</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -5131,31 +5131,31 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>1010.956020702704</v>
+        <v>1049.577375560766</v>
       </c>
       <c r="H4" t="n">
-        <v>-82.13157103119752</v>
+        <v>-57.93580190153996</v>
       </c>
       <c r="I4" t="n">
-        <v>200.7828073749423</v>
+        <v>289.1746264512425</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>161.9071957960046</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L4" t="n">
-        <v>635.52</v>
+        <v>715.24</v>
       </c>
       <c r="M4" t="n">
-        <v>-19.7</v>
+        <v>-8.17</v>
       </c>
     </row>
   </sheetData>
@@ -5268,31 +5268,31 @@
         <v>-21.42555</v>
       </c>
       <c r="G2" t="n">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="H2" t="n">
-        <v>92</v>
+        <v>38</v>
       </c>
       <c r="I2" t="n">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="J2" t="n">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="K2" t="n">
-        <v>-97</v>
+        <v>-83</v>
       </c>
       <c r="L2" t="n">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="M2" t="n">
-        <v>2.29</v>
+        <v>-3.18</v>
       </c>
       <c r="N2" t="n">
-        <v>30.8845871404001</v>
+        <v>30.87637282532287</v>
       </c>
       <c r="O2" t="n">
-        <v>78.0067935064543</v>
+        <v>74.38660067954987</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: results graph display
</commit_message>
<xml_diff>
--- a/test_alldata.xlsx
+++ b/test_alldata.xlsx
@@ -516,25 +516,25 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>16000</v>
+        <v>13000</v>
       </c>
       <c r="H2" t="n">
-        <v>-50</v>
+        <v>-100</v>
       </c>
       <c r="I2" t="n">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>147.8003722664622</v>
+        <v>494.634653528818</v>
       </c>
       <c r="L2" t="n">
-        <v>3434.76</v>
+        <v>9486.24</v>
       </c>
       <c r="M2" t="n">
-        <v>89.78</v>
+        <v>-37.34</v>
       </c>
     </row>
     <row r="3">
@@ -561,25 +561,25 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="H3" t="n">
-        <v>-650</v>
+        <v>-350</v>
       </c>
       <c r="I3" t="n">
-        <v>750</v>
+        <v>700</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>733.0660072843224</v>
+        <v>686.9140564215176</v>
       </c>
       <c r="L3" t="n">
-        <v>1302.14</v>
+        <v>1040.18</v>
       </c>
       <c r="M3" t="n">
-        <v>-578.55</v>
+        <v>-307.9</v>
       </c>
     </row>
     <row r="4">
@@ -606,25 +606,25 @@
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>16000</v>
+        <v>8000</v>
       </c>
       <c r="H4" t="n">
-        <v>-600</v>
+        <v>-250</v>
       </c>
       <c r="I4" t="n">
-        <v>850</v>
+        <v>650</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>869.3878716987178</v>
+        <v>674.0734091148975</v>
       </c>
       <c r="L4" t="n">
-        <v>13774.54</v>
+        <v>6684.26</v>
       </c>
       <c r="M4" t="n">
-        <v>-515.13</v>
+        <v>-195.63</v>
       </c>
     </row>
     <row r="5">
@@ -654,22 +654,22 @@
         <v>9000</v>
       </c>
       <c r="H5" t="n">
-        <v>-650</v>
+        <v>-250</v>
       </c>
       <c r="I5" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="J5" t="n">
         <v>0.5</v>
       </c>
       <c r="K5" t="n">
-        <v>627.0638729490693</v>
+        <v>727.081694872685</v>
       </c>
       <c r="L5" t="n">
-        <v>7387.98</v>
+        <v>7549.2</v>
       </c>
       <c r="M5" t="n">
-        <v>-517.85</v>
+        <v>-194.39</v>
       </c>
     </row>
     <row r="6">
@@ -696,25 +696,25 @@
         <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>1500</v>
+        <v>1100</v>
       </c>
       <c r="H6" t="n">
-        <v>-50</v>
+        <v>-250</v>
       </c>
       <c r="I6" t="n">
-        <v>650</v>
+        <v>350</v>
       </c>
       <c r="J6" t="n">
         <v>0.5</v>
       </c>
       <c r="K6" t="n">
-        <v>660.9833589751682</v>
+        <v>355.9504322854629</v>
       </c>
       <c r="L6" t="n">
-        <v>1261.13</v>
+        <v>850.78</v>
       </c>
       <c r="M6" t="n">
-        <v>-21.37</v>
+        <v>-167.07</v>
       </c>
     </row>
     <row r="7">
@@ -741,25 +741,25 @@
         <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>1100</v>
+        <v>5000</v>
       </c>
       <c r="H7" t="n">
-        <v>-600</v>
+        <v>-850</v>
       </c>
       <c r="I7" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="J7" t="n">
         <v>0.5</v>
       </c>
       <c r="K7" t="n">
-        <v>385.4162169477469</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L7" t="n">
-        <v>854.63</v>
+        <v>3721.11</v>
       </c>
       <c r="M7" t="n">
-        <v>-462.13</v>
+        <v>-598.1900000000001</v>
       </c>
     </row>
     <row r="8">
@@ -786,25 +786,25 @@
         <v>6</v>
       </c>
       <c r="G8" t="n">
-        <v>2000</v>
+        <v>900</v>
       </c>
       <c r="H8" t="n">
         <v>-150</v>
       </c>
       <c r="I8" t="n">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="J8" t="n">
         <v>0.5</v>
       </c>
       <c r="K8" t="n">
-        <v>310.0286763918156</v>
+        <v>428.3661755480705</v>
       </c>
       <c r="L8" t="n">
-        <v>1371.01</v>
+        <v>733.8200000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>-52.2</v>
+        <v>-96.70999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -831,25 +831,25 @@
         <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="H9" t="n">
-        <v>-100</v>
+        <v>-800</v>
       </c>
       <c r="I9" t="n">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="J9" t="n">
         <v>0.5</v>
       </c>
       <c r="K9" t="n">
-        <v>804.1209618249621</v>
+        <v>310.0286763918156</v>
       </c>
       <c r="L9" t="n">
-        <v>2634.42</v>
+        <v>2799.97</v>
       </c>
       <c r="M9" t="n">
-        <v>-74.76000000000001</v>
+        <v>-519.8099999999999</v>
       </c>
     </row>
     <row r="10">
@@ -876,25 +876,25 @@
         <v>8</v>
       </c>
       <c r="G10" t="n">
-        <v>18000</v>
+        <v>800</v>
       </c>
       <c r="H10" t="n">
-        <v>-700</v>
+        <v>-250</v>
       </c>
       <c r="I10" t="n">
-        <v>850</v>
+        <v>100</v>
       </c>
       <c r="J10" t="n">
         <v>0.5</v>
       </c>
       <c r="K10" t="n">
-        <v>891.7153029597591</v>
+        <v>114.4856760702529</v>
       </c>
       <c r="L10" t="n">
-        <v>15279.63</v>
+        <v>321.13</v>
       </c>
       <c r="M10" t="n">
-        <v>-584.6900000000001</v>
+        <v>68.23999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -921,25 +921,25 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="H11" t="n">
-        <v>-60</v>
+        <v>-110</v>
       </c>
       <c r="I11" t="n">
-        <v>90</v>
+        <v>350</v>
       </c>
       <c r="J11" t="n">
         <v>0.5</v>
       </c>
       <c r="K11" t="n">
-        <v>147.8003722664622</v>
+        <v>385.4162169477469</v>
       </c>
       <c r="L11" t="n">
-        <v>2750.88</v>
+        <v>8181.54</v>
       </c>
       <c r="M11" t="n">
-        <v>63.84</v>
+        <v>-38.01</v>
       </c>
     </row>
     <row r="12">
@@ -966,25 +966,25 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>1400</v>
+        <v>1100</v>
       </c>
       <c r="H12" t="n">
-        <v>-750</v>
+        <v>-450</v>
       </c>
       <c r="I12" t="n">
-        <v>650</v>
+        <v>600</v>
       </c>
       <c r="J12" t="n">
         <v>0.5</v>
       </c>
       <c r="K12" t="n">
-        <v>605.8012551219755</v>
+        <v>594.8850230776515</v>
       </c>
       <c r="L12" t="n">
-        <v>1250.44</v>
+        <v>911.09</v>
       </c>
       <c r="M12" t="n">
-        <v>-682.08</v>
+        <v>-371.24</v>
       </c>
     </row>
     <row r="13">
@@ -1011,25 +1011,25 @@
         <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>15000</v>
+        <v>7000</v>
       </c>
       <c r="H13" t="n">
-        <v>-700</v>
+        <v>-260</v>
       </c>
       <c r="I13" t="n">
-        <v>750</v>
+        <v>550</v>
       </c>
       <c r="J13" t="n">
         <v>0.5</v>
       </c>
       <c r="K13" t="n">
-        <v>801.3997324917706</v>
+        <v>591.2014890658488</v>
       </c>
       <c r="L13" t="n">
-        <v>12234.27</v>
+        <v>5457.83</v>
       </c>
       <c r="M13" t="n">
-        <v>-554.61</v>
+        <v>-184.59</v>
       </c>
     </row>
     <row r="14">
@@ -1059,22 +1059,22 @@
         <v>8000</v>
       </c>
       <c r="H14" t="n">
-        <v>-750</v>
+        <v>-260</v>
       </c>
       <c r="I14" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="J14" t="n">
         <v>0.5</v>
       </c>
       <c r="K14" t="n">
-        <v>532.9018207393951</v>
+        <v>616.5242336945269</v>
       </c>
       <c r="L14" t="n">
-        <v>6197.48</v>
+        <v>6504.31</v>
       </c>
       <c r="M14" t="n">
-        <v>-567.14</v>
+        <v>-206.03</v>
       </c>
     </row>
     <row r="15">
@@ -1101,25 +1101,25 @@
         <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>1400</v>
+        <v>1000</v>
       </c>
       <c r="H15" t="n">
-        <v>-60</v>
+        <v>-260</v>
       </c>
       <c r="I15" t="n">
-        <v>550</v>
+        <v>250</v>
       </c>
       <c r="J15" t="n">
         <v>0.5</v>
       </c>
       <c r="K15" t="n">
-        <v>511.9955082862131</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L15" t="n">
-        <v>1191.94</v>
+        <v>690.4400000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>-45.79</v>
+        <v>-166.85</v>
       </c>
     </row>
     <row r="16">
@@ -1146,13 +1146,13 @@
         <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="H16" t="n">
-        <v>-700</v>
+        <v>-950</v>
       </c>
       <c r="I16" t="n">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="J16" t="n">
         <v>0.5</v>
@@ -1161,10 +1161,10 @@
         <v>302.9006275609877</v>
       </c>
       <c r="L16" t="n">
-        <v>728.99</v>
+        <v>2780.83</v>
       </c>
       <c r="M16" t="n">
-        <v>-455.73</v>
+        <v>-626.96</v>
       </c>
     </row>
     <row r="17">
@@ -1191,25 +1191,25 @@
         <v>6</v>
       </c>
       <c r="G17" t="n">
-        <v>1900</v>
+        <v>800</v>
       </c>
       <c r="H17" t="n">
         <v>-160</v>
       </c>
       <c r="I17" t="n">
-        <v>290</v>
+        <v>350</v>
       </c>
       <c r="J17" t="n">
         <v>0.5</v>
       </c>
       <c r="K17" t="n">
-        <v>280.4314892296821</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L17" t="n">
-        <v>1334.83</v>
+        <v>614.03</v>
       </c>
       <c r="M17" t="n">
-        <v>-88.59</v>
+        <v>-63.87</v>
       </c>
     </row>
     <row r="18">
@@ -1236,25 +1236,25 @@
         <v>7</v>
       </c>
       <c r="G18" t="n">
-        <v>2900</v>
+        <v>3000</v>
       </c>
       <c r="H18" t="n">
-        <v>-110</v>
+        <v>-900</v>
       </c>
       <c r="I18" t="n">
-        <v>700</v>
+        <v>290</v>
       </c>
       <c r="J18" t="n">
         <v>0.5</v>
       </c>
       <c r="K18" t="n">
-        <v>721.0477175625025</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L18" t="n">
-        <v>2435.11</v>
+        <v>1998.15</v>
       </c>
       <c r="M18" t="n">
-        <v>-76.88</v>
+        <v>-565.5</v>
       </c>
     </row>
     <row r="19">
@@ -1281,25 +1281,25 @@
         <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>17000</v>
+        <v>700</v>
       </c>
       <c r="H19" t="n">
-        <v>-800</v>
+        <v>-260</v>
       </c>
       <c r="I19" t="n">
-        <v>750</v>
+        <v>90</v>
       </c>
       <c r="J19" t="n">
         <v>0.5</v>
       </c>
       <c r="K19" t="n">
-        <v>787.6525764547314</v>
+        <v>114.4856760702529</v>
       </c>
       <c r="L19" t="n">
-        <v>14349.02</v>
+        <v>324.32</v>
       </c>
       <c r="M19" t="n">
-        <v>-663.39</v>
+        <v>92.84</v>
       </c>
     </row>
     <row r="20">
@@ -1326,25 +1326,25 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>14001.77852921273</v>
+        <v>11000.24611493832</v>
       </c>
       <c r="H20" t="n">
-        <v>-69.99999199863345</v>
+        <v>-100.0005642535693</v>
       </c>
       <c r="I20" t="n">
-        <v>99.83889423976993</v>
+        <v>250.9018119795456</v>
       </c>
       <c r="J20" t="n">
         <v>0.5</v>
       </c>
       <c r="K20" t="n">
-        <v>147.8003722664622</v>
+        <v>295.6007445329244</v>
       </c>
       <c r="L20" t="n">
-        <v>2930.37</v>
+        <v>6377.43</v>
       </c>
       <c r="M20" t="n">
-        <v>183.03</v>
+        <v>-19.37</v>
       </c>
     </row>
     <row r="21">
@@ -1371,25 +1371,25 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>1310.154300581582</v>
+        <v>1016.427042744672</v>
       </c>
       <c r="H21" t="n">
-        <v>-650.0000096439097</v>
+        <v>-350.0000195817747</v>
       </c>
       <c r="I21" t="n">
-        <v>550.426048659099</v>
+        <v>500.2842266235539</v>
       </c>
       <c r="J21" t="n">
         <v>0.5</v>
       </c>
       <c r="K21" t="n">
-        <v>472.0365350579011</v>
+        <v>499.0314924731653</v>
       </c>
       <c r="L21" t="n">
-        <v>1062.68</v>
+        <v>805.65</v>
       </c>
       <c r="M21" t="n">
-        <v>-521.46</v>
+        <v>-272.91</v>
       </c>
     </row>
     <row r="22">
@@ -1416,25 +1416,25 @@
         <v>2</v>
       </c>
       <c r="G22" t="n">
-        <v>14000.35243258604</v>
+        <v>6000.695184318414</v>
       </c>
       <c r="H22" t="n">
-        <v>-600.0000186326773</v>
+        <v>-250.0000061576394</v>
       </c>
       <c r="I22" t="n">
-        <v>650.382056893912</v>
+        <v>450.3520558660788</v>
       </c>
       <c r="J22" t="n">
         <v>0.5</v>
       </c>
       <c r="K22" t="n">
-        <v>686.9140564215176</v>
+        <v>423.2358566393677</v>
       </c>
       <c r="L22" t="n">
-        <v>11463.82</v>
+        <v>4711.47</v>
       </c>
       <c r="M22" t="n">
-        <v>-478.76</v>
+        <v>-177.96</v>
       </c>
     </row>
     <row r="23">
@@ -1461,25 +1461,25 @@
         <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>7001.052145694428</v>
+        <v>7000.569707888595</v>
       </c>
       <c r="H23" t="n">
-        <v>-650.0000143552476</v>
+        <v>-250.0000067117505</v>
       </c>
       <c r="I23" t="n">
-        <v>400.8530474728325</v>
+        <v>500.2940864750864</v>
       </c>
       <c r="J23" t="n">
         <v>0.5</v>
       </c>
       <c r="K23" t="n">
-        <v>428.3661755480705</v>
+        <v>528.7866871801347</v>
       </c>
       <c r="L23" t="n">
-        <v>4783.6</v>
+        <v>5442.55</v>
       </c>
       <c r="M23" t="n">
-        <v>-407.92</v>
+        <v>-180.77</v>
       </c>
     </row>
     <row r="24">
@@ -1506,25 +1506,25 @@
         <v>4</v>
       </c>
       <c r="G24" t="n">
-        <v>1301.005694904366</v>
+        <v>934.1355194678936</v>
       </c>
       <c r="H24" t="n">
-        <v>-66.41361308858089</v>
+        <v>-250.0000035952838</v>
       </c>
       <c r="I24" t="n">
-        <v>450.0447150940522</v>
+        <v>153.7076527310146</v>
       </c>
       <c r="J24" t="n">
         <v>0.5</v>
       </c>
       <c r="K24" t="n">
-        <v>423.2358566393677</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L24" t="n">
-        <v>1043.96</v>
+        <v>355.85</v>
       </c>
       <c r="M24" t="n">
-        <v>-59.69</v>
+        <v>-14.85</v>
       </c>
     </row>
     <row r="25">
@@ -1551,25 +1551,25 @@
         <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>953.2875846635555</v>
+        <v>3004.79069136813</v>
       </c>
       <c r="H25" t="n">
-        <v>-600.0000114576097</v>
+        <v>-850.0000098407239</v>
       </c>
       <c r="I25" t="n">
-        <v>205.4458625081447</v>
+        <v>288.2732712363093</v>
       </c>
       <c r="J25" t="n">
         <v>0.5</v>
       </c>
       <c r="K25" t="n">
-        <v>186.9543261531214</v>
+        <v>302.9006275609877</v>
       </c>
       <c r="L25" t="n">
-        <v>611.8200000000001</v>
+        <v>2027.2</v>
       </c>
       <c r="M25" t="n">
-        <v>-303.06</v>
+        <v>-524.95</v>
       </c>
     </row>
     <row r="26">
@@ -1596,25 +1596,25 @@
         <v>6</v>
       </c>
       <c r="G26" t="n">
-        <v>1800.804604707089</v>
+        <v>793.1152257303916</v>
       </c>
       <c r="H26" t="n">
-        <v>-150.0000270242403</v>
+        <v>-150.0000075316569</v>
       </c>
       <c r="I26" t="n">
-        <v>280.7608868442319</v>
+        <v>250.5675852492012</v>
       </c>
       <c r="J26" t="n">
         <v>0.5</v>
       </c>
       <c r="K26" t="n">
-        <v>264.3933435900673</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L26" t="n">
-        <v>1338.59</v>
+        <v>619.08</v>
       </c>
       <c r="M26" t="n">
-        <v>-74.62</v>
+        <v>-63.58</v>
       </c>
     </row>
     <row r="27">
@@ -1641,25 +1641,25 @@
         <v>7</v>
       </c>
       <c r="G27" t="n">
-        <v>2800.266111677523</v>
+        <v>2008.387671907359</v>
       </c>
       <c r="H27" t="n">
-        <v>-100.0000258654949</v>
+        <v>-800.00001112285</v>
       </c>
       <c r="I27" t="n">
-        <v>600.0786424741285</v>
+        <v>284.0777599761669</v>
       </c>
       <c r="J27" t="n">
         <v>0.5</v>
       </c>
       <c r="K27" t="n">
-        <v>602.1844988862963</v>
+        <v>295.6007445329244</v>
       </c>
       <c r="L27" t="n">
-        <v>2358.24</v>
+        <v>1345.29</v>
       </c>
       <c r="M27" t="n">
-        <v>-68.84</v>
+        <v>-475.64</v>
       </c>
     </row>
     <row r="28">
@@ -1686,25 +1686,25 @@
         <v>8</v>
       </c>
       <c r="G28" t="n">
-        <v>16000.31879978021</v>
+        <v>795.7634281047748</v>
       </c>
       <c r="H28" t="n">
-        <v>-700.0000161074539</v>
+        <v>-269.9999930087224</v>
       </c>
       <c r="I28" t="n">
-        <v>650.3989698248582</v>
+        <v>99.94062908745198</v>
       </c>
       <c r="J28" t="n">
         <v>0.5</v>
       </c>
       <c r="K28" t="n">
-        <v>702.6349485697167</v>
+        <v>114.4856760702529</v>
       </c>
       <c r="L28" t="n">
-        <v>12844.9</v>
+        <v>199.01</v>
       </c>
       <c r="M28" t="n">
-        <v>-544.24</v>
+        <v>120.67</v>
       </c>
     </row>
     <row r="29">
@@ -1731,25 +1731,25 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>13046.96148023747</v>
+        <v>10019.82426360569</v>
       </c>
       <c r="H29" t="n">
-        <v>-79.6402725068038</v>
+        <v>-89.70569086990514</v>
       </c>
       <c r="I29" t="n">
-        <v>109.9954851352551</v>
+        <v>171.1494795877462</v>
       </c>
       <c r="J29" t="n">
         <v>0.5</v>
       </c>
       <c r="K29" t="n">
-        <v>147.8003722664622</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L29" t="n">
-        <v>3148.88</v>
+        <v>4347.36</v>
       </c>
       <c r="M29" t="n">
-        <v>17.84</v>
+        <v>36.58</v>
       </c>
     </row>
     <row r="30">
@@ -1776,25 +1776,25 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>1225.68608921074</v>
+        <v>953.5289157604102</v>
       </c>
       <c r="H30" t="n">
-        <v>-547.6514396085951</v>
+        <v>-247.0985614126917</v>
       </c>
       <c r="I30" t="n">
-        <v>462.6325435628922</v>
+        <v>410.0908232346522</v>
       </c>
       <c r="J30" t="n">
         <v>0.5</v>
       </c>
       <c r="K30" t="n">
-        <v>443.4011167993866</v>
+        <v>402.0604809124811</v>
       </c>
       <c r="L30" t="n">
-        <v>1017.71</v>
+        <v>729.96</v>
       </c>
       <c r="M30" t="n">
-        <v>-439.11</v>
+        <v>-174.92</v>
       </c>
     </row>
     <row r="31">
@@ -1821,25 +1821,25 @@
         <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>13032.25511269434</v>
+        <v>5042.846115763668</v>
       </c>
       <c r="H31" t="n">
-        <v>-498.0287210202926</v>
+        <v>-239.9741289934778</v>
       </c>
       <c r="I31" t="n">
-        <v>553.8675308112345</v>
+        <v>355.0518595457356</v>
       </c>
       <c r="J31" t="n">
         <v>0.5</v>
       </c>
       <c r="K31" t="n">
-        <v>591.2014890658488</v>
+        <v>391.0430286998269</v>
       </c>
       <c r="L31" t="n">
-        <v>10044.43</v>
+        <v>3420.61</v>
       </c>
       <c r="M31" t="n">
-        <v>-363.92</v>
+        <v>-129.5</v>
       </c>
     </row>
     <row r="32">
@@ -1866,25 +1866,25 @@
         <v>3</v>
       </c>
       <c r="G32" t="n">
-        <v>6057.31548080692</v>
+        <v>6035.967780342778</v>
       </c>
       <c r="H32" t="n">
-        <v>-547.8748569533839</v>
+        <v>-239.7645093774938</v>
       </c>
       <c r="I32" t="n">
-        <v>311.047839387307</v>
+        <v>407.569218160852</v>
       </c>
       <c r="J32" t="n">
         <v>0.5</v>
       </c>
       <c r="K32" t="n">
-        <v>337.0367045574487</v>
+        <v>438.4467588778851</v>
       </c>
       <c r="L32" t="n">
-        <v>4085.63</v>
+        <v>4375.47</v>
       </c>
       <c r="M32" t="n">
-        <v>-338.29</v>
+        <v>-148.24</v>
       </c>
     </row>
     <row r="33">
@@ -1911,25 +1911,25 @@
         <v>4</v>
       </c>
       <c r="G33" t="n">
-        <v>1209.042552352751</v>
+        <v>934.5287930215312</v>
       </c>
       <c r="H33" t="n">
-        <v>-55.73898185861684</v>
+        <v>-239.9439386170428</v>
       </c>
       <c r="I33" t="n">
-        <v>368.4870223911405</v>
+        <v>146.2890460803963</v>
       </c>
       <c r="J33" t="n">
         <v>0.5</v>
       </c>
       <c r="K33" t="n">
-        <v>355.9504322854629</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L33" t="n">
-        <v>904.98</v>
+        <v>429.07</v>
       </c>
       <c r="M33" t="n">
-        <v>-29.34</v>
+        <v>-12.84</v>
       </c>
     </row>
     <row r="34">
@@ -1956,25 +1956,25 @@
         <v>5</v>
       </c>
       <c r="G34" t="n">
-        <v>941.3514482732445</v>
+        <v>2120.334010643724</v>
       </c>
       <c r="H34" t="n">
-        <v>-499.9047126525462</v>
+        <v>-748.8594242394379</v>
       </c>
       <c r="I34" t="n">
-        <v>155.2998775422665</v>
+        <v>284.2112679143011</v>
       </c>
       <c r="J34" t="n">
         <v>0.5</v>
       </c>
       <c r="K34" t="n">
-        <v>174.8797588600428</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L34" t="n">
-        <v>374.75</v>
+        <v>1505.85</v>
       </c>
       <c r="M34" t="n">
-        <v>-100.91</v>
+        <v>-482.17</v>
       </c>
     </row>
     <row r="35">
@@ -2001,25 +2001,25 @@
         <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>1710.367743176406</v>
+        <v>867.9326628634178</v>
       </c>
       <c r="H35" t="n">
-        <v>-139.0746289883452</v>
+        <v>-140.8427279988577</v>
       </c>
       <c r="I35" t="n">
-        <v>277.9596951593777</v>
+        <v>172.3298031798057</v>
       </c>
       <c r="J35" t="n">
         <v>0.5</v>
       </c>
       <c r="K35" t="n">
-        <v>288.1159665134826</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L35" t="n">
-        <v>1138.88</v>
+        <v>504.74</v>
       </c>
       <c r="M35" t="n">
-        <v>-67.05</v>
+        <v>-13.52</v>
       </c>
     </row>
     <row r="36">
@@ -2046,25 +2046,25 @@
         <v>7</v>
       </c>
       <c r="G36" t="n">
-        <v>2702.494429589704</v>
+        <v>1170.369572934555</v>
       </c>
       <c r="H36" t="n">
-        <v>-89.82350350259199</v>
+        <v>-698.3270805670745</v>
       </c>
       <c r="I36" t="n">
-        <v>503.8268420044408</v>
+        <v>281.3259291081103</v>
       </c>
       <c r="J36" t="n">
         <v>0.5</v>
       </c>
       <c r="K36" t="n">
-        <v>532.9018207393951</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L36" t="n">
-        <v>2117.78</v>
+        <v>870.1900000000001</v>
       </c>
       <c r="M36" t="n">
-        <v>-53.02</v>
+        <v>-556.22</v>
       </c>
     </row>
     <row r="37">
@@ -2091,25 +2091,25 @@
         <v>8</v>
       </c>
       <c r="G37" t="n">
-        <v>15023.11868049572</v>
+        <v>888.4677843863684</v>
       </c>
       <c r="H37" t="n">
-        <v>-597.4204471109011</v>
+        <v>-280.3324893698352</v>
       </c>
       <c r="I37" t="n">
-        <v>556.5192155775079</v>
+        <v>109.6234332991881</v>
       </c>
       <c r="J37" t="n">
         <v>0.5</v>
       </c>
       <c r="K37" t="n">
-        <v>499.0314924731653</v>
+        <v>132.1966717950337</v>
       </c>
       <c r="L37" t="n">
-        <v>12440.53</v>
+        <v>313.06</v>
       </c>
       <c r="M37" t="n">
-        <v>-481.28</v>
+        <v>36.12</v>
       </c>
     </row>
     <row r="38">
@@ -2136,13 +2136,13 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>12157.71600259174</v>
+        <v>9068.088507249551</v>
       </c>
       <c r="H38" t="n">
-        <v>-91.03429994640456</v>
+        <v>-87.38265579801036</v>
       </c>
       <c r="I38" t="n">
-        <v>119.0525508970402</v>
+        <v>128.6624508135351</v>
       </c>
       <c r="J38" t="n">
         <v>0.5</v>
@@ -2151,10 +2151,10 @@
         <v>198.2950076925505</v>
       </c>
       <c r="L38" t="n">
-        <v>3359.54</v>
+        <v>2721.47</v>
       </c>
       <c r="M38" t="n">
-        <v>51.83</v>
+        <v>88.38</v>
       </c>
     </row>
     <row r="39">
@@ -2181,25 +2181,25 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>1151.748523211517</v>
+        <v>909.6598516727203</v>
       </c>
       <c r="H39" t="n">
-        <v>-450.435630989574</v>
+        <v>-150.4129766062561</v>
       </c>
       <c r="I39" t="n">
-        <v>386.5974240265782</v>
+        <v>325.2903109865437</v>
       </c>
       <c r="J39" t="n">
         <v>0.5</v>
       </c>
       <c r="K39" t="n">
-        <v>373.9086523062428</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L39" t="n">
-        <v>889.39</v>
+        <v>675.28</v>
       </c>
       <c r="M39" t="n">
-        <v>-337.8</v>
+        <v>-104.72</v>
       </c>
     </row>
     <row r="40">
@@ -2226,25 +2226,25 @@
         <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>12059.60463998207</v>
+        <v>4112.887503526152</v>
       </c>
       <c r="H40" t="n">
-        <v>-399.6250655386197</v>
+        <v>-229.8661081454598</v>
       </c>
       <c r="I40" t="n">
-        <v>463.269304455952</v>
+        <v>283.1351769500222</v>
       </c>
       <c r="J40" t="n">
         <v>0.5</v>
       </c>
       <c r="K40" t="n">
-        <v>503.3899288706676</v>
+        <v>310.0286763918156</v>
       </c>
       <c r="L40" t="n">
-        <v>9146.33</v>
+        <v>2651.07</v>
       </c>
       <c r="M40" t="n">
-        <v>-276.75</v>
+        <v>-103.65</v>
       </c>
     </row>
     <row r="41">
@@ -2271,25 +2271,25 @@
         <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>5148.592042699991</v>
+        <v>5103.339338548314</v>
       </c>
       <c r="H41" t="n">
-        <v>-452.2891667264399</v>
+        <v>-229.7773332640361</v>
       </c>
       <c r="I41" t="n">
-        <v>232.7159793568155</v>
+        <v>321.1270759877012</v>
       </c>
       <c r="J41" t="n">
         <v>0.5</v>
       </c>
       <c r="K41" t="n">
-        <v>255.9977541431066</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L41" t="n">
-        <v>3070.31</v>
+        <v>3378.23</v>
       </c>
       <c r="M41" t="n">
-        <v>-228.29</v>
+        <v>-120.37</v>
       </c>
     </row>
     <row r="42">
@@ -2316,25 +2316,25 @@
         <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>1130.299444159703</v>
+        <v>1045.077130470538</v>
       </c>
       <c r="H42" t="n">
-        <v>-44.17968695509059</v>
+        <v>-237.2222750013117</v>
       </c>
       <c r="I42" t="n">
-        <v>301.6671373490805</v>
+        <v>254.4156288584925</v>
       </c>
       <c r="J42" t="n">
         <v>0.5</v>
       </c>
       <c r="K42" t="n">
-        <v>295.6007445329244</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L42" t="n">
-        <v>825.42</v>
+        <v>742.4</v>
       </c>
       <c r="M42" t="n">
-        <v>-1.91</v>
+        <v>-147.49</v>
       </c>
     </row>
     <row r="43">
@@ -2361,25 +2361,25 @@
         <v>5</v>
       </c>
       <c r="G43" t="n">
-        <v>973.6358608025605</v>
+        <v>1344.16804998633</v>
       </c>
       <c r="H43" t="n">
-        <v>-407.9523685995779</v>
+        <v>-650.7693533218935</v>
       </c>
       <c r="I43" t="n">
-        <v>222.4545536729751</v>
+        <v>279.5493252616245</v>
       </c>
       <c r="J43" t="n">
         <v>0.5</v>
       </c>
       <c r="K43" t="n">
-        <v>186.9543261531214</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L43" t="n">
-        <v>664.16</v>
+        <v>948.04</v>
       </c>
       <c r="M43" t="n">
-        <v>-234.04</v>
+        <v>-423.12</v>
       </c>
     </row>
     <row r="44">
@@ -2406,25 +2406,25 @@
         <v>6</v>
       </c>
       <c r="G44" t="n">
-        <v>1615.421225981708</v>
+        <v>946.61255177524</v>
       </c>
       <c r="H44" t="n">
-        <v>-128.9112897928376</v>
+        <v>-131.5271401200158</v>
       </c>
       <c r="I44" t="n">
-        <v>280.8506807929207</v>
+        <v>190.2605223021965</v>
       </c>
       <c r="J44" t="n">
         <v>0.5</v>
       </c>
       <c r="K44" t="n">
-        <v>280.4314892296821</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L44" t="n">
-        <v>1142.16</v>
+        <v>567.14</v>
       </c>
       <c r="M44" t="n">
-        <v>-54.18</v>
+        <v>-10.63</v>
       </c>
     </row>
     <row r="45">
@@ -2451,25 +2451,25 @@
         <v>7</v>
       </c>
       <c r="G45" t="n">
-        <v>2603.303689510175</v>
+        <v>517.1803651784227</v>
       </c>
       <c r="H45" t="n">
-        <v>-79.9676996839266</v>
+        <v>-599.6858269481017</v>
       </c>
       <c r="I45" t="n">
-        <v>415.2910762703204</v>
+        <v>277.6808138882571</v>
       </c>
       <c r="J45" t="n">
         <v>0.5</v>
       </c>
       <c r="K45" t="n">
-        <v>423.2358566393677</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L45" t="n">
-        <v>2016.66</v>
+        <v>323.57</v>
       </c>
       <c r="M45" t="n">
-        <v>-29.86</v>
+        <v>-390.07</v>
       </c>
     </row>
     <row r="46">
@@ -2496,25 +2496,25 @@
         <v>8</v>
       </c>
       <c r="G46" t="n">
-        <v>14051.78181473025</v>
+        <v>987.5133176613283</v>
       </c>
       <c r="H46" t="n">
-        <v>-499.5528525781684</v>
+        <v>-290.9401813229373</v>
       </c>
       <c r="I46" t="n">
-        <v>465.0331521314256</v>
+        <v>119.0006345413076</v>
       </c>
       <c r="J46" t="n">
         <v>0.5</v>
       </c>
       <c r="K46" t="n">
-        <v>503.3899288706676</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L46" t="n">
-        <v>10609.8</v>
+        <v>346.26</v>
       </c>
       <c r="M46" t="n">
-        <v>-354.3</v>
+        <v>-2.41</v>
       </c>
     </row>
     <row r="47">
@@ -2541,25 +2541,25 @@
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>11062.35219511693</v>
+        <v>8275.262935590812</v>
       </c>
       <c r="H47" t="n">
-        <v>-97.85995401436402</v>
+        <v>-98.90608281167626</v>
       </c>
       <c r="I47" t="n">
-        <v>129.7669178687061</v>
+        <v>150.0726628380948</v>
       </c>
       <c r="J47" t="n">
         <v>0.5</v>
       </c>
       <c r="K47" t="n">
-        <v>198.2950076925505</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L47" t="n">
-        <v>3406.75</v>
+        <v>3209.83</v>
       </c>
       <c r="M47" t="n">
-        <v>87.73</v>
+        <v>37.63</v>
       </c>
     </row>
     <row r="48">
@@ -2586,25 +2586,25 @@
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>1080.220775636587</v>
+        <v>889.7899109195167</v>
       </c>
       <c r="H48" t="n">
-        <v>-356.4689200906026</v>
+        <v>-62.63608059820302</v>
       </c>
       <c r="I48" t="n">
-        <v>312.4226597556309</v>
+        <v>251.1701036267572</v>
       </c>
       <c r="J48" t="n">
         <v>0.5</v>
       </c>
       <c r="K48" t="n">
-        <v>288.1159665134826</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L48" t="n">
-        <v>780.09</v>
+        <v>610.89</v>
       </c>
       <c r="M48" t="n">
-        <v>-249.87</v>
+        <v>-0.54</v>
       </c>
     </row>
     <row r="49">
@@ -2631,25 +2631,25 @@
         <v>2</v>
       </c>
       <c r="G49" t="n">
-        <v>11093.00372454842</v>
+        <v>3252.35047987053</v>
       </c>
       <c r="H49" t="n">
-        <v>-307.8451620964086</v>
+        <v>-220.4818283299811</v>
       </c>
       <c r="I49" t="n">
-        <v>377.7097208463673</v>
+        <v>214.1966351666642</v>
       </c>
       <c r="J49" t="n">
         <v>0.5</v>
       </c>
       <c r="K49" t="n">
-        <v>412.7839753774575</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L49" t="n">
-        <v>8021.33</v>
+        <v>1860.23</v>
       </c>
       <c r="M49" t="n">
-        <v>-195.07</v>
+        <v>-62.09</v>
       </c>
     </row>
     <row r="50">
@@ -2676,25 +2676,25 @@
         <v>3</v>
       </c>
       <c r="G50" t="n">
-        <v>4262.062593572969</v>
+        <v>4212.61909377913</v>
       </c>
       <c r="H50" t="n">
-        <v>-359.9502941912115</v>
+        <v>-220.1900154543873</v>
       </c>
       <c r="I50" t="n">
-        <v>178.1105325099239</v>
+        <v>245.3897146254757</v>
       </c>
       <c r="J50" t="n">
         <v>0.5</v>
       </c>
       <c r="K50" t="n">
-        <v>209.0212909830231</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L50" t="n">
-        <v>2066.8</v>
+        <v>2558.62</v>
       </c>
       <c r="M50" t="n">
-        <v>-97.02</v>
+        <v>-64.16</v>
       </c>
     </row>
     <row r="51">
@@ -2721,25 +2721,25 @@
         <v>4</v>
       </c>
       <c r="G51" t="n">
-        <v>1051.477175150365</v>
+        <v>1145.496357208988</v>
       </c>
       <c r="H51" t="n">
-        <v>-36.66069417959777</v>
+        <v>-236.5186037258011</v>
       </c>
       <c r="I51" t="n">
-        <v>237.2892518259536</v>
+        <v>369.5862066727457</v>
       </c>
       <c r="J51" t="n">
         <v>0.5</v>
       </c>
       <c r="K51" t="n">
-        <v>219.2233794389425</v>
+        <v>355.9504322854629</v>
       </c>
       <c r="L51" t="n">
-        <v>754.51</v>
+        <v>932.13</v>
       </c>
       <c r="M51" t="n">
-        <v>26.21</v>
+        <v>-199.11</v>
       </c>
     </row>
     <row r="52">
@@ -2766,25 +2766,25 @@
         <v>5</v>
       </c>
       <c r="G52" t="n">
-        <v>1082.535800751018</v>
+        <v>706.0876296532565</v>
       </c>
       <c r="H52" t="n">
-        <v>-339.8372708751267</v>
+        <v>-553.6521296825508</v>
       </c>
       <c r="I52" t="n">
-        <v>332.3615686700963</v>
+        <v>278.1046755440734</v>
       </c>
       <c r="J52" t="n">
         <v>0.5</v>
       </c>
       <c r="K52" t="n">
-        <v>288.1159665134826</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L52" t="n">
-        <v>831.49</v>
+        <v>529.98</v>
       </c>
       <c r="M52" t="n">
-        <v>-259.78</v>
+        <v>-380.63</v>
       </c>
     </row>
     <row r="53">
@@ -2811,25 +2811,25 @@
         <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>1530.627057091059</v>
+        <v>1066.357014912186</v>
       </c>
       <c r="H53" t="n">
-        <v>-118.9626789158286</v>
+        <v>-129.8722072943</v>
       </c>
       <c r="I53" t="n">
-        <v>278.6408443395536</v>
+        <v>286.0426223487677</v>
       </c>
       <c r="J53" t="n">
         <v>0.5</v>
       </c>
       <c r="K53" t="n">
-        <v>288.1159665134826</v>
+        <v>295.6007445329244</v>
       </c>
       <c r="L53" t="n">
-        <v>1031.05</v>
+        <v>799.84</v>
       </c>
       <c r="M53" t="n">
-        <v>-36.6</v>
+        <v>-62.83</v>
       </c>
     </row>
     <row r="54">
@@ -2856,25 +2856,25 @@
         <v>7</v>
       </c>
       <c r="G54" t="n">
-        <v>2504.954258586067</v>
+        <v>140.4685856305885</v>
       </c>
       <c r="H54" t="n">
-        <v>-71.14259769750032</v>
+        <v>-497.2496235670113</v>
       </c>
       <c r="I54" t="n">
-        <v>329.923315526312</v>
+        <v>282.4959182897016</v>
       </c>
       <c r="J54" t="n">
         <v>0.5</v>
       </c>
       <c r="K54" t="n">
-        <v>330.4916794875841</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L54" t="n">
-        <v>1789.14</v>
+        <v>-11.56</v>
       </c>
       <c r="M54" t="n">
-        <v>-32.56</v>
+        <v>-249.14</v>
       </c>
     </row>
     <row r="55">
@@ -2901,25 +2901,25 @@
         <v>8</v>
       </c>
       <c r="G55" t="n">
-        <v>13068.86876026682</v>
+        <v>1091.173715816988</v>
       </c>
       <c r="H55" t="n">
-        <v>-404.4518066335505</v>
+        <v>-299.4193221051651</v>
       </c>
       <c r="I55" t="n">
-        <v>393.9962950688081</v>
+        <v>129.4424306133734</v>
       </c>
       <c r="J55" t="n">
         <v>0.5</v>
       </c>
       <c r="K55" t="n">
-        <v>418.0425819660462</v>
+        <v>132.1966717950337</v>
       </c>
       <c r="L55" t="n">
-        <v>9610.18</v>
+        <v>468.97</v>
       </c>
       <c r="M55" t="n">
-        <v>-261.78</v>
+        <v>5.84</v>
       </c>
     </row>
     <row r="56">
@@ -2946,25 +2946,25 @@
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>9996.390145223857</v>
+        <v>7672.185487234441</v>
       </c>
       <c r="H56" t="n">
-        <v>-105.9514926791</v>
+        <v>-112.0513232451717</v>
       </c>
       <c r="I56" t="n">
-        <v>137.9681270943666</v>
+        <v>205.1572339388355</v>
       </c>
       <c r="J56" t="n">
         <v>0.5</v>
       </c>
       <c r="K56" t="n">
-        <v>198.2950076925505</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L56" t="n">
-        <v>4931.19</v>
+        <v>4140.24</v>
       </c>
       <c r="M56" t="n">
-        <v>22.97</v>
+        <v>-23.2</v>
       </c>
     </row>
     <row r="57">
@@ -2991,25 +2991,25 @@
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>1022.722065201188</v>
+        <v>903.6528017560341</v>
       </c>
       <c r="H57" t="n">
-        <v>-267.4711429832689</v>
+        <v>14.09442104164692</v>
       </c>
       <c r="I57" t="n">
-        <v>250.4409275158184</v>
+        <v>197.178743454091</v>
       </c>
       <c r="J57" t="n">
         <v>0.5</v>
       </c>
       <c r="K57" t="n">
-        <v>238.320939301339</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L57" t="n">
-        <v>632.09</v>
+        <v>577.04</v>
       </c>
       <c r="M57" t="n">
-        <v>-137</v>
+        <v>79.48</v>
       </c>
     </row>
     <row r="58">
@@ -3036,25 +3036,25 @@
         <v>2</v>
       </c>
       <c r="G58" t="n">
-        <v>10121.10607008271</v>
+        <v>2451.639729619361</v>
       </c>
       <c r="H58" t="n">
-        <v>-223.2198127021985</v>
+        <v>-211.5188557968147</v>
       </c>
       <c r="I58" t="n">
-        <v>300.0645920555126</v>
+        <v>170.8123143410118</v>
       </c>
       <c r="J58" t="n">
         <v>0.5</v>
       </c>
       <c r="K58" t="n">
-        <v>337.0367045574487</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L58" t="n">
-        <v>6513.56</v>
+        <v>1236.32</v>
       </c>
       <c r="M58" t="n">
-        <v>-94.44</v>
+        <v>-53.41</v>
       </c>
     </row>
     <row r="59">
@@ -3081,25 +3081,25 @@
         <v>3</v>
       </c>
       <c r="G59" t="n">
-        <v>3426.43879921457</v>
+        <v>3379.778180654522</v>
       </c>
       <c r="H59" t="n">
-        <v>-275.7743828486982</v>
+        <v>-210.9705804227473</v>
       </c>
       <c r="I59" t="n">
-        <v>164.2584156044719</v>
+        <v>193.1771767187937</v>
       </c>
       <c r="J59" t="n">
         <v>0.5</v>
       </c>
       <c r="K59" t="n">
-        <v>209.0212909830231</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L59" t="n">
-        <v>1470.49</v>
+        <v>1767.63</v>
       </c>
       <c r="M59" t="n">
-        <v>-41.93</v>
+        <v>-12.32</v>
       </c>
     </row>
     <row r="60">
@@ -3126,25 +3126,25 @@
         <v>4</v>
       </c>
       <c r="G60" t="n">
-        <v>993.3631107615867</v>
+        <v>1178.919403638545</v>
       </c>
       <c r="H60" t="n">
-        <v>-41.72220254210079</v>
+        <v>-227.5048711783242</v>
       </c>
       <c r="I60" t="n">
-        <v>201.9241925846892</v>
+        <v>429.2799221375635</v>
       </c>
       <c r="J60" t="n">
         <v>0.5</v>
       </c>
       <c r="K60" t="n">
-        <v>174.8797588600428</v>
+        <v>433.4357742066306</v>
       </c>
       <c r="L60" t="n">
-        <v>694.13</v>
+        <v>916.49</v>
       </c>
       <c r="M60" t="n">
-        <v>18.3</v>
+        <v>-150.57</v>
       </c>
     </row>
     <row r="61">
@@ -3171,25 +3171,25 @@
         <v>5</v>
       </c>
       <c r="G61" t="n">
-        <v>1124.813799302195</v>
+        <v>305.3579217559828</v>
       </c>
       <c r="H61" t="n">
-        <v>-252.995658034761</v>
+        <v>-458.4223422990248</v>
       </c>
       <c r="I61" t="n">
-        <v>420.782424249975</v>
+        <v>277.2730719852731</v>
       </c>
       <c r="J61" t="n">
         <v>0.5</v>
       </c>
       <c r="K61" t="n">
-        <v>396.590015385101</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L61" t="n">
-        <v>873.2</v>
+        <v>256.47</v>
       </c>
       <c r="M61" t="n">
-        <v>-189.46</v>
+        <v>-90.81</v>
       </c>
     </row>
     <row r="62">
@@ -3216,25 +3216,25 @@
         <v>6</v>
       </c>
       <c r="G62" t="n">
-        <v>1439.839316828994</v>
+        <v>1167.892093084745</v>
       </c>
       <c r="H62" t="n">
-        <v>-109.8471544405085</v>
+        <v>-131.024156688997</v>
       </c>
       <c r="I62" t="n">
-        <v>278.1746967412088</v>
+        <v>384.6150950665786</v>
       </c>
       <c r="J62" t="n">
         <v>0.5</v>
       </c>
       <c r="K62" t="n">
-        <v>255.9977541431066</v>
+        <v>373.9086523062428</v>
       </c>
       <c r="L62" t="n">
-        <v>1040.09</v>
+        <v>918.1900000000001</v>
       </c>
       <c r="M62" t="n">
-        <v>-47.53</v>
+        <v>-80.11</v>
       </c>
     </row>
     <row r="63">
@@ -3261,25 +3261,25 @@
         <v>7</v>
       </c>
       <c r="G63" t="n">
-        <v>2399.768567013934</v>
+        <v>227.8853739932531</v>
       </c>
       <c r="H63" t="n">
-        <v>-65.49094404203781</v>
+        <v>-403.2675097024474</v>
       </c>
       <c r="I63" t="n">
-        <v>255.9470890103535</v>
+        <v>290.4456456590701</v>
       </c>
       <c r="J63" t="n">
         <v>0.5</v>
       </c>
       <c r="K63" t="n">
-        <v>280.4314892296821</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L63" t="n">
-        <v>1498.9</v>
+        <v>-64.76000000000001</v>
       </c>
       <c r="M63" t="n">
-        <v>11.02</v>
+        <v>-10.88</v>
       </c>
     </row>
     <row r="64">
@@ -3306,25 +3306,25 @@
         <v>8</v>
       </c>
       <c r="G64" t="n">
-        <v>12101.89071253337</v>
+        <v>1206.78778446288</v>
       </c>
       <c r="H64" t="n">
-        <v>-317.0210794880514</v>
+        <v>-305.6298899316962</v>
       </c>
       <c r="I64" t="n">
-        <v>319.3796326336638</v>
+        <v>139.0602363101074</v>
       </c>
       <c r="J64" t="n">
         <v>0.5</v>
       </c>
       <c r="K64" t="n">
-        <v>362.0354958462345</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L64" t="n">
-        <v>7695.53</v>
+        <v>492.6</v>
       </c>
       <c r="M64" t="n">
-        <v>-154.48</v>
+        <v>-13.25</v>
       </c>
     </row>
     <row r="65">
@@ -3351,25 +3351,25 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>8976.577863166549</v>
+        <v>7000.619463702522</v>
       </c>
       <c r="H65" t="n">
-        <v>-115.4865786618157</v>
+        <v>-122.3748775955414</v>
       </c>
       <c r="I65" t="n">
-        <v>145.645574899756</v>
+        <v>286.8093496478072</v>
       </c>
       <c r="J65" t="n">
         <v>0.5</v>
       </c>
       <c r="K65" t="n">
-        <v>186.9543261531214</v>
+        <v>310.0286763918156</v>
       </c>
       <c r="L65" t="n">
-        <v>3403.06</v>
+        <v>4675.35</v>
       </c>
       <c r="M65" t="n">
-        <v>33.84</v>
+        <v>-33.27</v>
       </c>
     </row>
     <row r="66">
@@ -3396,25 +3396,25 @@
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>985.6631684384834</v>
+        <v>985.4325906549896</v>
       </c>
       <c r="H66" t="n">
-        <v>-184.135283405567</v>
+        <v>27.11408007246451</v>
       </c>
       <c r="I66" t="n">
-        <v>219.0252115834215</v>
+        <v>228.3598330513809</v>
       </c>
       <c r="J66" t="n">
         <v>0.5</v>
       </c>
       <c r="K66" t="n">
-        <v>209.0212909830231</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L66" t="n">
-        <v>608.89</v>
+        <v>646.5700000000001</v>
       </c>
       <c r="M66" t="n">
-        <v>-73.64</v>
+        <v>61.15</v>
       </c>
     </row>
     <row r="67">
@@ -3441,25 +3441,25 @@
         <v>2</v>
       </c>
       <c r="G67" t="n">
-        <v>9149.911154774773</v>
+        <v>1730.279533356723</v>
       </c>
       <c r="H67" t="n">
-        <v>-147.9386034386221</v>
+        <v>-204.0508608304035</v>
       </c>
       <c r="I67" t="n">
-        <v>235.3122205840817</v>
+        <v>176.3192932042115</v>
       </c>
       <c r="J67" t="n">
         <v>0.5</v>
       </c>
       <c r="K67" t="n">
-        <v>272.5304205830174</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L67" t="n">
-        <v>5201.34</v>
+        <v>899.75</v>
       </c>
       <c r="M67" t="n">
-        <v>-43.07</v>
+        <v>-22.34</v>
       </c>
     </row>
     <row r="68">
@@ -3486,25 +3486,25 @@
         <v>3</v>
       </c>
       <c r="G68" t="n">
-        <v>2639.652859927551</v>
+        <v>2565.427984934037</v>
       </c>
       <c r="H68" t="n">
-        <v>-211.2618638835868</v>
+        <v>-203.698056087992</v>
       </c>
       <c r="I68" t="n">
-        <v>209.3129769283018</v>
+        <v>171.0286750744761</v>
       </c>
       <c r="J68" t="n">
         <v>0.5</v>
       </c>
       <c r="K68" t="n">
-        <v>219.2233794389425</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L68" t="n">
-        <v>1550.48</v>
+        <v>1237.12</v>
       </c>
       <c r="M68" t="n">
-        <v>-52.06</v>
+        <v>20.59</v>
       </c>
     </row>
     <row r="69">
@@ -3531,25 +3531,25 @@
         <v>4</v>
       </c>
       <c r="G69" t="n">
-        <v>960.4411204732279</v>
+        <v>1176.614116731286</v>
       </c>
       <c r="H69" t="n">
-        <v>-51.86419713639165</v>
+        <v>-216.8601988224301</v>
       </c>
       <c r="I69" t="n">
-        <v>203.0476679464295</v>
+        <v>433.4279297170322</v>
       </c>
       <c r="J69" t="n">
         <v>0.5</v>
       </c>
       <c r="K69" t="n">
-        <v>198.2950076925505</v>
+        <v>402.0604809124811</v>
       </c>
       <c r="L69" t="n">
-        <v>589.6799999999999</v>
+        <v>953.21</v>
       </c>
       <c r="M69" t="n">
-        <v>38.94</v>
+        <v>-178.06</v>
       </c>
     </row>
     <row r="70">
@@ -3576,25 +3576,25 @@
         <v>5</v>
       </c>
       <c r="G70" t="n">
-        <v>1123.250489118219</v>
+        <v>201.9796078230057</v>
       </c>
       <c r="H70" t="n">
-        <v>-160.418552219151</v>
+        <v>-365.3792366197873</v>
       </c>
       <c r="I70" t="n">
-        <v>449.2914158082303</v>
+        <v>281.2568731550044</v>
       </c>
       <c r="J70" t="n">
         <v>0.5</v>
       </c>
       <c r="K70" t="n">
-        <v>433.4357742066306</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L70" t="n">
-        <v>904.8</v>
+        <v>11.44</v>
       </c>
       <c r="M70" t="n">
-        <v>-108.86</v>
+        <v>41.83</v>
       </c>
     </row>
     <row r="71">
@@ -3621,25 +3621,25 @@
         <v>6</v>
       </c>
       <c r="G71" t="n">
-        <v>1348.379432507424</v>
+        <v>1180.045759365336</v>
       </c>
       <c r="H71" t="n">
-        <v>-102.4924644161888</v>
+        <v>-123.1199656076542</v>
       </c>
       <c r="I71" t="n">
-        <v>273.8692346923003</v>
+        <v>407.4607313568296</v>
       </c>
       <c r="J71" t="n">
         <v>0.5</v>
       </c>
       <c r="K71" t="n">
-        <v>272.5304205830174</v>
+        <v>385.4162169477469</v>
       </c>
       <c r="L71" t="n">
-        <v>953.24</v>
+        <v>940.12</v>
       </c>
       <c r="M71" t="n">
-        <v>-34.11</v>
+        <v>-79.73999999999999</v>
       </c>
     </row>
     <row r="72">
@@ -3666,25 +3666,25 @@
         <v>7</v>
       </c>
       <c r="G72" t="n">
-        <v>2298.711745538368</v>
+        <v>822.0646371462506</v>
       </c>
       <c r="H72" t="n">
-        <v>-59.46157063534964</v>
+        <v>-320.6730861682562</v>
       </c>
       <c r="I72" t="n">
-        <v>206.4054375177427</v>
+        <v>303.0735635241507</v>
       </c>
       <c r="J72" t="n">
         <v>0.5</v>
       </c>
       <c r="K72" t="n">
-        <v>209.0212909830231</v>
+        <v>295.6007445329244</v>
       </c>
       <c r="L72" t="n">
-        <v>1307</v>
+        <v>600.9400000000001</v>
       </c>
       <c r="M72" t="n">
-        <v>8.470000000000001</v>
+        <v>-202.9</v>
       </c>
     </row>
     <row r="73">
@@ -3711,25 +3711,25 @@
         <v>8</v>
       </c>
       <c r="G73" t="n">
-        <v>11129.88535990703</v>
+        <v>1298.052235869256</v>
       </c>
       <c r="H73" t="n">
-        <v>-237.7948422627874</v>
+        <v>-312.1511062265459</v>
       </c>
       <c r="I73" t="n">
-        <v>256.0709530494113</v>
+        <v>150.7531717170063</v>
       </c>
       <c r="J73" t="n">
         <v>0.5</v>
       </c>
       <c r="K73" t="n">
-        <v>302.9006275609877</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L73" t="n">
-        <v>6301.24</v>
+        <v>556.5599999999999</v>
       </c>
       <c r="M73" t="n">
-        <v>-90.41</v>
+        <v>-11.15</v>
       </c>
     </row>
     <row r="74">
@@ -3756,25 +3756,25 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>7730.354834235022</v>
+        <v>6123.625509057643</v>
       </c>
       <c r="H74" t="n">
-        <v>-122.0583799601923</v>
+        <v>-126.0944492380486</v>
       </c>
       <c r="I74" t="n">
-        <v>153.4729769766308</v>
+        <v>349.5151828160974</v>
       </c>
       <c r="J74" t="n">
         <v>0.5</v>
       </c>
       <c r="K74" t="n">
-        <v>198.2950076925505</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L74" t="n">
-        <v>2891.78</v>
+        <v>4783.54</v>
       </c>
       <c r="M74" t="n">
-        <v>-9.220000000000001</v>
+        <v>-78.58</v>
       </c>
     </row>
     <row r="75">
@@ -3801,25 +3801,25 @@
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>998.9898372717624</v>
+        <v>1056.352336803373</v>
       </c>
       <c r="H75" t="n">
-        <v>-113.84404005753</v>
+        <v>-8.404530874247055</v>
       </c>
       <c r="I75" t="n">
-        <v>228.1353713444672</v>
+        <v>276.7577221947439</v>
       </c>
       <c r="J75" t="n">
         <v>0.5</v>
       </c>
       <c r="K75" t="n">
-        <v>228.9713521405058</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L75" t="n">
-        <v>685.05</v>
+        <v>737.1900000000001</v>
       </c>
       <c r="M75" t="n">
-        <v>-14.91</v>
+        <v>33.03</v>
       </c>
     </row>
     <row r="76">
@@ -3846,25 +3846,25 @@
         <v>2</v>
       </c>
       <c r="G76" t="n">
-        <v>8172.739780454887</v>
+        <v>1191.202044964468</v>
       </c>
       <c r="H76" t="n">
-        <v>-91.71072173097019</v>
+        <v>-196.9607106649994</v>
       </c>
       <c r="I76" t="n">
-        <v>187.047220298663</v>
+        <v>247.7666170094034</v>
       </c>
       <c r="J76" t="n">
         <v>0.5</v>
       </c>
       <c r="K76" t="n">
-        <v>228.9713521405058</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L76" t="n">
-        <v>3968.2</v>
+        <v>802.0599999999999</v>
       </c>
       <c r="M76" t="n">
-        <v>22.93</v>
+        <v>-69.84</v>
       </c>
     </row>
     <row r="77">
@@ -3891,25 +3891,25 @@
         <v>3</v>
       </c>
       <c r="G77" t="n">
-        <v>1896.934847896233</v>
+        <v>1810.830902282436</v>
       </c>
       <c r="H77" t="n">
-        <v>-167.0502441092096</v>
+        <v>-201.6804912776164</v>
       </c>
       <c r="I77" t="n">
-        <v>297.691882611655</v>
+        <v>205.3279592461455</v>
       </c>
       <c r="J77" t="n">
         <v>0.5</v>
       </c>
       <c r="K77" t="n">
-        <v>310.0286763918156</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L77" t="n">
-        <v>1371.88</v>
+        <v>1070.07</v>
       </c>
       <c r="M77" t="n">
-        <v>-79.87</v>
+        <v>-101.7</v>
       </c>
     </row>
     <row r="78">
@@ -3936,25 +3936,25 @@
         <v>4</v>
       </c>
       <c r="G78" t="n">
-        <v>948.4279449243487</v>
+        <v>1157.087928525535</v>
       </c>
       <c r="H78" t="n">
-        <v>-62.11783961966383</v>
+        <v>-206.8354477858767</v>
       </c>
       <c r="I78" t="n">
-        <v>236.0572052879782</v>
+        <v>386.1110652443137</v>
       </c>
       <c r="J78" t="n">
         <v>0.5</v>
       </c>
       <c r="K78" t="n">
-        <v>174.8797588600428</v>
+        <v>373.9086523062428</v>
       </c>
       <c r="L78" t="n">
-        <v>615.36</v>
+        <v>922.42</v>
       </c>
       <c r="M78" t="n">
-        <v>-35.51</v>
+        <v>-144.02</v>
       </c>
     </row>
     <row r="79">
@@ -3981,25 +3981,25 @@
         <v>5</v>
       </c>
       <c r="G79" t="n">
-        <v>1093.077259066999</v>
+        <v>664.0510017859363</v>
       </c>
       <c r="H79" t="n">
-        <v>-74.78251139051456</v>
+        <v>-303.3117675304483</v>
       </c>
       <c r="I79" t="n">
-        <v>383.6775482803339</v>
+        <v>293.4660350111529</v>
       </c>
       <c r="J79" t="n">
         <v>0.5</v>
       </c>
       <c r="K79" t="n">
-        <v>373.9086523062428</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L79" t="n">
-        <v>849.54</v>
+        <v>506.52</v>
       </c>
       <c r="M79" t="n">
-        <v>-32.13</v>
+        <v>-178.19</v>
       </c>
     </row>
     <row r="80">
@@ -4026,25 +4026,25 @@
         <v>6</v>
       </c>
       <c r="G80" t="n">
-        <v>1263.461006849141</v>
+        <v>1144.261490794253</v>
       </c>
       <c r="H80" t="n">
-        <v>-94.03020225474324</v>
+        <v>-113.4110737886242</v>
       </c>
       <c r="I80" t="n">
-        <v>281.7508111423556</v>
+        <v>374.1917192802561</v>
       </c>
       <c r="J80" t="n">
         <v>0.5</v>
       </c>
       <c r="K80" t="n">
-        <v>255.9977541431066</v>
+        <v>385.4162169477469</v>
       </c>
       <c r="L80" t="n">
-        <v>923.4</v>
+        <v>840.28</v>
       </c>
       <c r="M80" t="n">
-        <v>-39.42</v>
+        <v>-55.38</v>
       </c>
     </row>
     <row r="81">
@@ -4071,25 +4071,25 @@
         <v>7</v>
       </c>
       <c r="G81" t="n">
-        <v>2215.082600809384</v>
+        <v>2093.924947109726</v>
       </c>
       <c r="H81" t="n">
-        <v>-65.1736090109699</v>
+        <v>-291.6612975366837</v>
       </c>
       <c r="I81" t="n">
-        <v>180.9651670332532</v>
+        <v>313.0542339472323</v>
       </c>
       <c r="J81" t="n">
         <v>0.5</v>
       </c>
       <c r="K81" t="n">
-        <v>186.9543261531214</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L81" t="n">
-        <v>2119.21</v>
+        <v>1459.57</v>
       </c>
       <c r="M81" t="n">
-        <v>42.23</v>
+        <v>-182.96</v>
       </c>
     </row>
     <row r="82">
@@ -4116,25 +4116,25 @@
         <v>8</v>
       </c>
       <c r="G82" t="n">
-        <v>10174.60141269085</v>
+        <v>1398.764877488584</v>
       </c>
       <c r="H82" t="n">
-        <v>-172.2389656368968</v>
+        <v>-316.6279087795085</v>
       </c>
       <c r="I82" t="n">
-        <v>202.5363641500476</v>
+        <v>162.3006745578103</v>
       </c>
       <c r="J82" t="n">
         <v>0.5</v>
       </c>
       <c r="K82" t="n">
-        <v>255.9977541431066</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L82" t="n">
-        <v>5073.2</v>
+        <v>678.84</v>
       </c>
       <c r="M82" t="n">
-        <v>-22.98</v>
+        <v>-23.47</v>
       </c>
     </row>
     <row r="83">
@@ -4161,25 +4161,25 @@
         <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>6679.742734420605</v>
+        <v>5187.495717361434</v>
       </c>
       <c r="H83" t="n">
-        <v>-129.4365454467413</v>
+        <v>-126.8932192704564</v>
       </c>
       <c r="I83" t="n">
-        <v>162.4082351183447</v>
+        <v>348.2463326247159</v>
       </c>
       <c r="J83" t="n">
         <v>0.5</v>
       </c>
       <c r="K83" t="n">
-        <v>209.0212909830231</v>
+        <v>391.0430286998269</v>
       </c>
       <c r="L83" t="n">
-        <v>2453.43</v>
+        <v>3549.03</v>
       </c>
       <c r="M83" t="n">
-        <v>50.84</v>
+        <v>-50.21</v>
       </c>
     </row>
     <row r="84">
@@ -4206,25 +4206,25 @@
         <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>1049.577375560766</v>
+        <v>1112.265957171275</v>
       </c>
       <c r="H84" t="n">
-        <v>-57.93580190153996</v>
+        <v>-59.74920766254394</v>
       </c>
       <c r="I84" t="n">
-        <v>289.1746264512425</v>
+        <v>322.6802012782422</v>
       </c>
       <c r="J84" t="n">
         <v>0.5</v>
       </c>
       <c r="K84" t="n">
-        <v>272.5304205830174</v>
+        <v>330.4916794875841</v>
       </c>
       <c r="L84" t="n">
-        <v>715.24</v>
+        <v>803.85</v>
       </c>
       <c r="M84" t="n">
-        <v>-8.17</v>
+        <v>-13.9</v>
       </c>
     </row>
     <row r="85">
@@ -4251,25 +4251,25 @@
         <v>2</v>
       </c>
       <c r="G85" t="n">
-        <v>7201.578965891139</v>
+        <v>765.2940145861428</v>
       </c>
       <c r="H85" t="n">
-        <v>-54.85534803329845</v>
+        <v>-193.6616490756933</v>
       </c>
       <c r="I85" t="n">
-        <v>167.0509018539257</v>
+        <v>371.5785155021347</v>
       </c>
       <c r="J85" t="n">
         <v>0.5</v>
       </c>
       <c r="K85" t="n">
-        <v>209.0212909830231</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L85" t="n">
-        <v>3304.93</v>
+        <v>557.3200000000001</v>
       </c>
       <c r="M85" t="n">
-        <v>43.72</v>
+        <v>-121.03</v>
       </c>
     </row>
     <row r="86">
@@ -4296,25 +4296,25 @@
         <v>3</v>
       </c>
       <c r="G86" t="n">
-        <v>1153.655780451532</v>
+        <v>1303.118867031556</v>
       </c>
       <c r="H86" t="n">
-        <v>-123.5487997657273</v>
+        <v>-204.9859767609692</v>
       </c>
       <c r="I86" t="n">
-        <v>383.1039828470152</v>
+        <v>270.3599147440521</v>
       </c>
       <c r="J86" t="n">
         <v>0.5</v>
       </c>
       <c r="K86" t="n">
-        <v>396.590015385101</v>
+        <v>272.5304205830174</v>
       </c>
       <c r="L86" t="n">
-        <v>863.78</v>
+        <v>906.1900000000001</v>
       </c>
       <c r="M86" t="n">
-        <v>-66.92</v>
+        <v>-100.51</v>
       </c>
     </row>
     <row r="87">
@@ -4341,25 +4341,25 @@
         <v>4</v>
       </c>
       <c r="G87" t="n">
-        <v>964.9520007103177</v>
+        <v>1123.320400126065</v>
       </c>
       <c r="H87" t="n">
-        <v>-73.92988867493112</v>
+        <v>-196.1323994168356</v>
       </c>
       <c r="I87" t="n">
-        <v>269.3653491052601</v>
+        <v>334.1110084459722</v>
       </c>
       <c r="J87" t="n">
         <v>0.5</v>
       </c>
       <c r="K87" t="n">
-        <v>247.317326764409</v>
+        <v>343.4570282107588</v>
       </c>
       <c r="L87" t="n">
-        <v>608.14</v>
+        <v>841.09</v>
       </c>
       <c r="M87" t="n">
-        <v>4.17</v>
+        <v>-102.17</v>
       </c>
     </row>
     <row r="88">
@@ -4386,25 +4386,25 @@
         <v>5</v>
       </c>
       <c r="G88" t="n">
-        <v>1030.199254376652</v>
+        <v>1525.025314986135</v>
       </c>
       <c r="H88" t="n">
-        <v>-2.941570257932085</v>
+        <v>-297.9652380745541</v>
       </c>
       <c r="I88" t="n">
-        <v>267.4905745735769</v>
+        <v>305.5502336972414</v>
       </c>
       <c r="J88" t="n">
         <v>0.5</v>
       </c>
       <c r="K88" t="n">
-        <v>264.3933435900673</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L88" t="n">
-        <v>710.48</v>
+        <v>1099.32</v>
       </c>
       <c r="M88" t="n">
-        <v>60.12</v>
+        <v>-186.67</v>
       </c>
     </row>
     <row r="89">
@@ -4431,25 +4431,25 @@
         <v>6</v>
       </c>
       <c r="G89" t="n">
-        <v>1178.906678393879</v>
+        <v>1084.466425801775</v>
       </c>
       <c r="H89" t="n">
-        <v>-86.98887644845881</v>
+        <v>-103.1907882741176</v>
       </c>
       <c r="I89" t="n">
-        <v>287.2148691201639</v>
+        <v>315.4220580756721</v>
       </c>
       <c r="J89" t="n">
         <v>0.5</v>
       </c>
       <c r="K89" t="n">
-        <v>264.3933435900673</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L89" t="n">
-        <v>839.86</v>
+        <v>730.76</v>
       </c>
       <c r="M89" t="n">
-        <v>-37.15</v>
+        <v>-87</v>
       </c>
     </row>
     <row r="90">
@@ -4476,25 +4476,25 @@
         <v>7</v>
       </c>
       <c r="G90" t="n">
-        <v>2142.515168320037</v>
+        <v>2530.689042083179</v>
       </c>
       <c r="H90" t="n">
-        <v>-72.89604847396375</v>
+        <v>-221.5181348635559</v>
       </c>
       <c r="I90" t="n">
-        <v>192.3066843837999</v>
+        <v>314.7814355824629</v>
       </c>
       <c r="J90" t="n">
         <v>0.5</v>
       </c>
       <c r="K90" t="n">
-        <v>198.2950076925505</v>
+        <v>343.4570282107588</v>
       </c>
       <c r="L90" t="n">
-        <v>1270.99</v>
+        <v>1705.53</v>
       </c>
       <c r="M90" t="n">
-        <v>-16.25</v>
+        <v>-116.49</v>
       </c>
     </row>
     <row r="91">
@@ -4521,25 +4521,25 @@
         <v>8</v>
       </c>
       <c r="G91" t="n">
-        <v>9231.427182341828</v>
+        <v>1485.039566469768</v>
       </c>
       <c r="H91" t="n">
-        <v>-120.7163624288772</v>
+        <v>-321.1203250320734</v>
       </c>
       <c r="I91" t="n">
-        <v>168.7009603379393</v>
+        <v>173.6462845105228</v>
       </c>
       <c r="J91" t="n">
         <v>0.5</v>
       </c>
       <c r="K91" t="n">
-        <v>209.0212909830231</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L91" t="n">
-        <v>4226.75</v>
+        <v>749.33</v>
       </c>
       <c r="M91" t="n">
-        <v>27.9</v>
+        <v>-81.68000000000001</v>
       </c>
     </row>
     <row r="92">
@@ -4566,25 +4566,25 @@
         <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>5617.332938579431</v>
+        <v>4290.077032974634</v>
       </c>
       <c r="H92" t="n">
-        <v>-133.8292902717329</v>
+        <v>-121.0656081690849</v>
       </c>
       <c r="I92" t="n">
-        <v>172.2454659385792</v>
+        <v>313.3841357064874</v>
       </c>
       <c r="J92" t="n">
         <v>0.5</v>
       </c>
       <c r="K92" t="n">
-        <v>198.2950076925505</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L92" t="n">
-        <v>2773.91</v>
+        <v>2836.87</v>
       </c>
       <c r="M92" t="n">
-        <v>-26.23</v>
+        <v>-37.24</v>
       </c>
     </row>
     <row r="93">
@@ -4611,25 +4611,25 @@
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>1103.836964676151</v>
+        <v>1128.735927485365</v>
       </c>
       <c r="H93" t="n">
-        <v>-39.54127393015071</v>
+        <v>-115.9745722777635</v>
       </c>
       <c r="I93" t="n">
-        <v>394.4287036971203</v>
+        <v>344.6673342990532</v>
       </c>
       <c r="J93" t="n">
         <v>0.5</v>
       </c>
       <c r="K93" t="n">
-        <v>385.4162169477469</v>
+        <v>343.4570282107588</v>
       </c>
       <c r="L93" t="n">
-        <v>889.25</v>
+        <v>846.21</v>
       </c>
       <c r="M93" t="n">
-        <v>-1.17</v>
+        <v>-57.38</v>
       </c>
     </row>
     <row r="94">
@@ -4656,25 +4656,25 @@
         <v>2</v>
       </c>
       <c r="G94" t="n">
-        <v>6354.804093327559</v>
+        <v>515.6835788024292</v>
       </c>
       <c r="H94" t="n">
-        <v>-57.58146918787546</v>
+        <v>-185.3510118303306</v>
       </c>
       <c r="I94" t="n">
-        <v>179.6504578397151</v>
+        <v>440.6799261922779</v>
       </c>
       <c r="J94" t="n">
         <v>0.5</v>
       </c>
       <c r="K94" t="n">
-        <v>219.2233794389425</v>
+        <v>457.9427042810117</v>
       </c>
       <c r="L94" t="n">
-        <v>3110.14</v>
+        <v>354.48</v>
       </c>
       <c r="M94" t="n">
-        <v>45.01</v>
+        <v>-84.20999999999999</v>
       </c>
     </row>
     <row r="95">
@@ -4701,25 +4701,25 @@
         <v>3</v>
       </c>
       <c r="G95" t="n">
-        <v>534.6759451121488</v>
+        <v>935.8520111106213</v>
       </c>
       <c r="H95" t="n">
-        <v>-68.07543078208008</v>
+        <v>-197.5360651900623</v>
       </c>
       <c r="I95" t="n">
-        <v>384.0260855502955</v>
+        <v>327.9796020481474</v>
       </c>
       <c r="J95" t="n">
         <v>0.5</v>
       </c>
       <c r="K95" t="n">
-        <v>362.0354958462345</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L95" t="n">
-        <v>312.64</v>
+        <v>599.35</v>
       </c>
       <c r="M95" t="n">
-        <v>-15.99</v>
+        <v>-111.01</v>
       </c>
     </row>
     <row r="96">
@@ -4746,25 +4746,25 @@
         <v>4</v>
       </c>
       <c r="G96" t="n">
-        <v>1003.192647082326</v>
+        <v>1081.485784079449</v>
       </c>
       <c r="H96" t="n">
-        <v>-74.14173786160116</v>
+        <v>-185.9956770663789</v>
       </c>
       <c r="I96" t="n">
-        <v>339.6836054628201</v>
+        <v>277.8141438515309</v>
       </c>
       <c r="J96" t="n">
         <v>0.5</v>
       </c>
       <c r="K96" t="n">
-        <v>302.9006275609877</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L96" t="n">
-        <v>719.4400000000001</v>
+        <v>788.88</v>
       </c>
       <c r="M96" t="n">
-        <v>-36.26</v>
+        <v>-108</v>
       </c>
     </row>
     <row r="97">
@@ -4791,25 +4791,25 @@
         <v>5</v>
       </c>
       <c r="G97" t="n">
-        <v>934.7345346945779</v>
+        <v>1954.714755000457</v>
       </c>
       <c r="H97" t="n">
-        <v>39.55032836788105</v>
+        <v>-238.3653748326371</v>
       </c>
       <c r="I97" t="n">
-        <v>132.5800471057387</v>
+        <v>310.5851496172795</v>
       </c>
       <c r="J97" t="n">
         <v>0.5</v>
       </c>
       <c r="K97" t="n">
-        <v>132.1966717950337</v>
+        <v>310.0286763918156</v>
       </c>
       <c r="L97" t="n">
-        <v>382.42</v>
+        <v>1394.35</v>
       </c>
       <c r="M97" t="n">
-        <v>99.52</v>
+        <v>-139.33</v>
       </c>
     </row>
     <row r="98">
@@ -4836,25 +4836,25 @@
         <v>6</v>
       </c>
       <c r="G98" t="n">
-        <v>1104.430089366956</v>
+        <v>1029.215914217547</v>
       </c>
       <c r="H98" t="n">
-        <v>-79.16947248308036</v>
+        <v>-94.17359212002884</v>
       </c>
       <c r="I98" t="n">
-        <v>298.0322256331597</v>
+        <v>230.9222477195183</v>
       </c>
       <c r="J98" t="n">
         <v>0.5</v>
       </c>
       <c r="K98" t="n">
-        <v>272.5304205830174</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L98" t="n">
-        <v>755.75</v>
+        <v>700.5599999999999</v>
       </c>
       <c r="M98" t="n">
-        <v>-22.24</v>
+        <v>-18.15</v>
       </c>
     </row>
     <row r="99">
@@ -4881,25 +4881,25 @@
         <v>7</v>
       </c>
       <c r="G99" t="n">
-        <v>2051.034839792969</v>
+        <v>2221.310456089379</v>
       </c>
       <c r="H99" t="n">
-        <v>-83.93418281636359</v>
+        <v>-150.8521210825751</v>
       </c>
       <c r="I99" t="n">
-        <v>215.2141360603577</v>
+        <v>310.9399389338864</v>
       </c>
       <c r="J99" t="n">
         <v>0.5</v>
       </c>
       <c r="K99" t="n">
-        <v>228.9713521405058</v>
+        <v>310.0286763918156</v>
       </c>
       <c r="L99" t="n">
-        <v>1166.53</v>
+        <v>1545.58</v>
       </c>
       <c r="M99" t="n">
-        <v>24.82</v>
+        <v>-69.52</v>
       </c>
     </row>
     <row r="100">
@@ -4926,25 +4926,25 @@
         <v>8</v>
       </c>
       <c r="G100" t="n">
-        <v>8266.264942713562</v>
+        <v>1542.774716318924</v>
       </c>
       <c r="H100" t="n">
-        <v>-95.37308012207575</v>
+        <v>-322.3979342740296</v>
       </c>
       <c r="I100" t="n">
-        <v>165.382614517106</v>
+        <v>186.1954048850868</v>
       </c>
       <c r="J100" t="n">
         <v>0.5</v>
       </c>
       <c r="K100" t="n">
-        <v>209.0212909830231</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L100" t="n">
-        <v>3748.71</v>
+        <v>798.99</v>
       </c>
       <c r="M100" t="n">
-        <v>67.92</v>
+        <v>-91.43000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -5047,30 +5047,30 @@
         <v>6</v>
       </c>
       <c r="G2" t="n">
-        <v>1104.430089366956</v>
+        <v>1029.215914217547</v>
       </c>
       <c r="H2" t="n">
-        <v>-79.16947248308036</v>
+        <v>-94.17359212002884</v>
       </c>
       <c r="I2" t="n">
-        <v>298.0322256331597</v>
+        <v>230.9222477195183</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>272.5304205830174</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L2" t="n">
-        <v>755.75</v>
+        <v>700.5599999999999</v>
       </c>
       <c r="M2" t="n">
-        <v>-22.24</v>
+        <v>-18.15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -5089,28 +5089,28 @@
         <v>8</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G3" t="n">
-        <v>998.9898372717624</v>
+        <v>1398.764877488584</v>
       </c>
       <c r="H3" t="n">
-        <v>-113.84404005753</v>
+        <v>-316.6279087795085</v>
       </c>
       <c r="I3" t="n">
-        <v>228.1353713444672</v>
+        <v>162.3006745578103</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>228.9713521405058</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L3" t="n">
-        <v>685.05</v>
+        <v>678.84</v>
       </c>
       <c r="M3" t="n">
-        <v>-14.91</v>
+        <v>-23.47</v>
       </c>
     </row>
     <row r="4">
@@ -5137,25 +5137,25 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>1049.577375560766</v>
+        <v>1112.265957171275</v>
       </c>
       <c r="H4" t="n">
-        <v>-57.93580190153996</v>
+        <v>-59.74920766254394</v>
       </c>
       <c r="I4" t="n">
-        <v>289.1746264512425</v>
+        <v>322.6802012782422</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>272.5304205830174</v>
+        <v>330.4916794875841</v>
       </c>
       <c r="L4" t="n">
-        <v>715.24</v>
+        <v>803.85</v>
       </c>
       <c r="M4" t="n">
-        <v>-8.17</v>
+        <v>-13.9</v>
       </c>
     </row>
   </sheetData>
@@ -5268,31 +5268,31 @@
         <v>-21.42555</v>
       </c>
       <c r="G2" t="n">
-        <v>271</v>
+        <v>238</v>
       </c>
       <c r="H2" t="n">
-        <v>38</v>
+        <v>80</v>
       </c>
       <c r="I2" t="n">
-        <v>1050</v>
+        <v>1180</v>
       </c>
       <c r="J2" t="n">
-        <v>52</v>
+        <v>193</v>
       </c>
       <c r="K2" t="n">
-        <v>-83</v>
+        <v>-156</v>
       </c>
       <c r="L2" t="n">
-        <v>52</v>
+        <v>193</v>
       </c>
       <c r="M2" t="n">
-        <v>-3.18</v>
+        <v>-17.52</v>
       </c>
       <c r="N2" t="n">
-        <v>30.87637282532287</v>
+        <v>38.43745211570078</v>
       </c>
       <c r="O2" t="n">
-        <v>74.38660067954987</v>
+        <v>86.34012257756068</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: first version streamlit gui
</commit_message>
<xml_diff>
--- a/test_alldata.xlsx
+++ b/test_alldata.xlsx
@@ -516,25 +516,25 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>13000</v>
+        <v>1100</v>
       </c>
       <c r="H2" t="n">
-        <v>-100</v>
+        <v>-850</v>
       </c>
       <c r="I2" t="n">
-        <v>450</v>
+        <v>850</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>494.634653528818</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L2" t="n">
-        <v>9486.24</v>
+        <v>10563.78</v>
       </c>
       <c r="M2" t="n">
-        <v>-37.34</v>
+        <v>12.66</v>
       </c>
     </row>
     <row r="3">
@@ -561,25 +561,25 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1200</v>
+        <v>18000</v>
       </c>
       <c r="H3" t="n">
-        <v>-350</v>
+        <v>-250</v>
       </c>
       <c r="I3" t="n">
-        <v>700</v>
+        <v>850</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>686.9140564215176</v>
+        <v>856.7323510961411</v>
       </c>
       <c r="L3" t="n">
-        <v>1040.18</v>
+        <v>15821.55</v>
       </c>
       <c r="M3" t="n">
-        <v>-307.9</v>
+        <v>-219.23</v>
       </c>
     </row>
     <row r="4">
@@ -609,22 +609,22 @@
         <v>8000</v>
       </c>
       <c r="H4" t="n">
-        <v>-250</v>
+        <v>-400</v>
       </c>
       <c r="I4" t="n">
-        <v>650</v>
+        <v>500</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>674.0734091148975</v>
+        <v>541.0381969548956</v>
       </c>
       <c r="L4" t="n">
-        <v>6684.26</v>
+        <v>6040.45</v>
       </c>
       <c r="M4" t="n">
-        <v>-195.63</v>
+        <v>-274.63</v>
       </c>
     </row>
     <row r="5">
@@ -651,25 +651,25 @@
         <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>9000</v>
+        <v>1200</v>
       </c>
       <c r="H5" t="n">
-        <v>-250</v>
+        <v>-550</v>
       </c>
       <c r="I5" t="n">
-        <v>700</v>
+        <v>150</v>
       </c>
       <c r="J5" t="n">
         <v>0.5</v>
       </c>
       <c r="K5" t="n">
-        <v>727.081694872685</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L5" t="n">
-        <v>7549.2</v>
+        <v>547.12</v>
       </c>
       <c r="M5" t="n">
-        <v>-194.39</v>
+        <v>-159.89</v>
       </c>
     </row>
     <row r="6">
@@ -696,25 +696,25 @@
         <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>1100</v>
+        <v>6000</v>
       </c>
       <c r="H6" t="n">
-        <v>-250</v>
+        <v>-600</v>
       </c>
       <c r="I6" t="n">
-        <v>350</v>
+        <v>800</v>
       </c>
       <c r="J6" t="n">
         <v>0.5</v>
       </c>
       <c r="K6" t="n">
-        <v>355.9504322854629</v>
+        <v>809.5359789800231</v>
       </c>
       <c r="L6" t="n">
-        <v>850.78</v>
+        <v>5264.37</v>
       </c>
       <c r="M6" t="n">
-        <v>-167.07</v>
+        <v>-527.37</v>
       </c>
     </row>
     <row r="7">
@@ -741,25 +741,25 @@
         <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>5000</v>
+        <v>13000</v>
       </c>
       <c r="H7" t="n">
-        <v>-850</v>
+        <v>-800</v>
       </c>
       <c r="I7" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="J7" t="n">
         <v>0.5</v>
       </c>
       <c r="K7" t="n">
-        <v>288.1159665134826</v>
+        <v>549.0540142654876</v>
       </c>
       <c r="L7" t="n">
-        <v>3721.11</v>
+        <v>9855.559999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>-598.1900000000001</v>
+        <v>-578.12</v>
       </c>
     </row>
     <row r="8">
@@ -786,10 +786,10 @@
         <v>6</v>
       </c>
       <c r="G8" t="n">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="H8" t="n">
-        <v>-150</v>
+        <v>-400</v>
       </c>
       <c r="I8" t="n">
         <v>450</v>
@@ -801,10 +801,10 @@
         <v>428.3661755480705</v>
       </c>
       <c r="L8" t="n">
-        <v>733.8200000000001</v>
+        <v>814.77</v>
       </c>
       <c r="M8" t="n">
-        <v>-96.70999999999999</v>
+        <v>-324.13</v>
       </c>
     </row>
     <row r="9">
@@ -831,25 +831,25 @@
         <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>4000</v>
+        <v>800</v>
       </c>
       <c r="H9" t="n">
-        <v>-800</v>
+        <v>-550</v>
       </c>
       <c r="I9" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="J9" t="n">
         <v>0.5</v>
       </c>
       <c r="K9" t="n">
-        <v>310.0286763918156</v>
+        <v>93.4771630765607</v>
       </c>
       <c r="L9" t="n">
-        <v>2799.97</v>
+        <v>367.62</v>
       </c>
       <c r="M9" t="n">
-        <v>-519.8099999999999</v>
+        <v>-63.75</v>
       </c>
     </row>
     <row r="10">
@@ -876,25 +876,25 @@
         <v>8</v>
       </c>
       <c r="G10" t="n">
-        <v>800</v>
+        <v>18000</v>
       </c>
       <c r="H10" t="n">
-        <v>-250</v>
+        <v>-100</v>
       </c>
       <c r="I10" t="n">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="J10" t="n">
         <v>0.5</v>
       </c>
       <c r="K10" t="n">
-        <v>114.4856760702529</v>
+        <v>494.634653528818</v>
       </c>
       <c r="L10" t="n">
-        <v>321.13</v>
+        <v>13313.79</v>
       </c>
       <c r="M10" t="n">
-        <v>68.23999999999999</v>
+        <v>-37.27</v>
       </c>
     </row>
     <row r="11">
@@ -921,25 +921,25 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>12000</v>
+        <v>1000</v>
       </c>
       <c r="H11" t="n">
-        <v>-110</v>
+        <v>-950</v>
       </c>
       <c r="I11" t="n">
-        <v>350</v>
+        <v>750</v>
       </c>
       <c r="J11" t="n">
         <v>0.5</v>
       </c>
       <c r="K11" t="n">
-        <v>385.4162169477469</v>
+        <v>739.0018613323109</v>
       </c>
       <c r="L11" t="n">
-        <v>8181.54</v>
+        <v>875.11</v>
       </c>
       <c r="M11" t="n">
-        <v>-38.01</v>
+        <v>-833.9400000000001</v>
       </c>
     </row>
     <row r="12">
@@ -966,25 +966,25 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>1100</v>
+        <v>17000</v>
       </c>
       <c r="H12" t="n">
-        <v>-450</v>
+        <v>-260</v>
       </c>
       <c r="I12" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
       <c r="J12" t="n">
         <v>0.5</v>
       </c>
       <c r="K12" t="n">
-        <v>594.8850230776515</v>
+        <v>795.9293632107308</v>
       </c>
       <c r="L12" t="n">
-        <v>911.09</v>
+        <v>13855.29</v>
       </c>
       <c r="M12" t="n">
-        <v>-371.24</v>
+        <v>-202.72</v>
       </c>
     </row>
     <row r="13">
@@ -1014,22 +1014,22 @@
         <v>7000</v>
       </c>
       <c r="H13" t="n">
-        <v>-260</v>
+        <v>-500</v>
       </c>
       <c r="I13" t="n">
-        <v>550</v>
+        <v>400</v>
       </c>
       <c r="J13" t="n">
         <v>0.5</v>
       </c>
       <c r="K13" t="n">
-        <v>591.2014890658488</v>
+        <v>428.3661755480705</v>
       </c>
       <c r="L13" t="n">
-        <v>5457.83</v>
+        <v>5210.1</v>
       </c>
       <c r="M13" t="n">
-        <v>-184.59</v>
+        <v>-346.08</v>
       </c>
     </row>
     <row r="14">
@@ -1056,25 +1056,25 @@
         <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>8000</v>
+        <v>1100</v>
       </c>
       <c r="H14" t="n">
-        <v>-260</v>
+        <v>-650</v>
       </c>
       <c r="I14" t="n">
-        <v>600</v>
+        <v>140</v>
       </c>
       <c r="J14" t="n">
         <v>0.5</v>
       </c>
       <c r="K14" t="n">
-        <v>616.5242336945269</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L14" t="n">
-        <v>6504.31</v>
+        <v>471.27</v>
       </c>
       <c r="M14" t="n">
-        <v>-206.03</v>
+        <v>-122.49</v>
       </c>
     </row>
     <row r="15">
@@ -1101,25 +1101,25 @@
         <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="H15" t="n">
-        <v>-260</v>
+        <v>-700</v>
       </c>
       <c r="I15" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="J15" t="n">
         <v>0.5</v>
       </c>
       <c r="K15" t="n">
-        <v>264.3933435900673</v>
+        <v>736.039918105125</v>
       </c>
       <c r="L15" t="n">
-        <v>690.4400000000001</v>
+        <v>4142.37</v>
       </c>
       <c r="M15" t="n">
-        <v>-166.85</v>
+        <v>-571.37</v>
       </c>
     </row>
     <row r="16">
@@ -1146,25 +1146,25 @@
         <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>4000</v>
+        <v>12000</v>
       </c>
       <c r="H16" t="n">
-        <v>-950</v>
+        <v>-900</v>
       </c>
       <c r="I16" t="n">
-        <v>290</v>
+        <v>400</v>
       </c>
       <c r="J16" t="n">
         <v>0.5</v>
       </c>
       <c r="K16" t="n">
-        <v>302.9006275609877</v>
+        <v>438.4467588778851</v>
       </c>
       <c r="L16" t="n">
-        <v>2780.83</v>
+        <v>8578.07</v>
       </c>
       <c r="M16" t="n">
-        <v>-626.96</v>
+        <v>-615.6</v>
       </c>
     </row>
     <row r="17">
@@ -1191,10 +1191,10 @@
         <v>6</v>
       </c>
       <c r="G17" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
       <c r="H17" t="n">
-        <v>-160</v>
+        <v>-500</v>
       </c>
       <c r="I17" t="n">
         <v>350</v>
@@ -1203,13 +1203,13 @@
         <v>0.5</v>
       </c>
       <c r="K17" t="n">
-        <v>337.0367045574487</v>
+        <v>114.4856760702529</v>
       </c>
       <c r="L17" t="n">
-        <v>614.03</v>
+        <v>1915.19</v>
       </c>
       <c r="M17" t="n">
-        <v>-63.87</v>
+        <v>-39.01</v>
       </c>
     </row>
     <row r="18">
@@ -1236,25 +1236,25 @@
         <v>7</v>
       </c>
       <c r="G18" t="n">
-        <v>3000</v>
+        <v>700</v>
       </c>
       <c r="H18" t="n">
-        <v>-900</v>
+        <v>-650</v>
       </c>
       <c r="I18" t="n">
-        <v>290</v>
+        <v>90</v>
       </c>
       <c r="J18" t="n">
         <v>0.5</v>
       </c>
       <c r="K18" t="n">
-        <v>288.1159665134826</v>
+        <v>114.4856760702529</v>
       </c>
       <c r="L18" t="n">
-        <v>1998.15</v>
+        <v>175.53</v>
       </c>
       <c r="M18" t="n">
-        <v>-565.5</v>
+        <v>48.31</v>
       </c>
     </row>
     <row r="19">
@@ -1281,25 +1281,25 @@
         <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>700</v>
+        <v>17000</v>
       </c>
       <c r="H19" t="n">
-        <v>-260</v>
+        <v>-110</v>
       </c>
       <c r="I19" t="n">
-        <v>90</v>
+        <v>350</v>
       </c>
       <c r="J19" t="n">
         <v>0.5</v>
       </c>
       <c r="K19" t="n">
-        <v>114.4856760702529</v>
+        <v>385.4162169477469</v>
       </c>
       <c r="L19" t="n">
-        <v>324.32</v>
+        <v>11639.39</v>
       </c>
       <c r="M19" t="n">
-        <v>92.84</v>
+        <v>-47.68</v>
       </c>
     </row>
     <row r="20">
@@ -1326,25 +1326,25 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>11000.24611493832</v>
+        <v>900.0221924430583</v>
       </c>
       <c r="H20" t="n">
-        <v>-100.0005642535693</v>
+        <v>-999</v>
       </c>
       <c r="I20" t="n">
-        <v>250.9018119795456</v>
+        <v>843.6011140694814</v>
       </c>
       <c r="J20" t="n">
         <v>0.5</v>
       </c>
       <c r="K20" t="n">
-        <v>295.6007445329244</v>
+        <v>836.0851639320924</v>
       </c>
       <c r="L20" t="n">
-        <v>6377.43</v>
+        <v>761.87</v>
       </c>
       <c r="M20" t="n">
-        <v>-19.37</v>
+        <v>-875.25</v>
       </c>
     </row>
     <row r="21">
@@ -1371,25 +1371,25 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>1016.427042744672</v>
+        <v>16000.19594032481</v>
       </c>
       <c r="H21" t="n">
-        <v>-350.0000195817747</v>
+        <v>-250.0000086349739</v>
       </c>
       <c r="I21" t="n">
-        <v>500.2842266235539</v>
+        <v>650.2972178461241</v>
       </c>
       <c r="J21" t="n">
         <v>0.5</v>
       </c>
       <c r="K21" t="n">
-        <v>499.0314924731653</v>
+        <v>680.5240193355573</v>
       </c>
       <c r="L21" t="n">
-        <v>805.65</v>
+        <v>13158.92</v>
       </c>
       <c r="M21" t="n">
-        <v>-272.91</v>
+        <v>-190.58</v>
       </c>
     </row>
     <row r="22">
@@ -1416,25 +1416,25 @@
         <v>2</v>
       </c>
       <c r="G22" t="n">
-        <v>6000.695184318414</v>
+        <v>6000.988038215703</v>
       </c>
       <c r="H22" t="n">
-        <v>-250.0000061576394</v>
+        <v>-400.0000329703925</v>
       </c>
       <c r="I22" t="n">
-        <v>450.3520558660788</v>
+        <v>300.901101909499</v>
       </c>
       <c r="J22" t="n">
         <v>0.5</v>
       </c>
       <c r="K22" t="n">
-        <v>423.2358566393677</v>
+        <v>330.4916794875841</v>
       </c>
       <c r="L22" t="n">
-        <v>4711.47</v>
+        <v>3842.57</v>
       </c>
       <c r="M22" t="n">
-        <v>-177.96</v>
+        <v>-228.42</v>
       </c>
     </row>
     <row r="23">
@@ -1461,25 +1461,25 @@
         <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>7000.569707888595</v>
+        <v>1178.725481387519</v>
       </c>
       <c r="H23" t="n">
-        <v>-250.0000067117505</v>
+        <v>-550.0000389416664</v>
       </c>
       <c r="I23" t="n">
-        <v>500.2940864750864</v>
+        <v>149.8089472840586</v>
       </c>
       <c r="J23" t="n">
         <v>0.5</v>
       </c>
       <c r="K23" t="n">
-        <v>528.7866871801347</v>
+        <v>161.9071957960046</v>
       </c>
       <c r="L23" t="n">
-        <v>5442.55</v>
+        <v>545.1900000000001</v>
       </c>
       <c r="M23" t="n">
-        <v>-180.77</v>
+        <v>-149.06</v>
       </c>
     </row>
     <row r="24">
@@ -1506,25 +1506,25 @@
         <v>4</v>
       </c>
       <c r="G24" t="n">
-        <v>934.1355194678936</v>
+        <v>4002.140364645111</v>
       </c>
       <c r="H24" t="n">
-        <v>-250.0000035952838</v>
+        <v>-600.0000130676292</v>
       </c>
       <c r="I24" t="n">
-        <v>153.7076527310146</v>
+        <v>600.3488364403759</v>
       </c>
       <c r="J24" t="n">
         <v>0.5</v>
       </c>
       <c r="K24" t="n">
-        <v>174.8797588600428</v>
+        <v>602.1844988862963</v>
       </c>
       <c r="L24" t="n">
-        <v>355.85</v>
+        <v>3331.69</v>
       </c>
       <c r="M24" t="n">
-        <v>-14.85</v>
+        <v>-500.63</v>
       </c>
     </row>
     <row r="25">
@@ -1551,25 +1551,25 @@
         <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>3004.79069136813</v>
+        <v>11000.65958776293</v>
       </c>
       <c r="H25" t="n">
-        <v>-850.0000098407239</v>
+        <v>-800.0000134318004</v>
       </c>
       <c r="I25" t="n">
-        <v>288.2732712363093</v>
+        <v>301.6512052338647</v>
       </c>
       <c r="J25" t="n">
         <v>0.5</v>
       </c>
       <c r="K25" t="n">
-        <v>302.9006275609877</v>
+        <v>343.4570282107588</v>
       </c>
       <c r="L25" t="n">
-        <v>2027.2</v>
+        <v>6921.26</v>
       </c>
       <c r="M25" t="n">
-        <v>-524.95</v>
+        <v>-476.91</v>
       </c>
     </row>
     <row r="26">
@@ -1596,25 +1596,25 @@
         <v>6</v>
       </c>
       <c r="G26" t="n">
-        <v>793.1152257303916</v>
+        <v>860.1009665743843</v>
       </c>
       <c r="H26" t="n">
-        <v>-150.0000075316569</v>
+        <v>-400.0000169923563</v>
       </c>
       <c r="I26" t="n">
-        <v>250.5675852492012</v>
+        <v>252.0248000632765</v>
       </c>
       <c r="J26" t="n">
         <v>0.5</v>
       </c>
       <c r="K26" t="n">
-        <v>228.9713521405058</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L26" t="n">
-        <v>619.08</v>
+        <v>597.03</v>
       </c>
       <c r="M26" t="n">
-        <v>-63.58</v>
+        <v>-191.6</v>
       </c>
     </row>
     <row r="27">
@@ -1641,25 +1641,25 @@
         <v>7</v>
       </c>
       <c r="G27" t="n">
-        <v>2008.387671907359</v>
+        <v>796.7717756216276</v>
       </c>
       <c r="H27" t="n">
-        <v>-800.00001112285</v>
+        <v>-550.0001844585879</v>
       </c>
       <c r="I27" t="n">
-        <v>284.0777599761669</v>
+        <v>99.97236954527651</v>
       </c>
       <c r="J27" t="n">
         <v>0.5</v>
       </c>
       <c r="K27" t="n">
-        <v>295.6007445329244</v>
+        <v>66.09833589751683</v>
       </c>
       <c r="L27" t="n">
-        <v>1345.29</v>
+        <v>348.41</v>
       </c>
       <c r="M27" t="n">
-        <v>-475.64</v>
+        <v>27.66</v>
       </c>
     </row>
     <row r="28">
@@ -1686,25 +1686,25 @@
         <v>8</v>
       </c>
       <c r="G28" t="n">
-        <v>795.7634281047748</v>
+        <v>16000.16548271839</v>
       </c>
       <c r="H28" t="n">
-        <v>-269.9999930087224</v>
+        <v>-100.0007901915155</v>
       </c>
       <c r="I28" t="n">
-        <v>99.94062908745198</v>
+        <v>251.2453559127833</v>
       </c>
       <c r="J28" t="n">
         <v>0.5</v>
       </c>
       <c r="K28" t="n">
-        <v>114.4856760702529</v>
+        <v>295.6007445329244</v>
       </c>
       <c r="L28" t="n">
-        <v>199.01</v>
+        <v>9131.870000000001</v>
       </c>
       <c r="M28" t="n">
-        <v>120.67</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="29">
@@ -1731,25 +1731,25 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>10019.82426360569</v>
+        <v>866.2883353716604</v>
       </c>
       <c r="H29" t="n">
-        <v>-89.70569086990514</v>
+        <v>-894.4757518393312</v>
       </c>
       <c r="I29" t="n">
-        <v>171.1494795877462</v>
+        <v>750.1077159406559</v>
       </c>
       <c r="J29" t="n">
         <v>0.5</v>
       </c>
       <c r="K29" t="n">
-        <v>219.2233794389425</v>
+        <v>714.9628179040169</v>
       </c>
       <c r="L29" t="n">
-        <v>4347.36</v>
+        <v>751.98</v>
       </c>
       <c r="M29" t="n">
-        <v>36.58</v>
+        <v>-818.53</v>
       </c>
     </row>
     <row r="30">
@@ -1776,25 +1776,25 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>953.5289157604102</v>
+        <v>15020.67354378659</v>
       </c>
       <c r="H30" t="n">
-        <v>-247.0985614126917</v>
+        <v>-240.0654512029123</v>
       </c>
       <c r="I30" t="n">
-        <v>410.0908232346522</v>
+        <v>551.8895836164864</v>
       </c>
       <c r="J30" t="n">
         <v>0.5</v>
       </c>
       <c r="K30" t="n">
-        <v>402.0604809124811</v>
+        <v>591.2014890658488</v>
       </c>
       <c r="L30" t="n">
-        <v>729.96</v>
+        <v>11831.62</v>
       </c>
       <c r="M30" t="n">
-        <v>-174.92</v>
+        <v>-167.79</v>
       </c>
     </row>
     <row r="31">
@@ -1821,25 +1821,25 @@
         <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>5042.846115763668</v>
+        <v>5060.415963640736</v>
       </c>
       <c r="H31" t="n">
-        <v>-239.9741289934778</v>
+        <v>-295.4676751382063</v>
       </c>
       <c r="I31" t="n">
-        <v>355.0518595457356</v>
+        <v>220.5641205185179</v>
       </c>
       <c r="J31" t="n">
         <v>0.5</v>
       </c>
       <c r="K31" t="n">
-        <v>391.0430286998269</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L31" t="n">
-        <v>3420.61</v>
+        <v>2838.29</v>
       </c>
       <c r="M31" t="n">
-        <v>-129.5</v>
+        <v>-94.93000000000001</v>
       </c>
     </row>
     <row r="32">
@@ -1866,25 +1866,25 @@
         <v>3</v>
       </c>
       <c r="G32" t="n">
-        <v>6035.967780342778</v>
+        <v>1273.118328762266</v>
       </c>
       <c r="H32" t="n">
-        <v>-239.7645093774938</v>
+        <v>-454.8460058673284</v>
       </c>
       <c r="I32" t="n">
-        <v>407.569218160852</v>
+        <v>159.6550968654816</v>
       </c>
       <c r="J32" t="n">
         <v>0.5</v>
       </c>
       <c r="K32" t="n">
-        <v>438.4467588778851</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L32" t="n">
-        <v>4375.47</v>
+        <v>654.76</v>
       </c>
       <c r="M32" t="n">
-        <v>-148.24</v>
+        <v>-90.25</v>
       </c>
     </row>
     <row r="33">
@@ -1911,25 +1911,25 @@
         <v>4</v>
       </c>
       <c r="G33" t="n">
-        <v>934.5287930215312</v>
+        <v>3085.797164069763</v>
       </c>
       <c r="H33" t="n">
-        <v>-239.9439386170428</v>
+        <v>-498.1076709922474</v>
       </c>
       <c r="I33" t="n">
-        <v>146.2890460803963</v>
+        <v>504.8426958211736</v>
       </c>
       <c r="J33" t="n">
         <v>0.5</v>
       </c>
       <c r="K33" t="n">
-        <v>147.8003722664622</v>
+        <v>499.0314924731653</v>
       </c>
       <c r="L33" t="n">
-        <v>429.07</v>
+        <v>2536.22</v>
       </c>
       <c r="M33" t="n">
-        <v>-12.84</v>
+        <v>-402.42</v>
       </c>
     </row>
     <row r="34">
@@ -1956,25 +1956,25 @@
         <v>5</v>
       </c>
       <c r="G34" t="n">
-        <v>2120.334010643724</v>
+        <v>10040.22553325315</v>
       </c>
       <c r="H34" t="n">
-        <v>-748.8594242394379</v>
+        <v>-698.3182892952071</v>
       </c>
       <c r="I34" t="n">
-        <v>284.2112679143011</v>
+        <v>219.4913634523047</v>
       </c>
       <c r="J34" t="n">
         <v>0.5</v>
       </c>
       <c r="K34" t="n">
-        <v>280.4314892296821</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L34" t="n">
-        <v>1505.85</v>
+        <v>5332.74</v>
       </c>
       <c r="M34" t="n">
-        <v>-482.17</v>
+        <v>-326.92</v>
       </c>
     </row>
     <row r="35">
@@ -2001,25 +2001,25 @@
         <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>867.9326628634178</v>
+        <v>752.8933374628139</v>
       </c>
       <c r="H35" t="n">
-        <v>-140.8427279988577</v>
+        <v>-353.3290317841626</v>
       </c>
       <c r="I35" t="n">
-        <v>172.3298031798057</v>
+        <v>339.5292055459054</v>
       </c>
       <c r="J35" t="n">
         <v>0.5</v>
       </c>
       <c r="K35" t="n">
-        <v>174.8797588600428</v>
+        <v>349.7595177200857</v>
       </c>
       <c r="L35" t="n">
-        <v>504.74</v>
+        <v>540.1</v>
       </c>
       <c r="M35" t="n">
-        <v>-13.52</v>
+        <v>-189.34</v>
       </c>
     </row>
     <row r="36">
@@ -2046,25 +2046,25 @@
         <v>7</v>
       </c>
       <c r="G36" t="n">
-        <v>1170.369572934555</v>
+        <v>899.2739097867208</v>
       </c>
       <c r="H36" t="n">
-        <v>-698.3270805670745</v>
+        <v>-618.9033674775701</v>
       </c>
       <c r="I36" t="n">
-        <v>281.3259291081103</v>
+        <v>109.0554076898227</v>
       </c>
       <c r="J36" t="n">
         <v>0.5</v>
       </c>
       <c r="K36" t="n">
-        <v>238.320939301339</v>
+        <v>93.4771630765607</v>
       </c>
       <c r="L36" t="n">
-        <v>870.1900000000001</v>
+        <v>308.05</v>
       </c>
       <c r="M36" t="n">
-        <v>-556.22</v>
+        <v>-66.29000000000001</v>
       </c>
     </row>
     <row r="37">
@@ -2091,25 +2091,25 @@
         <v>8</v>
       </c>
       <c r="G37" t="n">
-        <v>888.4677843863684</v>
+        <v>15021.14953425163</v>
       </c>
       <c r="H37" t="n">
-        <v>-280.3324893698352</v>
+        <v>-89.04459075158418</v>
       </c>
       <c r="I37" t="n">
-        <v>109.6234332991881</v>
+        <v>172.724774453376</v>
       </c>
       <c r="J37" t="n">
         <v>0.5</v>
       </c>
       <c r="K37" t="n">
-        <v>132.1966717950337</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L37" t="n">
-        <v>313.06</v>
+        <v>6607.43</v>
       </c>
       <c r="M37" t="n">
-        <v>36.12</v>
+        <v>59.21</v>
       </c>
     </row>
     <row r="38">
@@ -2136,25 +2136,25 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>9068.088507249551</v>
+        <v>845.5491219477017</v>
       </c>
       <c r="H38" t="n">
-        <v>-87.38265579801036</v>
+        <v>-788.5205840465303</v>
       </c>
       <c r="I38" t="n">
-        <v>128.6624508135351</v>
+        <v>645.2068923416589</v>
       </c>
       <c r="J38" t="n">
         <v>0.5</v>
       </c>
       <c r="K38" t="n">
-        <v>198.2950076925505</v>
+        <v>633.9929658716479</v>
       </c>
       <c r="L38" t="n">
-        <v>2721.47</v>
+        <v>698.48</v>
       </c>
       <c r="M38" t="n">
-        <v>88.38</v>
+        <v>-668.22</v>
       </c>
     </row>
     <row r="39">
@@ -2181,25 +2181,25 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>909.6598516727203</v>
+        <v>14043.15063645182</v>
       </c>
       <c r="H39" t="n">
-        <v>-150.4129766062561</v>
+        <v>-230.231337430678</v>
       </c>
       <c r="I39" t="n">
-        <v>325.2903109865437</v>
+        <v>460.8589038118265</v>
       </c>
       <c r="J39" t="n">
         <v>0.5</v>
       </c>
       <c r="K39" t="n">
-        <v>323.8143915920092</v>
+        <v>494.634653528818</v>
       </c>
       <c r="L39" t="n">
-        <v>675.28</v>
+        <v>10787.27</v>
       </c>
       <c r="M39" t="n">
-        <v>-104.72</v>
+        <v>-145.54</v>
       </c>
     </row>
     <row r="40">
@@ -2226,25 +2226,25 @@
         <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>4112.887503526152</v>
+        <v>4160.263104637273</v>
       </c>
       <c r="H40" t="n">
-        <v>-229.8661081454598</v>
+        <v>-200.0186382545248</v>
       </c>
       <c r="I40" t="n">
-        <v>283.1351769500222</v>
+        <v>164.1852919914556</v>
       </c>
       <c r="J40" t="n">
         <v>0.5</v>
       </c>
       <c r="K40" t="n">
-        <v>310.0286763918156</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L40" t="n">
-        <v>2651.07</v>
+        <v>1702.27</v>
       </c>
       <c r="M40" t="n">
-        <v>-103.65</v>
+        <v>-15.79</v>
       </c>
     </row>
     <row r="41">
@@ -2271,25 +2271,25 @@
         <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>5103.339338548314</v>
+        <v>1350.523891647867</v>
       </c>
       <c r="H41" t="n">
-        <v>-229.7773332640361</v>
+        <v>-354.198104793664</v>
       </c>
       <c r="I41" t="n">
-        <v>321.1270759877012</v>
+        <v>169.9432012874786</v>
       </c>
       <c r="J41" t="n">
         <v>0.5</v>
       </c>
       <c r="K41" t="n">
-        <v>337.0367045574487</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L41" t="n">
-        <v>3378.23</v>
+        <v>702.8200000000001</v>
       </c>
       <c r="M41" t="n">
-        <v>-120.37</v>
+        <v>-109.64</v>
       </c>
     </row>
     <row r="42">
@@ -2316,25 +2316,25 @@
         <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>1045.077130470538</v>
+        <v>2222.271474551299</v>
       </c>
       <c r="H42" t="n">
-        <v>-237.2222750013117</v>
+        <v>-398.528047227725</v>
       </c>
       <c r="I42" t="n">
-        <v>254.4156288584925</v>
+        <v>417.9157497755654</v>
       </c>
       <c r="J42" t="n">
         <v>0.5</v>
       </c>
       <c r="K42" t="n">
-        <v>219.2233794389425</v>
+        <v>433.4357742066306</v>
       </c>
       <c r="L42" t="n">
-        <v>742.4</v>
+        <v>1694.69</v>
       </c>
       <c r="M42" t="n">
-        <v>-147.49</v>
+        <v>-286.74</v>
       </c>
     </row>
     <row r="43">
@@ -2361,25 +2361,25 @@
         <v>5</v>
       </c>
       <c r="G43" t="n">
-        <v>1344.16804998633</v>
+        <v>9108.433120175036</v>
       </c>
       <c r="H43" t="n">
-        <v>-650.7693533218935</v>
+        <v>-601.6101057717922</v>
       </c>
       <c r="I43" t="n">
-        <v>279.5493252616245</v>
+        <v>160.2004770424729</v>
       </c>
       <c r="J43" t="n">
         <v>0.5</v>
       </c>
       <c r="K43" t="n">
-        <v>280.4314892296821</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L43" t="n">
-        <v>948.04</v>
+        <v>3715.71</v>
       </c>
       <c r="M43" t="n">
-        <v>-423.12</v>
+        <v>-180.67</v>
       </c>
     </row>
     <row r="44">
@@ -2406,25 +2406,25 @@
         <v>6</v>
       </c>
       <c r="G44" t="n">
-        <v>946.61255177524</v>
+        <v>728.7813788581011</v>
       </c>
       <c r="H44" t="n">
-        <v>-131.5271401200158</v>
+        <v>-260.4814013966051</v>
       </c>
       <c r="I44" t="n">
-        <v>190.2605223021965</v>
+        <v>375.3647127849093</v>
       </c>
       <c r="J44" t="n">
         <v>0.5</v>
       </c>
       <c r="K44" t="n">
-        <v>186.9543261531214</v>
+        <v>362.0354958462345</v>
       </c>
       <c r="L44" t="n">
-        <v>567.14</v>
+        <v>539.11</v>
       </c>
       <c r="M44" t="n">
-        <v>-10.63</v>
+        <v>-176.84</v>
       </c>
     </row>
     <row r="45">
@@ -2451,25 +2451,25 @@
         <v>7</v>
       </c>
       <c r="G45" t="n">
-        <v>517.1803651784227</v>
+        <v>991.9246814264517</v>
       </c>
       <c r="H45" t="n">
-        <v>-599.6858269481017</v>
+        <v>-696.9721475406261</v>
       </c>
       <c r="I45" t="n">
-        <v>277.6808138882571</v>
+        <v>119.5799987664044</v>
       </c>
       <c r="J45" t="n">
         <v>0.5</v>
       </c>
       <c r="K45" t="n">
-        <v>228.9713521405058</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L45" t="n">
-        <v>323.57</v>
+        <v>373.41</v>
       </c>
       <c r="M45" t="n">
-        <v>-390.07</v>
+        <v>-97.76000000000001</v>
       </c>
     </row>
     <row r="46">
@@ -2496,25 +2496,25 @@
         <v>8</v>
       </c>
       <c r="G46" t="n">
-        <v>987.5133176613283</v>
+        <v>14084.73729347649</v>
       </c>
       <c r="H46" t="n">
-        <v>-290.9401813229373</v>
+        <v>-95.19031313627207</v>
       </c>
       <c r="I46" t="n">
-        <v>119.0006345413076</v>
+        <v>131.490722835922</v>
       </c>
       <c r="J46" t="n">
         <v>0.5</v>
       </c>
       <c r="K46" t="n">
-        <v>198.2950076925505</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L46" t="n">
-        <v>346.26</v>
+        <v>4605.03</v>
       </c>
       <c r="M46" t="n">
-        <v>-2.41</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="47">
@@ -2541,25 +2541,25 @@
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>8275.262935590812</v>
+        <v>832.1068285152841</v>
       </c>
       <c r="H47" t="n">
-        <v>-98.90608281167626</v>
+        <v>-683.7427711388443</v>
       </c>
       <c r="I47" t="n">
-        <v>150.0726628380948</v>
+        <v>547.4708696083355</v>
       </c>
       <c r="J47" t="n">
         <v>0.5</v>
       </c>
       <c r="K47" t="n">
-        <v>186.9543261531214</v>
+        <v>553.0183546587466</v>
       </c>
       <c r="L47" t="n">
-        <v>3209.83</v>
+        <v>686.87</v>
       </c>
       <c r="M47" t="n">
-        <v>37.63</v>
+        <v>-583.13</v>
       </c>
     </row>
     <row r="48">
@@ -2586,25 +2586,25 @@
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>889.7899109195167</v>
+        <v>13080.59017273367</v>
       </c>
       <c r="H48" t="n">
-        <v>-62.63608059820302</v>
+        <v>-220.6824156756402</v>
       </c>
       <c r="I48" t="n">
-        <v>251.1701036267572</v>
+        <v>376.2053498226772</v>
       </c>
       <c r="J48" t="n">
         <v>0.5</v>
       </c>
       <c r="K48" t="n">
-        <v>219.2233794389425</v>
+        <v>423.2358566393677</v>
       </c>
       <c r="L48" t="n">
-        <v>610.89</v>
+        <v>8991.549999999999</v>
       </c>
       <c r="M48" t="n">
-        <v>-0.54</v>
+        <v>-117.13</v>
       </c>
     </row>
     <row r="49">
@@ -2631,25 +2631,25 @@
         <v>2</v>
       </c>
       <c r="G49" t="n">
-        <v>3252.35047987053</v>
+        <v>3247.171175517745</v>
       </c>
       <c r="H49" t="n">
-        <v>-220.4818283299811</v>
+        <v>-127.0475353488663</v>
       </c>
       <c r="I49" t="n">
-        <v>214.1966351666642</v>
+        <v>157.2265119677134</v>
       </c>
       <c r="J49" t="n">
         <v>0.5</v>
       </c>
       <c r="K49" t="n">
-        <v>238.320939301339</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L49" t="n">
-        <v>1860.23</v>
+        <v>1535.33</v>
       </c>
       <c r="M49" t="n">
-        <v>-62.09</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="50">
@@ -2676,25 +2676,25 @@
         <v>3</v>
       </c>
       <c r="G50" t="n">
-        <v>4212.61909377913</v>
+        <v>1407.702251016555</v>
       </c>
       <c r="H50" t="n">
-        <v>-220.1900154543873</v>
+        <v>-265.4762656407886</v>
       </c>
       <c r="I50" t="n">
-        <v>245.3897146254757</v>
+        <v>179.9211508190592</v>
       </c>
       <c r="J50" t="n">
         <v>0.5</v>
       </c>
       <c r="K50" t="n">
-        <v>272.5304205830174</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L50" t="n">
-        <v>2558.62</v>
+        <v>657.52</v>
       </c>
       <c r="M50" t="n">
-        <v>-64.16</v>
+        <v>-79.95999999999999</v>
       </c>
     </row>
     <row r="51">
@@ -2721,13 +2721,13 @@
         <v>4</v>
       </c>
       <c r="G51" t="n">
-        <v>1145.496357208988</v>
+        <v>1434.598224096218</v>
       </c>
       <c r="H51" t="n">
-        <v>-236.5186037258011</v>
+        <v>-302.9393382022952</v>
       </c>
       <c r="I51" t="n">
-        <v>369.5862066727457</v>
+        <v>339.6352424664857</v>
       </c>
       <c r="J51" t="n">
         <v>0.5</v>
@@ -2736,10 +2736,10 @@
         <v>355.9504322854629</v>
       </c>
       <c r="L51" t="n">
-        <v>932.13</v>
+        <v>1080.92</v>
       </c>
       <c r="M51" t="n">
-        <v>-199.11</v>
+        <v>-186.32</v>
       </c>
     </row>
     <row r="52">
@@ -2766,25 +2766,25 @@
         <v>5</v>
       </c>
       <c r="G52" t="n">
-        <v>706.0876296532565</v>
+        <v>8210.977206600914</v>
       </c>
       <c r="H52" t="n">
-        <v>-553.6521296825508</v>
+        <v>-512.7998376194972</v>
       </c>
       <c r="I52" t="n">
-        <v>278.1046755440734</v>
+        <v>152.191940156669</v>
       </c>
       <c r="J52" t="n">
         <v>0.5</v>
       </c>
       <c r="K52" t="n">
-        <v>255.9977541431066</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L52" t="n">
-        <v>529.98</v>
+        <v>3318.76</v>
       </c>
       <c r="M52" t="n">
-        <v>-380.63</v>
+        <v>-108.46</v>
       </c>
     </row>
     <row r="53">
@@ -2811,25 +2811,25 @@
         <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>1066.357014912186</v>
+        <v>723.4829306919497</v>
       </c>
       <c r="H53" t="n">
-        <v>-129.8722072943</v>
+        <v>-164.249330184116</v>
       </c>
       <c r="I53" t="n">
-        <v>286.0426223487677</v>
+        <v>361.5799991253523</v>
       </c>
       <c r="J53" t="n">
         <v>0.5</v>
       </c>
       <c r="K53" t="n">
-        <v>295.6007445329244</v>
+        <v>349.7595177200857</v>
       </c>
       <c r="L53" t="n">
-        <v>799.84</v>
+        <v>541.25</v>
       </c>
       <c r="M53" t="n">
-        <v>-62.83</v>
+        <v>-95.75</v>
       </c>
     </row>
     <row r="54">
@@ -2856,25 +2856,25 @@
         <v>7</v>
       </c>
       <c r="G54" t="n">
-        <v>140.4685856305885</v>
+        <v>1090.087404661651</v>
       </c>
       <c r="H54" t="n">
-        <v>-497.2496235670113</v>
+        <v>-657.8839247651139</v>
       </c>
       <c r="I54" t="n">
-        <v>282.4959182897016</v>
+        <v>129.6470086303849</v>
       </c>
       <c r="J54" t="n">
         <v>0.5</v>
       </c>
       <c r="K54" t="n">
-        <v>174.8797588600428</v>
+        <v>161.9071957960046</v>
       </c>
       <c r="L54" t="n">
-        <v>-11.56</v>
+        <v>453.06</v>
       </c>
       <c r="M54" t="n">
-        <v>-249.14</v>
+        <v>-127.26</v>
       </c>
     </row>
     <row r="55">
@@ -2901,25 +2901,25 @@
         <v>8</v>
       </c>
       <c r="G55" t="n">
-        <v>1091.173715816988</v>
+        <v>13262.78901618686</v>
       </c>
       <c r="H55" t="n">
-        <v>-299.4193221051651</v>
+        <v>-107.0350012384318</v>
       </c>
       <c r="I55" t="n">
-        <v>129.4424306133734</v>
+        <v>151.3080446463362</v>
       </c>
       <c r="J55" t="n">
         <v>0.5</v>
       </c>
       <c r="K55" t="n">
-        <v>132.1966717950337</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L55" t="n">
-        <v>468.97</v>
+        <v>5003.71</v>
       </c>
       <c r="M55" t="n">
-        <v>5.84</v>
+        <v>42.44</v>
       </c>
     </row>
     <row r="56">
@@ -2946,25 +2946,25 @@
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>7672.185487234441</v>
+        <v>823.7746054435914</v>
       </c>
       <c r="H56" t="n">
-        <v>-112.0513232451717</v>
+        <v>-583.5119701780576</v>
       </c>
       <c r="I56" t="n">
-        <v>205.1572339388355</v>
+        <v>452.9251247505182</v>
       </c>
       <c r="J56" t="n">
         <v>0.5</v>
       </c>
       <c r="K56" t="n">
-        <v>238.320939301339</v>
+        <v>467.3858153828035</v>
       </c>
       <c r="L56" t="n">
-        <v>4140.24</v>
+        <v>643.62</v>
       </c>
       <c r="M56" t="n">
-        <v>-23.2</v>
+        <v>-416.51</v>
       </c>
     </row>
     <row r="57">
@@ -2991,25 +2991,25 @@
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>903.6528017560341</v>
+        <v>12128.19626930974</v>
       </c>
       <c r="H57" t="n">
-        <v>14.09442104164692</v>
+        <v>-211.5072626418036</v>
       </c>
       <c r="I57" t="n">
-        <v>197.178743454091</v>
+        <v>302.2262210398763</v>
       </c>
       <c r="J57" t="n">
         <v>0.5</v>
       </c>
       <c r="K57" t="n">
-        <v>174.8797588600428</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L57" t="n">
-        <v>577.04</v>
+        <v>8154.54</v>
       </c>
       <c r="M57" t="n">
-        <v>79.48</v>
+        <v>-124.91</v>
       </c>
     </row>
     <row r="58">
@@ -3036,25 +3036,25 @@
         <v>2</v>
       </c>
       <c r="G58" t="n">
-        <v>2451.639729619361</v>
+        <v>2384.81873079132</v>
       </c>
       <c r="H58" t="n">
-        <v>-211.5188557968147</v>
+        <v>-99.56764172941988</v>
       </c>
       <c r="I58" t="n">
-        <v>170.8123143410118</v>
+        <v>237.2796349484561</v>
       </c>
       <c r="J58" t="n">
         <v>0.5</v>
       </c>
       <c r="K58" t="n">
-        <v>174.8797588600428</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L58" t="n">
-        <v>1236.32</v>
+        <v>1445.85</v>
       </c>
       <c r="M58" t="n">
-        <v>-53.41</v>
+        <v>-11.3</v>
       </c>
     </row>
     <row r="59">
@@ -3081,25 +3081,25 @@
         <v>3</v>
       </c>
       <c r="G59" t="n">
-        <v>3379.778180654522</v>
+        <v>1441.590703226053</v>
       </c>
       <c r="H59" t="n">
-        <v>-210.9705804227473</v>
+        <v>-170.7985011689555</v>
       </c>
       <c r="I59" t="n">
-        <v>193.1771767187937</v>
+        <v>189.9512157942106</v>
       </c>
       <c r="J59" t="n">
         <v>0.5</v>
       </c>
       <c r="K59" t="n">
-        <v>219.2233794389425</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L59" t="n">
-        <v>1767.63</v>
+        <v>771.22</v>
       </c>
       <c r="M59" t="n">
-        <v>-12.32</v>
+        <v>-46.7</v>
       </c>
     </row>
     <row r="60">
@@ -3126,25 +3126,25 @@
         <v>4</v>
       </c>
       <c r="G60" t="n">
-        <v>1178.919403638545</v>
+        <v>784.1764014651656</v>
       </c>
       <c r="H60" t="n">
-        <v>-227.5048711783242</v>
+        <v>-213.8743987226921</v>
       </c>
       <c r="I60" t="n">
-        <v>429.2799221375635</v>
+        <v>266.8054258997851</v>
       </c>
       <c r="J60" t="n">
         <v>0.5</v>
       </c>
       <c r="K60" t="n">
-        <v>433.4357742066306</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L60" t="n">
-        <v>916.49</v>
+        <v>543.52</v>
       </c>
       <c r="M60" t="n">
-        <v>-150.57</v>
+        <v>-84.09999999999999</v>
       </c>
     </row>
     <row r="61">
@@ -3171,25 +3171,25 @@
         <v>5</v>
       </c>
       <c r="G61" t="n">
-        <v>305.3579217559828</v>
+        <v>7365.628978141092</v>
       </c>
       <c r="H61" t="n">
-        <v>-458.4223422990248</v>
+        <v>-437.3384923420676</v>
       </c>
       <c r="I61" t="n">
-        <v>277.2730719852731</v>
+        <v>196.3546132446432</v>
       </c>
       <c r="J61" t="n">
         <v>0.5</v>
       </c>
       <c r="K61" t="n">
-        <v>228.9713521405058</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L61" t="n">
-        <v>256.47</v>
+        <v>3505.61</v>
       </c>
       <c r="M61" t="n">
-        <v>-90.81</v>
+        <v>-145.92</v>
       </c>
     </row>
     <row r="62">
@@ -3216,25 +3216,25 @@
         <v>6</v>
       </c>
       <c r="G62" t="n">
-        <v>1167.892093084745</v>
+        <v>730.0806779229506</v>
       </c>
       <c r="H62" t="n">
-        <v>-131.024156688997</v>
+        <v>-67.83386747945734</v>
       </c>
       <c r="I62" t="n">
-        <v>384.6150950665786</v>
+        <v>323.974163527421</v>
       </c>
       <c r="J62" t="n">
         <v>0.5</v>
       </c>
       <c r="K62" t="n">
-        <v>373.9086523062428</v>
+        <v>330.4916794875841</v>
       </c>
       <c r="L62" t="n">
-        <v>918.1900000000001</v>
+        <v>408.85</v>
       </c>
       <c r="M62" t="n">
-        <v>-80.11</v>
+        <v>17.73</v>
       </c>
     </row>
     <row r="63">
@@ -3261,25 +3261,25 @@
         <v>7</v>
       </c>
       <c r="G63" t="n">
-        <v>227.8853739932531</v>
+        <v>1175.958614839077</v>
       </c>
       <c r="H63" t="n">
-        <v>-403.2675097024474</v>
+        <v>-574.9670053424455</v>
       </c>
       <c r="I63" t="n">
-        <v>290.4456456590701</v>
+        <v>136.6952894672236</v>
       </c>
       <c r="J63" t="n">
         <v>0.5</v>
       </c>
       <c r="K63" t="n">
-        <v>255.9977541431066</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L63" t="n">
-        <v>-64.76000000000001</v>
+        <v>401.6</v>
       </c>
       <c r="M63" t="n">
-        <v>-10.88</v>
+        <v>-142.85</v>
       </c>
     </row>
     <row r="64">
@@ -3306,25 +3306,25 @@
         <v>8</v>
       </c>
       <c r="G64" t="n">
-        <v>1206.78778446288</v>
+        <v>12529.89784759866</v>
       </c>
       <c r="H64" t="n">
-        <v>-305.6298899316962</v>
+        <v>-118.5062473860355</v>
       </c>
       <c r="I64" t="n">
-        <v>139.0602363101074</v>
+        <v>218.9482827942651</v>
       </c>
       <c r="J64" t="n">
         <v>0.5</v>
       </c>
       <c r="K64" t="n">
-        <v>174.8797588600428</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L64" t="n">
-        <v>492.6</v>
+        <v>6880.38</v>
       </c>
       <c r="M64" t="n">
-        <v>-13.25</v>
+        <v>-32.95</v>
       </c>
     </row>
     <row r="65">
@@ -3351,25 +3351,25 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>7000.619463702522</v>
+        <v>818.7489539459112</v>
       </c>
       <c r="H65" t="n">
-        <v>-122.3748775955414</v>
+        <v>-486.3406136600415</v>
       </c>
       <c r="I65" t="n">
-        <v>286.8093496478072</v>
+        <v>365.6313459358116</v>
       </c>
       <c r="J65" t="n">
         <v>0.5</v>
       </c>
       <c r="K65" t="n">
-        <v>310.0286763918156</v>
+        <v>355.9504322854629</v>
       </c>
       <c r="L65" t="n">
-        <v>4675.35</v>
+        <v>465.57</v>
       </c>
       <c r="M65" t="n">
-        <v>-33.27</v>
+        <v>-308.87</v>
       </c>
     </row>
     <row r="66">
@@ -3396,25 +3396,25 @@
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>985.4325906549896</v>
+        <v>11208.46299759916</v>
       </c>
       <c r="H66" t="n">
-        <v>27.11408007246451</v>
+        <v>-202.9104164836532</v>
       </c>
       <c r="I66" t="n">
-        <v>228.3598330513809</v>
+        <v>238.2564919616397</v>
       </c>
       <c r="J66" t="n">
         <v>0.5</v>
       </c>
       <c r="K66" t="n">
-        <v>219.2233794389425</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L66" t="n">
-        <v>646.5700000000001</v>
+        <v>6991.86</v>
       </c>
       <c r="M66" t="n">
-        <v>61.15</v>
+        <v>-73.22</v>
       </c>
     </row>
     <row r="67">
@@ -3441,25 +3441,25 @@
         <v>2</v>
       </c>
       <c r="G67" t="n">
-        <v>1730.279533356723</v>
+        <v>1658.189936353333</v>
       </c>
       <c r="H67" t="n">
-        <v>-204.0508608304035</v>
+        <v>-106.4775954631906</v>
       </c>
       <c r="I67" t="n">
-        <v>176.3192932042115</v>
+        <v>329.3060083699041</v>
       </c>
       <c r="J67" t="n">
         <v>0.5</v>
       </c>
       <c r="K67" t="n">
-        <v>174.8797588600428</v>
+        <v>349.7595177200857</v>
       </c>
       <c r="L67" t="n">
-        <v>899.75</v>
+        <v>1189.2</v>
       </c>
       <c r="M67" t="n">
-        <v>-22.34</v>
+        <v>-35.97</v>
       </c>
     </row>
     <row r="68">
@@ -3486,13 +3486,13 @@
         <v>3</v>
       </c>
       <c r="G68" t="n">
-        <v>2565.427984934037</v>
+        <v>1490.268035655453</v>
       </c>
       <c r="H68" t="n">
-        <v>-203.698056087992</v>
+        <v>-85.33500992719787</v>
       </c>
       <c r="I68" t="n">
-        <v>171.0286750744761</v>
+        <v>201.2386351544646</v>
       </c>
       <c r="J68" t="n">
         <v>0.5</v>
@@ -3501,10 +3501,10 @@
         <v>186.9543261531214</v>
       </c>
       <c r="L68" t="n">
-        <v>1237.12</v>
+        <v>950.66</v>
       </c>
       <c r="M68" t="n">
-        <v>20.59</v>
+        <v>-5.48</v>
       </c>
     </row>
     <row r="69">
@@ -3531,25 +3531,25 @@
         <v>4</v>
       </c>
       <c r="G69" t="n">
-        <v>1176.614116731286</v>
+        <v>319.463847046663</v>
       </c>
       <c r="H69" t="n">
-        <v>-216.8601988224301</v>
+        <v>-133.1115528354184</v>
       </c>
       <c r="I69" t="n">
-        <v>433.4279297170322</v>
+        <v>207.5514995966694</v>
       </c>
       <c r="J69" t="n">
         <v>0.5</v>
       </c>
       <c r="K69" t="n">
-        <v>402.0604809124811</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L69" t="n">
-        <v>953.21</v>
+        <v>191.93</v>
       </c>
       <c r="M69" t="n">
-        <v>-178.06</v>
+        <v>-17.51</v>
       </c>
     </row>
     <row r="70">
@@ -3576,25 +3576,25 @@
         <v>5</v>
       </c>
       <c r="G70" t="n">
-        <v>201.9796078230057</v>
+        <v>6491.537042048481</v>
       </c>
       <c r="H70" t="n">
-        <v>-365.3792366197873</v>
+        <v>-375.3696247864177</v>
       </c>
       <c r="I70" t="n">
-        <v>281.2568731550044</v>
+        <v>275.3237063475563</v>
       </c>
       <c r="J70" t="n">
         <v>0.5</v>
       </c>
       <c r="K70" t="n">
-        <v>228.9713521405058</v>
+        <v>302.9006275609877</v>
       </c>
       <c r="L70" t="n">
-        <v>11.44</v>
+        <v>4191.27</v>
       </c>
       <c r="M70" t="n">
-        <v>41.83</v>
+        <v>-189.92</v>
       </c>
     </row>
     <row r="71">
@@ -3621,25 +3621,25 @@
         <v>6</v>
       </c>
       <c r="G71" t="n">
-        <v>1180.045759365336</v>
+        <v>751.1571321010358</v>
       </c>
       <c r="H71" t="n">
-        <v>-123.1199656076542</v>
+        <v>13.30518684700617</v>
       </c>
       <c r="I71" t="n">
-        <v>407.4607313568296</v>
+        <v>265.9975404529526</v>
       </c>
       <c r="J71" t="n">
         <v>0.5</v>
       </c>
       <c r="K71" t="n">
-        <v>385.4162169477469</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L71" t="n">
-        <v>940.12</v>
+        <v>550.63</v>
       </c>
       <c r="M71" t="n">
-        <v>-79.73999999999999</v>
+        <v>43.82</v>
       </c>
     </row>
     <row r="72">
@@ -3666,25 +3666,25 @@
         <v>7</v>
       </c>
       <c r="G72" t="n">
-        <v>822.0646371462506</v>
+        <v>1247.235472100062</v>
       </c>
       <c r="H72" t="n">
-        <v>-320.6730861682562</v>
+        <v>-470.9187130292537</v>
       </c>
       <c r="I72" t="n">
-        <v>303.0735635241507</v>
+        <v>143.7400183170452</v>
       </c>
       <c r="J72" t="n">
         <v>0.5</v>
       </c>
       <c r="K72" t="n">
-        <v>295.6007445329244</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L72" t="n">
-        <v>600.9400000000001</v>
+        <v>513.8</v>
       </c>
       <c r="M72" t="n">
-        <v>-202.9</v>
+        <v>-81.93000000000001</v>
       </c>
     </row>
     <row r="73">
@@ -3711,25 +3711,25 @@
         <v>8</v>
       </c>
       <c r="G73" t="n">
-        <v>1298.052235869256</v>
+        <v>11773.75896009435</v>
       </c>
       <c r="H73" t="n">
-        <v>-312.1511062265459</v>
+        <v>-129.6902847560621</v>
       </c>
       <c r="I73" t="n">
-        <v>150.7531717170063</v>
+        <v>293.7241276398042</v>
       </c>
       <c r="J73" t="n">
         <v>0.5</v>
       </c>
       <c r="K73" t="n">
-        <v>174.8797588600428</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L73" t="n">
-        <v>556.5599999999999</v>
+        <v>7387.63</v>
       </c>
       <c r="M73" t="n">
-        <v>-11.15</v>
+        <v>-45.99</v>
       </c>
     </row>
     <row r="74">
@@ -3756,25 +3756,25 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>6123.625509057643</v>
+        <v>816.7640532917177</v>
       </c>
       <c r="H74" t="n">
-        <v>-126.0944492380486</v>
+        <v>-396.8970305161423</v>
       </c>
       <c r="I74" t="n">
-        <v>349.5151828160974</v>
+        <v>286.3293059780282</v>
       </c>
       <c r="J74" t="n">
         <v>0.5</v>
       </c>
       <c r="K74" t="n">
-        <v>337.0367045574487</v>
+        <v>316.996482935824</v>
       </c>
       <c r="L74" t="n">
-        <v>4783.54</v>
+        <v>577.66</v>
       </c>
       <c r="M74" t="n">
-        <v>-78.58</v>
+        <v>-176.49</v>
       </c>
     </row>
     <row r="75">
@@ -3801,25 +3801,25 @@
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>1056.352336803373</v>
+        <v>10315.92996728079</v>
       </c>
       <c r="H75" t="n">
-        <v>-8.404530874247055</v>
+        <v>-193.8058669567699</v>
       </c>
       <c r="I75" t="n">
-        <v>276.7577221947439</v>
+        <v>198.3088171349527</v>
       </c>
       <c r="J75" t="n">
         <v>0.5</v>
       </c>
       <c r="K75" t="n">
-        <v>272.5304205830174</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L75" t="n">
-        <v>737.1900000000001</v>
+        <v>4919.24</v>
       </c>
       <c r="M75" t="n">
-        <v>33.03</v>
+        <v>-15.02</v>
       </c>
     </row>
     <row r="76">
@@ -3846,25 +3846,25 @@
         <v>2</v>
       </c>
       <c r="G76" t="n">
-        <v>1191.202044964468</v>
+        <v>886.7159940299642</v>
       </c>
       <c r="H76" t="n">
-        <v>-196.9607106649994</v>
+        <v>-113.8476671679928</v>
       </c>
       <c r="I76" t="n">
-        <v>247.7666170094034</v>
+        <v>409.5604024279473</v>
       </c>
       <c r="J76" t="n">
         <v>0.5</v>
       </c>
       <c r="K76" t="n">
-        <v>219.2233794389425</v>
+        <v>379.7060313951988</v>
       </c>
       <c r="L76" t="n">
-        <v>802.0599999999999</v>
+        <v>727.86</v>
       </c>
       <c r="M76" t="n">
-        <v>-69.84</v>
+        <v>-77.08</v>
       </c>
     </row>
     <row r="77">
@@ -3891,25 +3891,25 @@
         <v>3</v>
       </c>
       <c r="G77" t="n">
-        <v>1810.830902282436</v>
+        <v>1477.954285552303</v>
       </c>
       <c r="H77" t="n">
-        <v>-201.6804912776164</v>
+        <v>-16.75663061960482</v>
       </c>
       <c r="I77" t="n">
-        <v>205.3279592461455</v>
+        <v>212.9416116612993</v>
       </c>
       <c r="J77" t="n">
         <v>0.5</v>
       </c>
       <c r="K77" t="n">
-        <v>209.0212909830231</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L77" t="n">
-        <v>1070.07</v>
+        <v>890.99</v>
       </c>
       <c r="M77" t="n">
-        <v>-101.7</v>
+        <v>47.79</v>
       </c>
     </row>
     <row r="78">
@@ -3936,25 +3936,25 @@
         <v>4</v>
       </c>
       <c r="G78" t="n">
-        <v>1157.087928525535</v>
+        <v>242.7852657437815</v>
       </c>
       <c r="H78" t="n">
-        <v>-206.8354477858767</v>
+        <v>-68.70923324113743</v>
       </c>
       <c r="I78" t="n">
-        <v>386.1110652443137</v>
+        <v>180.2735873558817</v>
       </c>
       <c r="J78" t="n">
         <v>0.5</v>
       </c>
       <c r="K78" t="n">
-        <v>373.9086523062428</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L78" t="n">
-        <v>922.42</v>
+        <v>25.5</v>
       </c>
       <c r="M78" t="n">
-        <v>-144.02</v>
+        <v>78.15000000000001</v>
       </c>
     </row>
     <row r="79">
@@ -3981,25 +3981,25 @@
         <v>5</v>
       </c>
       <c r="G79" t="n">
-        <v>664.0510017859363</v>
+        <v>5620.831425210465</v>
       </c>
       <c r="H79" t="n">
-        <v>-303.3117675304483</v>
+        <v>-307.567542712957</v>
       </c>
       <c r="I79" t="n">
-        <v>293.4660350111529</v>
+        <v>332.4949242359778</v>
       </c>
       <c r="J79" t="n">
         <v>0.5</v>
       </c>
       <c r="K79" t="n">
-        <v>272.5304205830174</v>
+        <v>362.0354958462345</v>
       </c>
       <c r="L79" t="n">
-        <v>506.52</v>
+        <v>3925.8</v>
       </c>
       <c r="M79" t="n">
-        <v>-178.19</v>
+        <v>-181.45</v>
       </c>
     </row>
     <row r="80">
@@ -4026,25 +4026,25 @@
         <v>6</v>
       </c>
       <c r="G80" t="n">
-        <v>1144.261490794253</v>
+        <v>806.618904117484</v>
       </c>
       <c r="H80" t="n">
-        <v>-113.4110737886242</v>
+        <v>14.04905820615261</v>
       </c>
       <c r="I80" t="n">
-        <v>374.1917192802561</v>
+        <v>201.2551056857135</v>
       </c>
       <c r="J80" t="n">
         <v>0.5</v>
       </c>
       <c r="K80" t="n">
-        <v>385.4162169477469</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L80" t="n">
-        <v>840.28</v>
+        <v>484.51</v>
       </c>
       <c r="M80" t="n">
-        <v>-55.38</v>
+        <v>55.75</v>
       </c>
     </row>
     <row r="81">
@@ -4071,25 +4071,25 @@
         <v>7</v>
       </c>
       <c r="G81" t="n">
-        <v>2093.924947109726</v>
+        <v>1320.316003645021</v>
       </c>
       <c r="H81" t="n">
-        <v>-291.6612975366837</v>
+        <v>-359.3403078337209</v>
       </c>
       <c r="I81" t="n">
-        <v>313.0542339472323</v>
+        <v>150.9190682696963</v>
       </c>
       <c r="J81" t="n">
         <v>0.5</v>
       </c>
       <c r="K81" t="n">
-        <v>323.8143915920092</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L81" t="n">
-        <v>1459.57</v>
+        <v>603.48</v>
       </c>
       <c r="M81" t="n">
-        <v>-182.96</v>
+        <v>-56.08</v>
       </c>
     </row>
     <row r="82">
@@ -4116,25 +4116,25 @@
         <v>8</v>
       </c>
       <c r="G82" t="n">
-        <v>1398.764877488584</v>
+        <v>10845.18061696473</v>
       </c>
       <c r="H82" t="n">
-        <v>-316.6279087795085</v>
+        <v>-132.2103748407683</v>
       </c>
       <c r="I82" t="n">
-        <v>162.3006745578103</v>
+        <v>337.5811162484855</v>
       </c>
       <c r="J82" t="n">
         <v>0.5</v>
       </c>
       <c r="K82" t="n">
-        <v>186.9543261531214</v>
+        <v>368.0199590525625</v>
       </c>
       <c r="L82" t="n">
-        <v>678.84</v>
+        <v>7699.2</v>
       </c>
       <c r="M82" t="n">
-        <v>-23.47</v>
+        <v>-59.77</v>
       </c>
     </row>
     <row r="83">
@@ -4161,25 +4161,25 @@
         <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>5187.495717361434</v>
+        <v>821.0094095015329</v>
       </c>
       <c r="H83" t="n">
-        <v>-126.8932192704564</v>
+        <v>-314.4737157130965</v>
       </c>
       <c r="I83" t="n">
-        <v>348.2463326247159</v>
+        <v>230.1167372677171</v>
       </c>
       <c r="J83" t="n">
         <v>0.5</v>
       </c>
       <c r="K83" t="n">
-        <v>391.0430286998269</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L83" t="n">
-        <v>3549.03</v>
+        <v>288.38</v>
       </c>
       <c r="M83" t="n">
-        <v>-50.21</v>
+        <v>-60.42</v>
       </c>
     </row>
     <row r="84">
@@ -4206,25 +4206,25 @@
         <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>1112.265957171275</v>
+        <v>9424.366600550547</v>
       </c>
       <c r="H84" t="n">
-        <v>-59.74920766254394</v>
+        <v>-186.6688346955743</v>
       </c>
       <c r="I84" t="n">
-        <v>322.6802012782422</v>
+        <v>176.7816210304546</v>
       </c>
       <c r="J84" t="n">
         <v>0.5</v>
       </c>
       <c r="K84" t="n">
-        <v>330.4916794875841</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L84" t="n">
-        <v>803.85</v>
+        <v>4464.87</v>
       </c>
       <c r="M84" t="n">
-        <v>-13.9</v>
+        <v>-13.99</v>
       </c>
     </row>
     <row r="85">
@@ -4251,25 +4251,25 @@
         <v>2</v>
       </c>
       <c r="G85" t="n">
-        <v>765.2940145861428</v>
+        <v>251.9262162017246</v>
       </c>
       <c r="H85" t="n">
-        <v>-193.6616490756933</v>
+        <v>-91.6158237965068</v>
       </c>
       <c r="I85" t="n">
-        <v>371.5785155021347</v>
+        <v>353.2153082206629</v>
       </c>
       <c r="J85" t="n">
         <v>0.5</v>
       </c>
       <c r="K85" t="n">
-        <v>323.8143915920092</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L85" t="n">
-        <v>557.3200000000001</v>
+        <v>-13.27</v>
       </c>
       <c r="M85" t="n">
-        <v>-121.03</v>
+        <v>87.08</v>
       </c>
     </row>
     <row r="86">
@@ -4296,25 +4296,25 @@
         <v>3</v>
       </c>
       <c r="G86" t="n">
-        <v>1303.118867031556</v>
+        <v>1367.609086963569</v>
       </c>
       <c r="H86" t="n">
-        <v>-204.9859767609692</v>
+        <v>-10.40511787042215</v>
       </c>
       <c r="I86" t="n">
-        <v>270.3599147440521</v>
+        <v>225.3103954119474</v>
       </c>
       <c r="J86" t="n">
         <v>0.5</v>
       </c>
       <c r="K86" t="n">
-        <v>272.5304205830174</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L86" t="n">
-        <v>906.1900000000001</v>
+        <v>881.1799999999999</v>
       </c>
       <c r="M86" t="n">
-        <v>-100.51</v>
+        <v>32.43</v>
       </c>
     </row>
     <row r="87">
@@ -4341,25 +4341,25 @@
         <v>4</v>
       </c>
       <c r="G87" t="n">
-        <v>1123.320400126065</v>
+        <v>843.173184300985</v>
       </c>
       <c r="H87" t="n">
-        <v>-196.1323994168356</v>
+        <v>-42.35362889704457</v>
       </c>
       <c r="I87" t="n">
-        <v>334.1110084459722</v>
+        <v>262.2646910600982</v>
       </c>
       <c r="J87" t="n">
         <v>0.5</v>
       </c>
       <c r="K87" t="n">
-        <v>343.4570282107588</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L87" t="n">
-        <v>841.09</v>
+        <v>585.86</v>
       </c>
       <c r="M87" t="n">
-        <v>-102.17</v>
+        <v>-4.8</v>
       </c>
     </row>
     <row r="88">
@@ -4386,25 +4386,25 @@
         <v>5</v>
       </c>
       <c r="G88" t="n">
-        <v>1525.025314986135</v>
+        <v>4698.991489091691</v>
       </c>
       <c r="H88" t="n">
-        <v>-297.9652380745541</v>
+        <v>-231.5252617430352</v>
       </c>
       <c r="I88" t="n">
-        <v>305.5502336972414</v>
+        <v>336.9590265698472</v>
       </c>
       <c r="J88" t="n">
         <v>0.5</v>
       </c>
       <c r="K88" t="n">
-        <v>288.1159665134826</v>
+        <v>355.9504322854629</v>
       </c>
       <c r="L88" t="n">
-        <v>1099.32</v>
+        <v>3310.05</v>
       </c>
       <c r="M88" t="n">
-        <v>-186.67</v>
+        <v>-131.8</v>
       </c>
     </row>
     <row r="89">
@@ -4431,25 +4431,25 @@
         <v>6</v>
       </c>
       <c r="G89" t="n">
-        <v>1084.466425801775</v>
+        <v>847.4753349047522</v>
       </c>
       <c r="H89" t="n">
-        <v>-103.1907882741176</v>
+        <v>-20.96975929029902</v>
       </c>
       <c r="I89" t="n">
-        <v>315.4220580756721</v>
+        <v>222.6392387311265</v>
       </c>
       <c r="J89" t="n">
         <v>0.5</v>
       </c>
       <c r="K89" t="n">
-        <v>288.1159665134826</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L89" t="n">
-        <v>730.76</v>
+        <v>512.3</v>
       </c>
       <c r="M89" t="n">
-        <v>-87</v>
+        <v>49.23</v>
       </c>
     </row>
     <row r="90">
@@ -4476,25 +4476,25 @@
         <v>7</v>
       </c>
       <c r="G90" t="n">
-        <v>2530.689042083179</v>
+        <v>1390.090753640867</v>
       </c>
       <c r="H90" t="n">
-        <v>-221.5181348635559</v>
+        <v>-264.6526271373666</v>
       </c>
       <c r="I90" t="n">
-        <v>314.7814355824629</v>
+        <v>158.1147062953137</v>
       </c>
       <c r="J90" t="n">
         <v>0.5</v>
       </c>
       <c r="K90" t="n">
-        <v>343.4570282107588</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L90" t="n">
-        <v>1705.53</v>
+        <v>612.12</v>
       </c>
       <c r="M90" t="n">
-        <v>-116.49</v>
+        <v>-22.75</v>
       </c>
     </row>
     <row r="91">
@@ -4521,25 +4521,25 @@
         <v>8</v>
       </c>
       <c r="G91" t="n">
-        <v>1485.039566469768</v>
+        <v>9884.615649716707</v>
       </c>
       <c r="H91" t="n">
-        <v>-321.1203250320734</v>
+        <v>-131.0861663068135</v>
       </c>
       <c r="I91" t="n">
-        <v>173.6462845105228</v>
+        <v>313.6707438378427</v>
       </c>
       <c r="J91" t="n">
         <v>0.5</v>
       </c>
       <c r="K91" t="n">
-        <v>174.8797588600428</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L91" t="n">
-        <v>749.33</v>
+        <v>6845.78</v>
       </c>
       <c r="M91" t="n">
-        <v>-81.68000000000001</v>
+        <v>-49.65</v>
       </c>
     </row>
     <row r="92">
@@ -4566,25 +4566,25 @@
         <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>4290.077032974634</v>
+        <v>826.4930828588435</v>
       </c>
       <c r="H92" t="n">
-        <v>-121.0656081690849</v>
+        <v>-243.998280895391</v>
       </c>
       <c r="I92" t="n">
-        <v>313.3841357064874</v>
+        <v>186.5681578794358</v>
       </c>
       <c r="J92" t="n">
         <v>0.5</v>
       </c>
       <c r="K92" t="n">
-        <v>337.0367045574487</v>
+        <v>132.1966717950337</v>
       </c>
       <c r="L92" t="n">
-        <v>2836.87</v>
+        <v>458.33</v>
       </c>
       <c r="M92" t="n">
-        <v>-37.24</v>
+        <v>-120.26</v>
       </c>
     </row>
     <row r="93">
@@ -4611,25 +4611,25 @@
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>1128.735927485365</v>
+        <v>8575.481353782689</v>
       </c>
       <c r="H93" t="n">
-        <v>-115.9745722777635</v>
+        <v>-184.1518087039896</v>
       </c>
       <c r="I93" t="n">
-        <v>344.6673342990532</v>
+        <v>178.7833690185174</v>
       </c>
       <c r="J93" t="n">
         <v>0.5</v>
       </c>
       <c r="K93" t="n">
-        <v>343.4570282107588</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L93" t="n">
-        <v>846.21</v>
+        <v>3865.53</v>
       </c>
       <c r="M93" t="n">
-        <v>-57.38</v>
+        <v>23.65</v>
       </c>
     </row>
     <row r="94">
@@ -4656,25 +4656,25 @@
         <v>2</v>
       </c>
       <c r="G94" t="n">
-        <v>515.6835788024292</v>
+        <v>-30.04072426406509</v>
       </c>
       <c r="H94" t="n">
-        <v>-185.3510118303306</v>
+        <v>-25.77923704665935</v>
       </c>
       <c r="I94" t="n">
-        <v>440.6799261922779</v>
+        <v>269.8827281243955</v>
       </c>
       <c r="J94" t="n">
         <v>0.5</v>
       </c>
       <c r="K94" t="n">
-        <v>457.9427042810117</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L94" t="n">
-        <v>354.48</v>
+        <v>-24.9</v>
       </c>
       <c r="M94" t="n">
-        <v>-84.20999999999999</v>
+        <v>42.83</v>
       </c>
     </row>
     <row r="95">
@@ -4701,25 +4701,25 @@
         <v>3</v>
       </c>
       <c r="G95" t="n">
-        <v>935.8520111106213</v>
+        <v>1292.018921704342</v>
       </c>
       <c r="H95" t="n">
-        <v>-197.5360651900623</v>
+        <v>-62.31087824737482</v>
       </c>
       <c r="I95" t="n">
-        <v>327.9796020481474</v>
+        <v>233.4158168795942</v>
       </c>
       <c r="J95" t="n">
         <v>0.5</v>
       </c>
       <c r="K95" t="n">
-        <v>337.0367045574487</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L95" t="n">
-        <v>599.35</v>
+        <v>837.4299999999999</v>
       </c>
       <c r="M95" t="n">
-        <v>-111.01</v>
+        <v>-1.65</v>
       </c>
     </row>
     <row r="96">
@@ -4746,25 +4746,25 @@
         <v>4</v>
       </c>
       <c r="G96" t="n">
-        <v>1081.485784079449</v>
+        <v>1389.740183847462</v>
       </c>
       <c r="H96" t="n">
-        <v>-185.9956770663789</v>
+        <v>-65.2318865221127</v>
       </c>
       <c r="I96" t="n">
-        <v>277.8141438515309</v>
+        <v>332.4624970133045</v>
       </c>
       <c r="J96" t="n">
         <v>0.5</v>
       </c>
       <c r="K96" t="n">
-        <v>255.9977541431066</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L96" t="n">
-        <v>788.88</v>
+        <v>1039.1</v>
       </c>
       <c r="M96" t="n">
-        <v>-108</v>
+        <v>-17.83</v>
       </c>
     </row>
     <row r="97">
@@ -4791,25 +4791,25 @@
         <v>5</v>
       </c>
       <c r="G97" t="n">
-        <v>1954.714755000457</v>
+        <v>3789.688206014015</v>
       </c>
       <c r="H97" t="n">
-        <v>-238.3653748326371</v>
+        <v>-153.7511288858043</v>
       </c>
       <c r="I97" t="n">
-        <v>310.5851496172795</v>
+        <v>280.4378759920298</v>
       </c>
       <c r="J97" t="n">
         <v>0.5</v>
       </c>
       <c r="K97" t="n">
-        <v>310.0286763918156</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L97" t="n">
-        <v>1394.35</v>
+        <v>2590.76</v>
       </c>
       <c r="M97" t="n">
-        <v>-139.33</v>
+        <v>-62.01</v>
       </c>
     </row>
     <row r="98">
@@ -4836,25 +4836,25 @@
         <v>6</v>
       </c>
       <c r="G98" t="n">
-        <v>1029.215914217547</v>
+        <v>897.6241205430479</v>
       </c>
       <c r="H98" t="n">
-        <v>-94.17359212002884</v>
+        <v>-77.97791948380879</v>
       </c>
       <c r="I98" t="n">
-        <v>230.9222477195183</v>
+        <v>253.791505850277</v>
       </c>
       <c r="J98" t="n">
         <v>0.5</v>
       </c>
       <c r="K98" t="n">
-        <v>219.2233794389425</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L98" t="n">
-        <v>700.5599999999999</v>
+        <v>391.67</v>
       </c>
       <c r="M98" t="n">
-        <v>-18.15</v>
+        <v>13.52</v>
       </c>
     </row>
     <row r="99">
@@ -4881,25 +4881,25 @@
         <v>7</v>
       </c>
       <c r="G99" t="n">
-        <v>2221.310456089379</v>
+        <v>1450.067170507529</v>
       </c>
       <c r="H99" t="n">
-        <v>-150.8521210825751</v>
+        <v>-183.3673764041169</v>
       </c>
       <c r="I99" t="n">
-        <v>310.9399389338864</v>
+        <v>166.4951427877066</v>
       </c>
       <c r="J99" t="n">
         <v>0.5</v>
       </c>
       <c r="K99" t="n">
-        <v>310.0286763918156</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L99" t="n">
-        <v>1545.58</v>
+        <v>666.95</v>
       </c>
       <c r="M99" t="n">
-        <v>-69.52</v>
+        <v>-15.68</v>
       </c>
     </row>
     <row r="100">
@@ -4926,25 +4926,25 @@
         <v>8</v>
       </c>
       <c r="G100" t="n">
-        <v>1542.774716318924</v>
+        <v>8910.642062467716</v>
       </c>
       <c r="H100" t="n">
-        <v>-322.3979342740296</v>
+        <v>-126.5533634414246</v>
       </c>
       <c r="I100" t="n">
-        <v>186.1954048850868</v>
+        <v>252.0964037627788</v>
       </c>
       <c r="J100" t="n">
         <v>0.5</v>
       </c>
       <c r="K100" t="n">
-        <v>219.2233794389425</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L100" t="n">
-        <v>798.99</v>
+        <v>5335.98</v>
       </c>
       <c r="M100" t="n">
-        <v>-91.43000000000001</v>
+        <v>-26.28</v>
       </c>
     </row>
   </sheetData>
@@ -5025,7 +5025,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -5041,36 +5041,36 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G2" t="n">
-        <v>1029.215914217547</v>
+        <v>1390.090753640867</v>
       </c>
       <c r="H2" t="n">
-        <v>-94.17359212002884</v>
+        <v>-264.6526271373666</v>
       </c>
       <c r="I2" t="n">
-        <v>230.9222477195183</v>
+        <v>158.1147062953137</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>219.2233794389425</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L2" t="n">
-        <v>700.5599999999999</v>
+        <v>612.12</v>
       </c>
       <c r="M2" t="n">
-        <v>-18.15</v>
+        <v>-22.75</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -5086,36 +5086,36 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G3" t="n">
-        <v>1398.764877488584</v>
+        <v>1450.067170507529</v>
       </c>
       <c r="H3" t="n">
-        <v>-316.6279087795085</v>
+        <v>-183.3673764041169</v>
       </c>
       <c r="I3" t="n">
-        <v>162.3006745578103</v>
+        <v>166.4951427877066</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>186.9543261531214</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L3" t="n">
-        <v>678.84</v>
+        <v>666.95</v>
       </c>
       <c r="M3" t="n">
-        <v>-23.47</v>
+        <v>-15.68</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -5131,31 +5131,31 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>1112.265957171275</v>
+        <v>1389.740183847462</v>
       </c>
       <c r="H4" t="n">
-        <v>-59.74920766254394</v>
+        <v>-65.2318865221127</v>
       </c>
       <c r="I4" t="n">
-        <v>322.6802012782422</v>
+        <v>332.4624970133045</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>330.4916794875841</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L4" t="n">
-        <v>803.85</v>
+        <v>1039.1</v>
       </c>
       <c r="M4" t="n">
-        <v>-13.9</v>
+        <v>-17.83</v>
       </c>
     </row>
   </sheetData>
@@ -5268,31 +5268,31 @@
         <v>-21.42555</v>
       </c>
       <c r="G2" t="n">
-        <v>238</v>
+        <v>219</v>
       </c>
       <c r="H2" t="n">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="I2" t="n">
-        <v>1180</v>
+        <v>1409</v>
       </c>
       <c r="J2" t="n">
-        <v>193</v>
+        <v>34</v>
       </c>
       <c r="K2" t="n">
-        <v>-156</v>
+        <v>-171</v>
       </c>
       <c r="L2" t="n">
-        <v>193</v>
+        <v>34</v>
       </c>
       <c r="M2" t="n">
-        <v>-17.52</v>
+        <v>-28.04</v>
       </c>
       <c r="N2" t="n">
-        <v>38.43745211570078</v>
+        <v>48.47473758575618</v>
       </c>
       <c r="O2" t="n">
-        <v>86.34012257756068</v>
+        <v>87.47658776433622</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: improved sidebar and progress bar
</commit_message>
<xml_diff>
--- a/test_alldata.xlsx
+++ b/test_alldata.xlsx
@@ -516,25 +516,25 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="H2" t="n">
-        <v>-850</v>
+        <v>-400</v>
       </c>
       <c r="I2" t="n">
-        <v>850</v>
+        <v>350</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>198.2950076925505</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L2" t="n">
-        <v>10563.78</v>
+        <v>756.45</v>
       </c>
       <c r="M2" t="n">
-        <v>12.66</v>
+        <v>-278.73</v>
       </c>
     </row>
     <row r="3">
@@ -561,25 +561,25 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>18000</v>
+        <v>19000</v>
       </c>
       <c r="H3" t="n">
-        <v>-250</v>
+        <v>-500</v>
       </c>
       <c r="I3" t="n">
-        <v>850</v>
+        <v>700</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>856.7323510961411</v>
+        <v>741.9519802932271</v>
       </c>
       <c r="L3" t="n">
-        <v>15821.55</v>
+        <v>15726.82</v>
       </c>
       <c r="M3" t="n">
-        <v>-219.23</v>
+        <v>-400.35</v>
       </c>
     </row>
     <row r="4">
@@ -606,25 +606,25 @@
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>8000</v>
+        <v>18000</v>
       </c>
       <c r="H4" t="n">
-        <v>-400</v>
+        <v>-300</v>
       </c>
       <c r="I4" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>541.0381969548956</v>
+        <v>854.1787467540389</v>
       </c>
       <c r="L4" t="n">
-        <v>6040.45</v>
+        <v>14858.2</v>
       </c>
       <c r="M4" t="n">
-        <v>-274.63</v>
+        <v>-230.76</v>
       </c>
     </row>
     <row r="5">
@@ -654,7 +654,7 @@
         <v>1200</v>
       </c>
       <c r="H5" t="n">
-        <v>-550</v>
+        <v>-50</v>
       </c>
       <c r="I5" t="n">
         <v>150</v>
@@ -666,10 +666,10 @@
         <v>174.8797588600428</v>
       </c>
       <c r="L5" t="n">
-        <v>547.12</v>
+        <v>558.0700000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>-159.89</v>
+        <v>109.74</v>
       </c>
     </row>
     <row r="6">
@@ -696,25 +696,25 @@
         <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>6000</v>
+        <v>1300</v>
       </c>
       <c r="H6" t="n">
-        <v>-600</v>
+        <v>-100</v>
       </c>
       <c r="I6" t="n">
-        <v>800</v>
+        <v>450</v>
       </c>
       <c r="J6" t="n">
         <v>0.5</v>
       </c>
       <c r="K6" t="n">
-        <v>809.5359789800231</v>
+        <v>443.4011167993866</v>
       </c>
       <c r="L6" t="n">
-        <v>5264.37</v>
+        <v>1017.09</v>
       </c>
       <c r="M6" t="n">
-        <v>-527.37</v>
+        <v>-63.46</v>
       </c>
     </row>
     <row r="7">
@@ -744,22 +744,22 @@
         <v>13000</v>
       </c>
       <c r="H7" t="n">
-        <v>-800</v>
+        <v>-850</v>
       </c>
       <c r="I7" t="n">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="J7" t="n">
         <v>0.5</v>
       </c>
       <c r="K7" t="n">
-        <v>549.0540142654876</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L7" t="n">
-        <v>9855.559999999999</v>
+        <v>5342.96</v>
       </c>
       <c r="M7" t="n">
-        <v>-578.12</v>
+        <v>-249.76</v>
       </c>
     </row>
     <row r="8">
@@ -786,25 +786,25 @@
         <v>6</v>
       </c>
       <c r="G8" t="n">
-        <v>1000</v>
+        <v>8000</v>
       </c>
       <c r="H8" t="n">
-        <v>-400</v>
+        <v>-250</v>
       </c>
       <c r="I8" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="J8" t="n">
         <v>0.5</v>
       </c>
       <c r="K8" t="n">
-        <v>428.3661755480705</v>
+        <v>391.0430286998269</v>
       </c>
       <c r="L8" t="n">
-        <v>814.77</v>
+        <v>5391.19</v>
       </c>
       <c r="M8" t="n">
-        <v>-324.13</v>
+        <v>-113.72</v>
       </c>
     </row>
     <row r="9">
@@ -831,25 +831,25 @@
         <v>7</v>
       </c>
       <c r="G9" t="n">
-        <v>800</v>
+        <v>1200</v>
       </c>
       <c r="H9" t="n">
         <v>-550</v>
       </c>
       <c r="I9" t="n">
-        <v>100</v>
+        <v>850</v>
       </c>
       <c r="J9" t="n">
         <v>0.5</v>
       </c>
       <c r="K9" t="n">
-        <v>93.4771630765607</v>
+        <v>809.5359789800231</v>
       </c>
       <c r="L9" t="n">
-        <v>367.62</v>
+        <v>1072.69</v>
       </c>
       <c r="M9" t="n">
-        <v>-63.75</v>
+        <v>-510.7</v>
       </c>
     </row>
     <row r="10">
@@ -876,25 +876,25 @@
         <v>8</v>
       </c>
       <c r="G10" t="n">
-        <v>18000</v>
+        <v>11000</v>
       </c>
       <c r="H10" t="n">
-        <v>-100</v>
+        <v>-800</v>
       </c>
       <c r="I10" t="n">
-        <v>450</v>
+        <v>550</v>
       </c>
       <c r="J10" t="n">
         <v>0.5</v>
       </c>
       <c r="K10" t="n">
-        <v>494.634653528818</v>
+        <v>580.0105435665924</v>
       </c>
       <c r="L10" t="n">
-        <v>13313.79</v>
+        <v>8833.74</v>
       </c>
       <c r="M10" t="n">
-        <v>-37.27</v>
+        <v>-631.64</v>
       </c>
     </row>
     <row r="11">
@@ -921,25 +921,25 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="H11" t="n">
-        <v>-950</v>
+        <v>-500</v>
       </c>
       <c r="I11" t="n">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="J11" t="n">
         <v>0.5</v>
       </c>
       <c r="K11" t="n">
-        <v>739.0018613323109</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L11" t="n">
-        <v>875.11</v>
+        <v>650.6</v>
       </c>
       <c r="M11" t="n">
-        <v>-833.9400000000001</v>
+        <v>-330.6</v>
       </c>
     </row>
     <row r="12">
@@ -966,25 +966,25 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="H12" t="n">
-        <v>-260</v>
+        <v>-600</v>
       </c>
       <c r="I12" t="n">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="J12" t="n">
         <v>0.5</v>
       </c>
       <c r="K12" t="n">
-        <v>795.9293632107308</v>
+        <v>633.9929658716479</v>
       </c>
       <c r="L12" t="n">
-        <v>13855.29</v>
+        <v>14332.23</v>
       </c>
       <c r="M12" t="n">
-        <v>-202.72</v>
+        <v>-462.26</v>
       </c>
     </row>
     <row r="13">
@@ -1011,25 +1011,25 @@
         <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>7000</v>
+        <v>17000</v>
       </c>
       <c r="H13" t="n">
-        <v>-500</v>
+        <v>-310</v>
       </c>
       <c r="I13" t="n">
-        <v>400</v>
+        <v>700</v>
       </c>
       <c r="J13" t="n">
         <v>0.5</v>
       </c>
       <c r="K13" t="n">
-        <v>428.3661755480705</v>
+        <v>744.890415476976</v>
       </c>
       <c r="L13" t="n">
-        <v>5210.1</v>
+        <v>13960.14</v>
       </c>
       <c r="M13" t="n">
-        <v>-346.08</v>
+        <v>-236.84</v>
       </c>
     </row>
     <row r="14">
@@ -1059,7 +1059,7 @@
         <v>1100</v>
       </c>
       <c r="H14" t="n">
-        <v>-650</v>
+        <v>-60</v>
       </c>
       <c r="I14" t="n">
         <v>140</v>
@@ -1068,13 +1068,13 @@
         <v>0.5</v>
       </c>
       <c r="K14" t="n">
-        <v>186.9543261531214</v>
+        <v>161.9071957960046</v>
       </c>
       <c r="L14" t="n">
-        <v>471.27</v>
+        <v>540.63</v>
       </c>
       <c r="M14" t="n">
-        <v>-122.49</v>
+        <v>27.19</v>
       </c>
     </row>
     <row r="15">
@@ -1101,25 +1101,25 @@
         <v>4</v>
       </c>
       <c r="G15" t="n">
-        <v>5000</v>
+        <v>1200</v>
       </c>
       <c r="H15" t="n">
-        <v>-700</v>
+        <v>-110</v>
       </c>
       <c r="I15" t="n">
-        <v>700</v>
+        <v>350</v>
       </c>
       <c r="J15" t="n">
         <v>0.5</v>
       </c>
       <c r="K15" t="n">
-        <v>736.039918105125</v>
+        <v>355.9504322854629</v>
       </c>
       <c r="L15" t="n">
-        <v>4142.37</v>
+        <v>885.73</v>
       </c>
       <c r="M15" t="n">
-        <v>-571.37</v>
+        <v>-44.48</v>
       </c>
     </row>
     <row r="16">
@@ -1149,22 +1149,22 @@
         <v>12000</v>
       </c>
       <c r="H16" t="n">
-        <v>-900</v>
+        <v>-950</v>
       </c>
       <c r="I16" t="n">
-        <v>400</v>
+        <v>140</v>
       </c>
       <c r="J16" t="n">
         <v>0.5</v>
       </c>
       <c r="K16" t="n">
-        <v>438.4467588778851</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L16" t="n">
-        <v>8578.07</v>
+        <v>4046.58</v>
       </c>
       <c r="M16" t="n">
-        <v>-615.6</v>
+        <v>-229.91</v>
       </c>
     </row>
     <row r="17">
@@ -1191,25 +1191,25 @@
         <v>6</v>
       </c>
       <c r="G17" t="n">
-        <v>900</v>
+        <v>7000</v>
       </c>
       <c r="H17" t="n">
-        <v>-500</v>
+        <v>-260</v>
       </c>
       <c r="I17" t="n">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="J17" t="n">
         <v>0.5</v>
       </c>
       <c r="K17" t="n">
-        <v>114.4856760702529</v>
+        <v>280.4314892296821</v>
       </c>
       <c r="L17" t="n">
-        <v>1915.19</v>
+        <v>4083.45</v>
       </c>
       <c r="M17" t="n">
-        <v>-39.01</v>
+        <v>-87.95</v>
       </c>
     </row>
     <row r="18">
@@ -1236,25 +1236,25 @@
         <v>7</v>
       </c>
       <c r="G18" t="n">
-        <v>700</v>
+        <v>1100</v>
       </c>
       <c r="H18" t="n">
         <v>-650</v>
       </c>
       <c r="I18" t="n">
-        <v>90</v>
+        <v>750</v>
       </c>
       <c r="J18" t="n">
         <v>0.5</v>
       </c>
       <c r="K18" t="n">
-        <v>114.4856760702529</v>
+        <v>654.3401415359249</v>
       </c>
       <c r="L18" t="n">
-        <v>175.53</v>
+        <v>943.54</v>
       </c>
       <c r="M18" t="n">
-        <v>48.31</v>
+        <v>-578.98</v>
       </c>
     </row>
     <row r="19">
@@ -1281,25 +1281,25 @@
         <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>17000</v>
+        <v>10000</v>
       </c>
       <c r="H19" t="n">
-        <v>-110</v>
+        <v>-900</v>
       </c>
       <c r="I19" t="n">
-        <v>350</v>
+        <v>450</v>
       </c>
       <c r="J19" t="n">
         <v>0.5</v>
       </c>
       <c r="K19" t="n">
-        <v>385.4162169477469</v>
+        <v>485.7215873880137</v>
       </c>
       <c r="L19" t="n">
-        <v>11639.39</v>
+        <v>7440.16</v>
       </c>
       <c r="M19" t="n">
-        <v>-47.68</v>
+        <v>-647.49</v>
       </c>
     </row>
     <row r="20">
@@ -1326,25 +1326,25 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>900.0221924430583</v>
+        <v>883.9912992430009</v>
       </c>
       <c r="H20" t="n">
-        <v>-999</v>
+        <v>-400.0000194994221</v>
       </c>
       <c r="I20" t="n">
-        <v>843.6011140694814</v>
+        <v>160.0699829847259</v>
       </c>
       <c r="J20" t="n">
         <v>0.5</v>
       </c>
       <c r="K20" t="n">
-        <v>836.0851639320924</v>
+        <v>161.9071957960046</v>
       </c>
       <c r="L20" t="n">
-        <v>761.87</v>
+        <v>355.48</v>
       </c>
       <c r="M20" t="n">
-        <v>-875.25</v>
+        <v>-138.94</v>
       </c>
     </row>
     <row r="21">
@@ -1371,25 +1371,25 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>16000.19594032481</v>
+        <v>17000.24737488236</v>
       </c>
       <c r="H21" t="n">
-        <v>-250.0000086349739</v>
+        <v>-500.0000293376613</v>
       </c>
       <c r="I21" t="n">
-        <v>650.2972178461241</v>
+        <v>500.5753965319273</v>
       </c>
       <c r="J21" t="n">
         <v>0.5</v>
       </c>
       <c r="K21" t="n">
-        <v>680.5240193355573</v>
+        <v>536.9854193139544</v>
       </c>
       <c r="L21" t="n">
-        <v>13158.92</v>
+        <v>12861.18</v>
       </c>
       <c r="M21" t="n">
-        <v>-190.58</v>
+        <v>-353.86</v>
       </c>
     </row>
     <row r="22">
@@ -1416,25 +1416,25 @@
         <v>2</v>
       </c>
       <c r="G22" t="n">
-        <v>6000.988038215703</v>
+        <v>16000.2180010993</v>
       </c>
       <c r="H22" t="n">
-        <v>-400.0000329703925</v>
+        <v>-300.0000075183198</v>
       </c>
       <c r="I22" t="n">
-        <v>300.901101909499</v>
+        <v>600.2924370625308</v>
       </c>
       <c r="J22" t="n">
         <v>0.5</v>
       </c>
       <c r="K22" t="n">
-        <v>330.4916794875841</v>
+        <v>644.2468865272003</v>
       </c>
       <c r="L22" t="n">
-        <v>3842.57</v>
+        <v>12730.73</v>
       </c>
       <c r="M22" t="n">
-        <v>-228.42</v>
+        <v>-214.62</v>
       </c>
     </row>
     <row r="23">
@@ -1461,25 +1461,25 @@
         <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>1178.725481387519</v>
+        <v>1177.593200874206</v>
       </c>
       <c r="H23" t="n">
-        <v>-550.0000389416664</v>
+        <v>-69.99999587824597</v>
       </c>
       <c r="I23" t="n">
-        <v>149.8089472840586</v>
+        <v>149.818278981262</v>
       </c>
       <c r="J23" t="n">
         <v>0.5</v>
       </c>
       <c r="K23" t="n">
-        <v>161.9071957960046</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L23" t="n">
-        <v>545.1900000000001</v>
+        <v>526.9299999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>-149.06</v>
+        <v>-2.35</v>
       </c>
     </row>
     <row r="24">
@@ -1506,25 +1506,25 @@
         <v>4</v>
       </c>
       <c r="G24" t="n">
-        <v>4002.140364645111</v>
+        <v>1104.526796348649</v>
       </c>
       <c r="H24" t="n">
-        <v>-600.0000130676292</v>
+        <v>-100.0000175501522</v>
       </c>
       <c r="I24" t="n">
-        <v>600.3488364403759</v>
+        <v>250.340905115194</v>
       </c>
       <c r="J24" t="n">
         <v>0.5</v>
       </c>
       <c r="K24" t="n">
-        <v>602.1844988862963</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L24" t="n">
-        <v>3331.69</v>
+        <v>722.45</v>
       </c>
       <c r="M24" t="n">
-        <v>-500.63</v>
+        <v>-9.039999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -1551,25 +1551,25 @@
         <v>5</v>
       </c>
       <c r="G25" t="n">
-        <v>11000.65958776293</v>
+        <v>11001.12898541345</v>
       </c>
       <c r="H25" t="n">
-        <v>-800.0000134318004</v>
+        <v>-850.0000349714724</v>
       </c>
       <c r="I25" t="n">
-        <v>301.6512052338647</v>
+        <v>149.2902419083157</v>
       </c>
       <c r="J25" t="n">
         <v>0.5</v>
       </c>
       <c r="K25" t="n">
-        <v>343.4570282107588</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L25" t="n">
-        <v>6921.26</v>
+        <v>4552.27</v>
       </c>
       <c r="M25" t="n">
-        <v>-476.91</v>
+        <v>-229.2</v>
       </c>
     </row>
     <row r="26">
@@ -1596,25 +1596,25 @@
         <v>6</v>
       </c>
       <c r="G26" t="n">
-        <v>860.1009665743843</v>
+        <v>6000.711207396811</v>
       </c>
       <c r="H26" t="n">
-        <v>-400.0000169923563</v>
+        <v>-250.0000137583971</v>
       </c>
       <c r="I26" t="n">
-        <v>252.0248000632765</v>
+        <v>152.6979909331236</v>
       </c>
       <c r="J26" t="n">
         <v>0.5</v>
       </c>
       <c r="K26" t="n">
-        <v>247.317326764409</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L26" t="n">
-        <v>597.03</v>
+        <v>2405.82</v>
       </c>
       <c r="M26" t="n">
-        <v>-191.6</v>
+        <v>-30.15</v>
       </c>
     </row>
     <row r="27">
@@ -1641,25 +1641,25 @@
         <v>7</v>
       </c>
       <c r="G27" t="n">
-        <v>796.7717756216276</v>
+        <v>1020.586429564732</v>
       </c>
       <c r="H27" t="n">
-        <v>-550.0001844585879</v>
+        <v>-550.0000110912778</v>
       </c>
       <c r="I27" t="n">
-        <v>99.97236954527651</v>
+        <v>650.277188031244</v>
       </c>
       <c r="J27" t="n">
         <v>0.5</v>
       </c>
       <c r="K27" t="n">
-        <v>66.09833589751683</v>
+        <v>630.5379376106623</v>
       </c>
       <c r="L27" t="n">
-        <v>348.41</v>
+        <v>870.02</v>
       </c>
       <c r="M27" t="n">
-        <v>27.66</v>
+        <v>-469.41</v>
       </c>
     </row>
     <row r="28">
@@ -1686,25 +1686,25 @@
         <v>8</v>
       </c>
       <c r="G28" t="n">
-        <v>16000.16548271839</v>
+        <v>9000.86151225546</v>
       </c>
       <c r="H28" t="n">
-        <v>-100.0007901915155</v>
+        <v>-800.0000115190761</v>
       </c>
       <c r="I28" t="n">
-        <v>251.2453559127833</v>
+        <v>351.3737803359644</v>
       </c>
       <c r="J28" t="n">
         <v>0.5</v>
       </c>
       <c r="K28" t="n">
-        <v>295.6007445329244</v>
+        <v>402.0604809124811</v>
       </c>
       <c r="L28" t="n">
-        <v>9131.870000000001</v>
+        <v>6570.72</v>
       </c>
       <c r="M28" t="n">
-        <v>6.4</v>
+        <v>-553.86</v>
       </c>
     </row>
     <row r="29">
@@ -1731,25 +1731,25 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>866.2883353716604</v>
+        <v>908.327203522347</v>
       </c>
       <c r="H29" t="n">
-        <v>-894.4757518393312</v>
+        <v>-297.8535568927633</v>
       </c>
       <c r="I29" t="n">
-        <v>750.1077159406559</v>
+        <v>208.816787859742</v>
       </c>
       <c r="J29" t="n">
         <v>0.5</v>
       </c>
       <c r="K29" t="n">
-        <v>714.9628179040169</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L29" t="n">
-        <v>751.98</v>
+        <v>609.59</v>
       </c>
       <c r="M29" t="n">
-        <v>-818.53</v>
+        <v>-156.36</v>
       </c>
     </row>
     <row r="30">
@@ -1776,25 +1776,25 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>15020.67354378659</v>
+        <v>16027.97206201873</v>
       </c>
       <c r="H30" t="n">
-        <v>-240.0654512029123</v>
+        <v>-396.7009358451684</v>
       </c>
       <c r="I30" t="n">
-        <v>551.8895836164864</v>
+        <v>408.9303243615153</v>
       </c>
       <c r="J30" t="n">
         <v>0.5</v>
       </c>
       <c r="K30" t="n">
-        <v>591.2014890658488</v>
+        <v>453.1473605746647</v>
       </c>
       <c r="L30" t="n">
-        <v>11831.62</v>
+        <v>11615.56</v>
       </c>
       <c r="M30" t="n">
-        <v>-167.79</v>
+        <v>-263.25</v>
       </c>
     </row>
     <row r="31">
@@ -1821,25 +1821,25 @@
         <v>2</v>
       </c>
       <c r="G31" t="n">
-        <v>5060.415963640736</v>
+        <v>15011.56362837459</v>
       </c>
       <c r="H31" t="n">
-        <v>-295.4676751382063</v>
+        <v>-289.8776748589506</v>
       </c>
       <c r="I31" t="n">
-        <v>220.5641205185179</v>
+        <v>505.7685708438686</v>
       </c>
       <c r="J31" t="n">
         <v>0.5</v>
       </c>
       <c r="K31" t="n">
-        <v>255.9977541431066</v>
+        <v>553.0183546587466</v>
       </c>
       <c r="L31" t="n">
-        <v>2838.29</v>
+        <v>11171.7</v>
       </c>
       <c r="M31" t="n">
-        <v>-94.93000000000001</v>
+        <v>-207.89</v>
       </c>
     </row>
     <row r="32">
@@ -1866,25 +1866,25 @@
         <v>3</v>
       </c>
       <c r="G32" t="n">
-        <v>1273.118328762266</v>
+        <v>1271.728488650264</v>
       </c>
       <c r="H32" t="n">
-        <v>-454.8460058673284</v>
+        <v>-78.24601540368199</v>
       </c>
       <c r="I32" t="n">
-        <v>159.6550968654816</v>
+        <v>160.6367485098576</v>
       </c>
       <c r="J32" t="n">
         <v>0.5</v>
       </c>
       <c r="K32" t="n">
-        <v>198.2950076925505</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L32" t="n">
-        <v>654.76</v>
+        <v>575.73</v>
       </c>
       <c r="M32" t="n">
-        <v>-90.25</v>
+        <v>34.34</v>
       </c>
     </row>
     <row r="33">
@@ -1911,25 +1911,25 @@
         <v>4</v>
       </c>
       <c r="G33" t="n">
-        <v>3085.797164069763</v>
+        <v>1017.860587302342</v>
       </c>
       <c r="H33" t="n">
-        <v>-498.1076709922474</v>
+        <v>-90.80118200640453</v>
       </c>
       <c r="I33" t="n">
-        <v>504.8426958211736</v>
+        <v>164.1525405226318</v>
       </c>
       <c r="J33" t="n">
         <v>0.5</v>
       </c>
       <c r="K33" t="n">
-        <v>499.0314924731653</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L33" t="n">
-        <v>2536.22</v>
+        <v>493.44</v>
       </c>
       <c r="M33" t="n">
-        <v>-402.42</v>
+        <v>16.44</v>
       </c>
     </row>
     <row r="34">
@@ -1956,25 +1956,25 @@
         <v>5</v>
       </c>
       <c r="G34" t="n">
-        <v>10040.22553325315</v>
+        <v>10070.26635717995</v>
       </c>
       <c r="H34" t="n">
-        <v>-698.3182892952071</v>
+        <v>-750.1436188053829</v>
       </c>
       <c r="I34" t="n">
-        <v>219.4913634523047</v>
+        <v>158.826545126614</v>
       </c>
       <c r="J34" t="n">
         <v>0.5</v>
       </c>
       <c r="K34" t="n">
-        <v>247.317326764409</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L34" t="n">
-        <v>5332.74</v>
+        <v>3833.83</v>
       </c>
       <c r="M34" t="n">
-        <v>-326.92</v>
+        <v>-153.46</v>
       </c>
     </row>
     <row r="35">
@@ -2001,25 +2001,25 @@
         <v>6</v>
       </c>
       <c r="G35" t="n">
-        <v>752.8933374628139</v>
+        <v>5040.658736941074</v>
       </c>
       <c r="H35" t="n">
-        <v>-353.3290317841626</v>
+        <v>-240.3871550538341</v>
       </c>
       <c r="I35" t="n">
-        <v>339.5292055459054</v>
+        <v>121.7892249198237</v>
       </c>
       <c r="J35" t="n">
         <v>0.5</v>
       </c>
       <c r="K35" t="n">
-        <v>349.7595177200857</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L35" t="n">
-        <v>540.1</v>
+        <v>1554.01</v>
       </c>
       <c r="M35" t="n">
-        <v>-189.34</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="36">
@@ -2046,25 +2046,25 @@
         <v>7</v>
       </c>
       <c r="G36" t="n">
-        <v>899.2739097867208</v>
+        <v>958.9241404145301</v>
       </c>
       <c r="H36" t="n">
-        <v>-618.9033674775701</v>
+        <v>-448.0028631844229</v>
       </c>
       <c r="I36" t="n">
-        <v>109.0554076898227</v>
+        <v>562.0720256271778</v>
       </c>
       <c r="J36" t="n">
         <v>0.5</v>
       </c>
       <c r="K36" t="n">
-        <v>93.4771630765607</v>
+        <v>568.5993850006796</v>
       </c>
       <c r="L36" t="n">
-        <v>308.05</v>
+        <v>791.42</v>
       </c>
       <c r="M36" t="n">
-        <v>-66.29000000000001</v>
+        <v>-342.8</v>
       </c>
     </row>
     <row r="37">
@@ -2091,25 +2091,25 @@
         <v>8</v>
       </c>
       <c r="G37" t="n">
-        <v>15021.14953425163</v>
+        <v>8047.539625237621</v>
       </c>
       <c r="H37" t="n">
-        <v>-89.04459075158418</v>
+        <v>-698.9173207259678</v>
       </c>
       <c r="I37" t="n">
-        <v>172.724774453376</v>
+        <v>263.3892063069378</v>
       </c>
       <c r="J37" t="n">
         <v>0.5</v>
       </c>
       <c r="K37" t="n">
-        <v>219.2233794389425</v>
+        <v>295.6007445329244</v>
       </c>
       <c r="L37" t="n">
-        <v>6607.43</v>
+        <v>5137.52</v>
       </c>
       <c r="M37" t="n">
-        <v>59.21</v>
+        <v>-404.37</v>
       </c>
     </row>
     <row r="38">
@@ -2136,25 +2136,25 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>845.5491219477017</v>
+        <v>1010.176953087521</v>
       </c>
       <c r="H38" t="n">
-        <v>-788.5205840465303</v>
+        <v>-215.4657636112456</v>
       </c>
       <c r="I38" t="n">
-        <v>645.2068923416589</v>
+        <v>315.2148742463816</v>
       </c>
       <c r="J38" t="n">
         <v>0.5</v>
       </c>
       <c r="K38" t="n">
-        <v>633.9929658716479</v>
+        <v>295.6007445329244</v>
       </c>
       <c r="L38" t="n">
-        <v>698.48</v>
+        <v>747.35</v>
       </c>
       <c r="M38" t="n">
-        <v>-668.22</v>
+        <v>-144.95</v>
       </c>
     </row>
     <row r="39">
@@ -2181,25 +2181,25 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>14043.15063645182</v>
+        <v>15054.20205510001</v>
       </c>
       <c r="H39" t="n">
-        <v>-230.231337430678</v>
+        <v>-300.409043801938</v>
       </c>
       <c r="I39" t="n">
-        <v>460.8589038118265</v>
+        <v>323.8091765463003</v>
       </c>
       <c r="J39" t="n">
         <v>0.5</v>
       </c>
       <c r="K39" t="n">
-        <v>494.634653528818</v>
+        <v>362.0354958462345</v>
       </c>
       <c r="L39" t="n">
-        <v>10787.27</v>
+        <v>10148.92</v>
       </c>
       <c r="M39" t="n">
-        <v>-145.54</v>
+        <v>-150.03</v>
       </c>
     </row>
     <row r="40">
@@ -2226,25 +2226,25 @@
         <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>4160.263104637273</v>
+        <v>14035.09428077944</v>
       </c>
       <c r="H40" t="n">
-        <v>-200.0186382545248</v>
+        <v>-279.9693111287669</v>
       </c>
       <c r="I40" t="n">
-        <v>164.1852919914556</v>
+        <v>416.9836918690202</v>
       </c>
       <c r="J40" t="n">
         <v>0.5</v>
       </c>
       <c r="K40" t="n">
-        <v>209.0212909830231</v>
+        <v>457.9427042810117</v>
       </c>
       <c r="L40" t="n">
-        <v>1702.27</v>
+        <v>10233.2</v>
       </c>
       <c r="M40" t="n">
-        <v>-15.79</v>
+        <v>-171.85</v>
       </c>
     </row>
     <row r="41">
@@ -2271,25 +2271,25 @@
         <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>1350.523891647867</v>
+        <v>1378.444743324646</v>
       </c>
       <c r="H41" t="n">
-        <v>-354.198104793664</v>
+        <v>-84.75320775219322</v>
       </c>
       <c r="I41" t="n">
-        <v>169.9432012874786</v>
+        <v>171.4883948743638</v>
       </c>
       <c r="J41" t="n">
         <v>0.5</v>
       </c>
       <c r="K41" t="n">
-        <v>186.9543261531214</v>
+        <v>161.9071957960046</v>
       </c>
       <c r="L41" t="n">
-        <v>702.8200000000001</v>
+        <v>745.0599999999999</v>
       </c>
       <c r="M41" t="n">
-        <v>-109.64</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="42">
@@ -2316,25 +2316,25 @@
         <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>2222.271474551299</v>
+        <v>988.1251157022266</v>
       </c>
       <c r="H42" t="n">
-        <v>-398.528047227725</v>
+        <v>-93.28179062426983</v>
       </c>
       <c r="I42" t="n">
-        <v>417.9157497755654</v>
+        <v>152.6028653793934</v>
       </c>
       <c r="J42" t="n">
         <v>0.5</v>
       </c>
       <c r="K42" t="n">
-        <v>433.4357742066306</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L42" t="n">
-        <v>1694.69</v>
+        <v>418.71</v>
       </c>
       <c r="M42" t="n">
-        <v>-286.74</v>
+        <v>57.27</v>
       </c>
     </row>
     <row r="43">
@@ -2361,25 +2361,25 @@
         <v>5</v>
       </c>
       <c r="G43" t="n">
-        <v>9108.433120175036</v>
+        <v>9085.139528441141</v>
       </c>
       <c r="H43" t="n">
-        <v>-601.6101057717922</v>
+        <v>-651.1673986962879</v>
       </c>
       <c r="I43" t="n">
-        <v>160.2004770424729</v>
+        <v>168.700371589819</v>
       </c>
       <c r="J43" t="n">
         <v>0.5</v>
       </c>
       <c r="K43" t="n">
-        <v>209.0212909830231</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L43" t="n">
-        <v>3715.71</v>
+        <v>4325.92</v>
       </c>
       <c r="M43" t="n">
-        <v>-180.67</v>
+        <v>-218.72</v>
       </c>
     </row>
     <row r="44">
@@ -2406,25 +2406,25 @@
         <v>6</v>
       </c>
       <c r="G44" t="n">
-        <v>728.7813788581011</v>
+        <v>4150.941282512392</v>
       </c>
       <c r="H44" t="n">
-        <v>-260.4814013966051</v>
+        <v>-235.0751045506096</v>
       </c>
       <c r="I44" t="n">
-        <v>375.3647127849093</v>
+        <v>207.1048912951469</v>
       </c>
       <c r="J44" t="n">
         <v>0.5</v>
       </c>
       <c r="K44" t="n">
-        <v>362.0354958462345</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L44" t="n">
-        <v>539.11</v>
+        <v>2426.39</v>
       </c>
       <c r="M44" t="n">
-        <v>-176.84</v>
+        <v>-85.12</v>
       </c>
     </row>
     <row r="45">
@@ -2451,25 +2451,25 @@
         <v>7</v>
       </c>
       <c r="G45" t="n">
-        <v>991.9246814264517</v>
+        <v>907.7152543364526</v>
       </c>
       <c r="H45" t="n">
-        <v>-696.9721475406261</v>
+        <v>-350.3214130887135</v>
       </c>
       <c r="I45" t="n">
-        <v>119.5799987664044</v>
+        <v>470.6356024477872</v>
       </c>
       <c r="J45" t="n">
         <v>0.5</v>
       </c>
       <c r="K45" t="n">
-        <v>186.9543261531214</v>
+        <v>443.4011167993866</v>
       </c>
       <c r="L45" t="n">
-        <v>373.41</v>
+        <v>727.1799999999999</v>
       </c>
       <c r="M45" t="n">
-        <v>-97.76000000000001</v>
+        <v>-279.99</v>
       </c>
     </row>
     <row r="46">
@@ -2496,25 +2496,25 @@
         <v>8</v>
       </c>
       <c r="G46" t="n">
-        <v>14084.73729347649</v>
+        <v>7105.042995641218</v>
       </c>
       <c r="H46" t="n">
-        <v>-95.19031313627207</v>
+        <v>-600.8502653922587</v>
       </c>
       <c r="I46" t="n">
-        <v>131.490722835922</v>
+        <v>189.3940133883631</v>
       </c>
       <c r="J46" t="n">
         <v>0.5</v>
       </c>
       <c r="K46" t="n">
-        <v>186.9543261531214</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L46" t="n">
-        <v>4605.03</v>
+        <v>3225.32</v>
       </c>
       <c r="M46" t="n">
-        <v>43.9</v>
+        <v>-198.47</v>
       </c>
     </row>
     <row r="47">
@@ -2541,25 +2541,25 @@
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>832.1068285152841</v>
+        <v>1068.811513090334</v>
       </c>
       <c r="H47" t="n">
-        <v>-683.7427711388443</v>
+        <v>-128.7319760545768</v>
       </c>
       <c r="I47" t="n">
-        <v>547.4708696083355</v>
+        <v>417.0908266753535</v>
       </c>
       <c r="J47" t="n">
         <v>0.5</v>
       </c>
       <c r="K47" t="n">
-        <v>553.0183546587466</v>
+        <v>407.4575073795997</v>
       </c>
       <c r="L47" t="n">
-        <v>686.87</v>
+        <v>817.0599999999999</v>
       </c>
       <c r="M47" t="n">
-        <v>-583.13</v>
+        <v>-85.23</v>
       </c>
     </row>
     <row r="48">
@@ -2586,25 +2586,25 @@
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>13080.59017273367</v>
+        <v>14077.48620897812</v>
       </c>
       <c r="H48" t="n">
-        <v>-220.6824156756402</v>
+        <v>-212.0107753670498</v>
       </c>
       <c r="I48" t="n">
-        <v>376.2053498226772</v>
+        <v>248.163019541582</v>
       </c>
       <c r="J48" t="n">
         <v>0.5</v>
       </c>
       <c r="K48" t="n">
-        <v>423.2358566393677</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L48" t="n">
-        <v>8991.549999999999</v>
+        <v>8111.46</v>
       </c>
       <c r="M48" t="n">
-        <v>-117.13</v>
+        <v>-37</v>
       </c>
     </row>
     <row r="49">
@@ -2631,25 +2631,25 @@
         <v>2</v>
       </c>
       <c r="G49" t="n">
-        <v>3247.171175517745</v>
+        <v>13087.86982769902</v>
       </c>
       <c r="H49" t="n">
-        <v>-127.0475353488663</v>
+        <v>-269.9783357915607</v>
       </c>
       <c r="I49" t="n">
-        <v>157.2265119677134</v>
+        <v>335.9367127306308</v>
       </c>
       <c r="J49" t="n">
         <v>0.5</v>
       </c>
       <c r="K49" t="n">
-        <v>198.2950076925505</v>
+        <v>368.0199590525625</v>
       </c>
       <c r="L49" t="n">
-        <v>1535.33</v>
+        <v>8861.42</v>
       </c>
       <c r="M49" t="n">
-        <v>7.22</v>
+        <v>-134.76</v>
       </c>
     </row>
     <row r="50">
@@ -2676,25 +2676,25 @@
         <v>3</v>
       </c>
       <c r="G50" t="n">
-        <v>1407.702251016555</v>
+        <v>1458.003604795252</v>
       </c>
       <c r="H50" t="n">
-        <v>-265.4762656407886</v>
+        <v>-93.76836417218166</v>
       </c>
       <c r="I50" t="n">
-        <v>179.9211508190592</v>
+        <v>180.7374817572443</v>
       </c>
       <c r="J50" t="n">
         <v>0.5</v>
       </c>
       <c r="K50" t="n">
-        <v>174.8797588600428</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L50" t="n">
-        <v>657.52</v>
+        <v>807.54</v>
       </c>
       <c r="M50" t="n">
-        <v>-79.95999999999999</v>
+        <v>34.61</v>
       </c>
     </row>
     <row r="51">
@@ -2721,25 +2721,25 @@
         <v>4</v>
       </c>
       <c r="G51" t="n">
-        <v>1434.598224096218</v>
+        <v>1045.791700644014</v>
       </c>
       <c r="H51" t="n">
-        <v>-302.9393382022952</v>
+        <v>-100.7964975435617</v>
       </c>
       <c r="I51" t="n">
-        <v>339.6352424664857</v>
+        <v>197.6528747556653</v>
       </c>
       <c r="J51" t="n">
         <v>0.5</v>
       </c>
       <c r="K51" t="n">
-        <v>355.9504322854629</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L51" t="n">
-        <v>1080.92</v>
+        <v>662.96</v>
       </c>
       <c r="M51" t="n">
-        <v>-186.32</v>
+        <v>-2.36</v>
       </c>
     </row>
     <row r="52">
@@ -2766,25 +2766,25 @@
         <v>5</v>
       </c>
       <c r="G52" t="n">
-        <v>8210.977206600914</v>
+        <v>8105.779581899331</v>
       </c>
       <c r="H52" t="n">
-        <v>-512.7998376194972</v>
+        <v>-562.5172861300368</v>
       </c>
       <c r="I52" t="n">
-        <v>152.191940156669</v>
+        <v>177.5699924234619</v>
       </c>
       <c r="J52" t="n">
         <v>0.5</v>
       </c>
       <c r="K52" t="n">
-        <v>198.2950076925505</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L52" t="n">
-        <v>3318.76</v>
+        <v>3665.2</v>
       </c>
       <c r="M52" t="n">
-        <v>-108.46</v>
+        <v>-166.22</v>
       </c>
     </row>
     <row r="53">
@@ -2811,25 +2811,25 @@
         <v>6</v>
       </c>
       <c r="G53" t="n">
-        <v>723.4829306919497</v>
+        <v>3488.75398840527</v>
       </c>
       <c r="H53" t="n">
-        <v>-164.249330184116</v>
+        <v>-238.8636432301214</v>
       </c>
       <c r="I53" t="n">
-        <v>361.5799991253523</v>
+        <v>313.2688475832693</v>
       </c>
       <c r="J53" t="n">
         <v>0.5</v>
       </c>
       <c r="K53" t="n">
-        <v>349.7595177200857</v>
+        <v>310.0286763918156</v>
       </c>
       <c r="L53" t="n">
-        <v>541.25</v>
+        <v>2467.58</v>
       </c>
       <c r="M53" t="n">
-        <v>-95.75</v>
+        <v>-129.91</v>
       </c>
     </row>
     <row r="54">
@@ -2856,25 +2856,25 @@
         <v>7</v>
       </c>
       <c r="G54" t="n">
-        <v>1090.087404661651</v>
+        <v>871.7543762291754</v>
       </c>
       <c r="H54" t="n">
-        <v>-657.8839247651139</v>
+        <v>-258.9242934775276</v>
       </c>
       <c r="I54" t="n">
-        <v>129.6470086303849</v>
+        <v>379.0238768439938</v>
       </c>
       <c r="J54" t="n">
         <v>0.5</v>
       </c>
       <c r="K54" t="n">
-        <v>161.9071957960046</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L54" t="n">
-        <v>453.06</v>
+        <v>577.51</v>
       </c>
       <c r="M54" t="n">
-        <v>-127.26</v>
+        <v>-171.21</v>
       </c>
     </row>
     <row r="55">
@@ -2901,13 +2901,13 @@
         <v>8</v>
       </c>
       <c r="G55" t="n">
-        <v>13262.78901618686</v>
+        <v>6199.711752674156</v>
       </c>
       <c r="H55" t="n">
-        <v>-107.0350012384318</v>
+        <v>-508.9590654024236</v>
       </c>
       <c r="I55" t="n">
-        <v>151.3080446463362</v>
+        <v>150.6592067094864</v>
       </c>
       <c r="J55" t="n">
         <v>0.5</v>
@@ -2916,10 +2916,10 @@
         <v>198.2950076925505</v>
       </c>
       <c r="L55" t="n">
-        <v>5003.71</v>
+        <v>2573.53</v>
       </c>
       <c r="M55" t="n">
-        <v>42.44</v>
+        <v>-80.78</v>
       </c>
     </row>
     <row r="56">
@@ -2946,25 +2946,25 @@
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>823.7746054435914</v>
+        <v>1087.007504540361</v>
       </c>
       <c r="H56" t="n">
-        <v>-583.5119701780576</v>
+        <v>-40.9939625188524</v>
       </c>
       <c r="I56" t="n">
-        <v>452.9251247505182</v>
+        <v>439.4669728658225</v>
       </c>
       <c r="J56" t="n">
         <v>0.5</v>
       </c>
       <c r="K56" t="n">
-        <v>467.3858153828035</v>
+        <v>428.3661755480705</v>
       </c>
       <c r="L56" t="n">
-        <v>643.62</v>
+        <v>858.59</v>
       </c>
       <c r="M56" t="n">
-        <v>-416.51</v>
+        <v>-19.39</v>
       </c>
     </row>
     <row r="57">
@@ -2991,25 +2991,25 @@
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>12128.19626930974</v>
+        <v>13088.04477629632</v>
       </c>
       <c r="H57" t="n">
-        <v>-211.5072626418036</v>
+        <v>-139.9776438493367</v>
       </c>
       <c r="I57" t="n">
-        <v>302.2262210398763</v>
+        <v>189.9034643156239</v>
       </c>
       <c r="J57" t="n">
         <v>0.5</v>
       </c>
       <c r="K57" t="n">
-        <v>323.8143915920092</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L57" t="n">
-        <v>8154.54</v>
+        <v>6144.83</v>
       </c>
       <c r="M57" t="n">
-        <v>-124.91</v>
+        <v>-8.02</v>
       </c>
     </row>
     <row r="58">
@@ -3036,25 +3036,25 @@
         <v>2</v>
       </c>
       <c r="G58" t="n">
-        <v>2384.81873079132</v>
+        <v>12144.6000732387</v>
       </c>
       <c r="H58" t="n">
-        <v>-99.56764172941988</v>
+        <v>-260.5642679194355</v>
       </c>
       <c r="I58" t="n">
-        <v>237.2796349484561</v>
+        <v>266.7162233146056</v>
       </c>
       <c r="J58" t="n">
         <v>0.5</v>
       </c>
       <c r="K58" t="n">
-        <v>238.320939301339</v>
+        <v>302.9006275609877</v>
       </c>
       <c r="L58" t="n">
-        <v>1445.85</v>
+        <v>7602.84</v>
       </c>
       <c r="M58" t="n">
-        <v>-11.3</v>
+        <v>-134.42</v>
       </c>
     </row>
     <row r="59">
@@ -3081,13 +3081,13 @@
         <v>3</v>
       </c>
       <c r="G59" t="n">
-        <v>1441.590703226053</v>
+        <v>1482.574580175288</v>
       </c>
       <c r="H59" t="n">
-        <v>-170.7985011689555</v>
+        <v>-101.4207793034801</v>
       </c>
       <c r="I59" t="n">
-        <v>189.9512157942106</v>
+        <v>192.1976071051158</v>
       </c>
       <c r="J59" t="n">
         <v>0.5</v>
@@ -3096,10 +3096,10 @@
         <v>198.2950076925505</v>
       </c>
       <c r="L59" t="n">
-        <v>771.22</v>
+        <v>811.1799999999999</v>
       </c>
       <c r="M59" t="n">
-        <v>-46.7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60">
@@ -3126,25 +3126,25 @@
         <v>4</v>
       </c>
       <c r="G60" t="n">
-        <v>784.1764014651656</v>
+        <v>1120.786951322453</v>
       </c>
       <c r="H60" t="n">
-        <v>-213.8743987226921</v>
+        <v>-111.5724788140298</v>
       </c>
       <c r="I60" t="n">
-        <v>266.8054258997851</v>
+        <v>259.7125702096749</v>
       </c>
       <c r="J60" t="n">
         <v>0.5</v>
       </c>
       <c r="K60" t="n">
-        <v>280.4314892296821</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L60" t="n">
-        <v>543.52</v>
+        <v>794.33</v>
       </c>
       <c r="M60" t="n">
-        <v>-84.09999999999999</v>
+        <v>-21.13</v>
       </c>
     </row>
     <row r="61">
@@ -3171,13 +3171,13 @@
         <v>5</v>
       </c>
       <c r="G61" t="n">
-        <v>7365.628978141092</v>
+        <v>7125.225883010933</v>
       </c>
       <c r="H61" t="n">
-        <v>-437.3384923420676</v>
+        <v>-463.3089974650201</v>
       </c>
       <c r="I61" t="n">
-        <v>196.3546132446432</v>
+        <v>186.9961833908445</v>
       </c>
       <c r="J61" t="n">
         <v>0.5</v>
@@ -3186,10 +3186,10 @@
         <v>238.320939301339</v>
       </c>
       <c r="L61" t="n">
-        <v>3505.61</v>
+        <v>3319.16</v>
       </c>
       <c r="M61" t="n">
-        <v>-145.92</v>
+        <v>-132.79</v>
       </c>
     </row>
     <row r="62">
@@ -3216,25 +3216,25 @@
         <v>6</v>
       </c>
       <c r="G62" t="n">
-        <v>730.0806779229506</v>
+        <v>2706.973814135334</v>
       </c>
       <c r="H62" t="n">
-        <v>-67.83386747945734</v>
+        <v>-230.7902408806186</v>
       </c>
       <c r="I62" t="n">
-        <v>323.974163527421</v>
+        <v>386.8914571696399</v>
       </c>
       <c r="J62" t="n">
         <v>0.5</v>
       </c>
       <c r="K62" t="n">
-        <v>330.4916794875841</v>
+        <v>391.0430286998269</v>
       </c>
       <c r="L62" t="n">
-        <v>408.85</v>
+        <v>2072.65</v>
       </c>
       <c r="M62" t="n">
-        <v>17.73</v>
+        <v>-160.4</v>
       </c>
     </row>
     <row r="63">
@@ -3261,25 +3261,25 @@
         <v>7</v>
       </c>
       <c r="G63" t="n">
-        <v>1175.958614839077</v>
+        <v>855.8943425645599</v>
       </c>
       <c r="H63" t="n">
-        <v>-574.9670053424455</v>
+        <v>-171.0115086530423</v>
       </c>
       <c r="I63" t="n">
-        <v>136.6952894672236</v>
+        <v>303.3849584363368</v>
       </c>
       <c r="J63" t="n">
         <v>0.5</v>
       </c>
       <c r="K63" t="n">
-        <v>147.8003722664622</v>
+        <v>330.4916794875841</v>
       </c>
       <c r="L63" t="n">
-        <v>401.6</v>
+        <v>611.85</v>
       </c>
       <c r="M63" t="n">
-        <v>-142.85</v>
+        <v>-76.48999999999999</v>
       </c>
     </row>
     <row r="64">
@@ -3306,25 +3306,25 @@
         <v>8</v>
       </c>
       <c r="G64" t="n">
-        <v>12529.89784759866</v>
+        <v>5371.316102758541</v>
       </c>
       <c r="H64" t="n">
-        <v>-118.5062473860355</v>
+        <v>-432.3876320737483</v>
       </c>
       <c r="I64" t="n">
-        <v>218.9482827942651</v>
+        <v>152.4302236915877</v>
       </c>
       <c r="J64" t="n">
         <v>0.5</v>
       </c>
       <c r="K64" t="n">
-        <v>255.9977541431066</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L64" t="n">
-        <v>6880.38</v>
+        <v>2894.24</v>
       </c>
       <c r="M64" t="n">
-        <v>-32.95</v>
+        <v>-188.31</v>
       </c>
     </row>
     <row r="65">
@@ -3351,25 +3351,25 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>818.7489539459112</v>
+        <v>1063.031104544045</v>
       </c>
       <c r="H65" t="n">
-        <v>-486.3406136600415</v>
+        <v>32.36245043005154</v>
       </c>
       <c r="I65" t="n">
-        <v>365.6313459358116</v>
+        <v>347.0000110683562</v>
       </c>
       <c r="J65" t="n">
         <v>0.5</v>
       </c>
       <c r="K65" t="n">
-        <v>355.9504322854629</v>
+        <v>343.4570282107588</v>
       </c>
       <c r="L65" t="n">
-        <v>465.57</v>
+        <v>789.83</v>
       </c>
       <c r="M65" t="n">
-        <v>-308.87</v>
+        <v>42.77</v>
       </c>
     </row>
     <row r="66">
@@ -3396,25 +3396,25 @@
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>11208.46299759916</v>
+        <v>12078.37833564107</v>
       </c>
       <c r="H66" t="n">
-        <v>-202.9104164836532</v>
+        <v>-100.863702585577</v>
       </c>
       <c r="I66" t="n">
-        <v>238.2564919616397</v>
+        <v>158.662235051113</v>
       </c>
       <c r="J66" t="n">
         <v>0.5</v>
       </c>
       <c r="K66" t="n">
-        <v>280.4314892296821</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L66" t="n">
-        <v>6991.86</v>
+        <v>4982.81</v>
       </c>
       <c r="M66" t="n">
-        <v>-73.22</v>
+        <v>17.15</v>
       </c>
     </row>
     <row r="67">
@@ -3441,25 +3441,25 @@
         <v>2</v>
       </c>
       <c r="G67" t="n">
-        <v>1658.189936353333</v>
+        <v>11217.96728615996</v>
       </c>
       <c r="H67" t="n">
-        <v>-106.4775954631906</v>
+        <v>-251.876875734282</v>
       </c>
       <c r="I67" t="n">
-        <v>329.3060083699041</v>
+        <v>214.4036933896692</v>
       </c>
       <c r="J67" t="n">
         <v>0.5</v>
       </c>
       <c r="K67" t="n">
-        <v>349.7595177200857</v>
+        <v>255.9977541431066</v>
       </c>
       <c r="L67" t="n">
-        <v>1189.2</v>
+        <v>6114.4</v>
       </c>
       <c r="M67" t="n">
-        <v>-35.97</v>
+        <v>-90.95999999999999</v>
       </c>
     </row>
     <row r="68">
@@ -3486,25 +3486,25 @@
         <v>3</v>
       </c>
       <c r="G68" t="n">
-        <v>1490.268035655453</v>
+        <v>1471.657351263134</v>
       </c>
       <c r="H68" t="n">
-        <v>-85.33500992719787</v>
+        <v>-111.1149111767326</v>
       </c>
       <c r="I68" t="n">
-        <v>201.2386351544646</v>
+        <v>200.2483052663786</v>
       </c>
       <c r="J68" t="n">
         <v>0.5</v>
       </c>
       <c r="K68" t="n">
-        <v>186.9543261531214</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L68" t="n">
-        <v>950.66</v>
+        <v>910.91</v>
       </c>
       <c r="M68" t="n">
-        <v>-5.48</v>
+        <v>23.18</v>
       </c>
     </row>
     <row r="69">
@@ -3531,25 +3531,25 @@
         <v>4</v>
       </c>
       <c r="G69" t="n">
-        <v>319.463847046663</v>
+        <v>1170.673508272454</v>
       </c>
       <c r="H69" t="n">
-        <v>-133.1115528354184</v>
+        <v>-119.2894980194102</v>
       </c>
       <c r="I69" t="n">
-        <v>207.5514995966694</v>
+        <v>345.3553591773253</v>
       </c>
       <c r="J69" t="n">
         <v>0.5</v>
       </c>
       <c r="K69" t="n">
-        <v>174.8797588600428</v>
+        <v>337.0367045574487</v>
       </c>
       <c r="L69" t="n">
-        <v>191.93</v>
+        <v>891.14</v>
       </c>
       <c r="M69" t="n">
-        <v>-17.51</v>
+        <v>-68.16</v>
       </c>
     </row>
     <row r="70">
@@ -3576,25 +3576,25 @@
         <v>5</v>
       </c>
       <c r="G70" t="n">
-        <v>6491.537042048481</v>
+        <v>6171.136880352984</v>
       </c>
       <c r="H70" t="n">
-        <v>-375.3696247864177</v>
+        <v>-370.8805170592382</v>
       </c>
       <c r="I70" t="n">
-        <v>275.3237063475563</v>
+        <v>195.7669930783102</v>
       </c>
       <c r="J70" t="n">
         <v>0.5</v>
       </c>
       <c r="K70" t="n">
-        <v>302.9006275609877</v>
+        <v>228.9713521405058</v>
       </c>
       <c r="L70" t="n">
-        <v>4191.27</v>
+        <v>3116.59</v>
       </c>
       <c r="M70" t="n">
-        <v>-189.92</v>
+        <v>-144.19</v>
       </c>
     </row>
     <row r="71">
@@ -3621,25 +3621,25 @@
         <v>6</v>
       </c>
       <c r="G71" t="n">
-        <v>751.1571321010358</v>
+        <v>1953.258713074089</v>
       </c>
       <c r="H71" t="n">
-        <v>13.30518684700617</v>
+        <v>-219.6540193296324</v>
       </c>
       <c r="I71" t="n">
-        <v>265.9975404529526</v>
+        <v>398.7787481693714</v>
       </c>
       <c r="J71" t="n">
         <v>0.5</v>
       </c>
       <c r="K71" t="n">
-        <v>228.9713521405058</v>
+        <v>391.0430286998269</v>
       </c>
       <c r="L71" t="n">
-        <v>550.63</v>
+        <v>1524.93</v>
       </c>
       <c r="M71" t="n">
-        <v>43.82</v>
+        <v>-161.45</v>
       </c>
     </row>
     <row r="72">
@@ -3666,25 +3666,25 @@
         <v>7</v>
       </c>
       <c r="G72" t="n">
-        <v>1247.235472100062</v>
+        <v>900.6380571745017</v>
       </c>
       <c r="H72" t="n">
-        <v>-470.9187130292537</v>
+        <v>-93.40022588136912</v>
       </c>
       <c r="I72" t="n">
-        <v>143.7400183170452</v>
+        <v>250.0738797828346</v>
       </c>
       <c r="J72" t="n">
         <v>0.5</v>
       </c>
       <c r="K72" t="n">
-        <v>186.9543261531214</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L72" t="n">
-        <v>513.8</v>
+        <v>603.61</v>
       </c>
       <c r="M72" t="n">
-        <v>-81.93000000000001</v>
+        <v>-47.85</v>
       </c>
     </row>
     <row r="73">
@@ -3711,25 +3711,25 @@
         <v>8</v>
       </c>
       <c r="G73" t="n">
-        <v>11773.75896009435</v>
+        <v>4511.663972151305</v>
       </c>
       <c r="H73" t="n">
-        <v>-129.6902847560621</v>
+        <v>-377.0119111133952</v>
       </c>
       <c r="I73" t="n">
-        <v>293.7241276398042</v>
+        <v>223.8643371247131</v>
       </c>
       <c r="J73" t="n">
         <v>0.5</v>
       </c>
       <c r="K73" t="n">
-        <v>337.0367045574487</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L73" t="n">
-        <v>7387.63</v>
+        <v>2664.06</v>
       </c>
       <c r="M73" t="n">
-        <v>-45.99</v>
+        <v>-168.88</v>
       </c>
     </row>
     <row r="74">
@@ -3756,25 +3756,25 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>816.7640532917177</v>
+        <v>968.9934130113459</v>
       </c>
       <c r="H74" t="n">
-        <v>-396.8970305161423</v>
+        <v>61.61468898666273</v>
       </c>
       <c r="I74" t="n">
-        <v>286.3293059780282</v>
+        <v>207.5807718673913</v>
       </c>
       <c r="J74" t="n">
         <v>0.5</v>
       </c>
       <c r="K74" t="n">
-        <v>316.996482935824</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L74" t="n">
-        <v>577.66</v>
+        <v>657.75</v>
       </c>
       <c r="M74" t="n">
-        <v>-176.49</v>
+        <v>92.98999999999999</v>
       </c>
     </row>
     <row r="75">
@@ -3801,25 +3801,25 @@
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>10315.92996728079</v>
+        <v>11142.63704714587</v>
       </c>
       <c r="H75" t="n">
-        <v>-193.8058669567699</v>
+        <v>-85.10494454141548</v>
       </c>
       <c r="I75" t="n">
-        <v>198.3088171349527</v>
+        <v>164.9221788181001</v>
       </c>
       <c r="J75" t="n">
         <v>0.5</v>
       </c>
       <c r="K75" t="n">
-        <v>247.317326764409</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L75" t="n">
-        <v>4919.24</v>
+        <v>4494.88</v>
       </c>
       <c r="M75" t="n">
-        <v>-15.02</v>
+        <v>49.82</v>
       </c>
     </row>
     <row r="76">
@@ -3846,25 +3846,25 @@
         <v>2</v>
       </c>
       <c r="G76" t="n">
-        <v>886.7159940299642</v>
+        <v>10332.09859762221</v>
       </c>
       <c r="H76" t="n">
-        <v>-113.8476671679928</v>
+        <v>-242.9486463885794</v>
       </c>
       <c r="I76" t="n">
-        <v>409.5604024279473</v>
+        <v>182.433463761614</v>
       </c>
       <c r="J76" t="n">
         <v>0.5</v>
       </c>
       <c r="K76" t="n">
-        <v>379.7060313951988</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L76" t="n">
-        <v>727.86</v>
+        <v>5017.75</v>
       </c>
       <c r="M76" t="n">
-        <v>-77.08</v>
+        <v>-42.36</v>
       </c>
     </row>
     <row r="77">
@@ -3891,25 +3891,25 @@
         <v>3</v>
       </c>
       <c r="G77" t="n">
-        <v>1477.954285552303</v>
+        <v>1436.083973909499</v>
       </c>
       <c r="H77" t="n">
-        <v>-16.75663061960482</v>
+        <v>-119.5249169031009</v>
       </c>
       <c r="I77" t="n">
-        <v>212.9416116612993</v>
+        <v>209.5574429532119</v>
       </c>
       <c r="J77" t="n">
         <v>0.5</v>
       </c>
       <c r="K77" t="n">
-        <v>219.2233794389425</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L77" t="n">
-        <v>890.99</v>
+        <v>885.9299999999999</v>
       </c>
       <c r="M77" t="n">
-        <v>47.79</v>
+        <v>-25.22</v>
       </c>
     </row>
     <row r="78">
@@ -3936,25 +3936,25 @@
         <v>4</v>
       </c>
       <c r="G78" t="n">
-        <v>242.7852657437815</v>
+        <v>1121.246691660897</v>
       </c>
       <c r="H78" t="n">
-        <v>-68.70923324113743</v>
+        <v>-122.6782237856445</v>
       </c>
       <c r="I78" t="n">
-        <v>180.2735873558817</v>
+        <v>442.2832804068054</v>
       </c>
       <c r="J78" t="n">
         <v>0.5</v>
       </c>
       <c r="K78" t="n">
-        <v>147.8003722664622</v>
+        <v>443.4011167993866</v>
       </c>
       <c r="L78" t="n">
-        <v>25.5</v>
+        <v>849.98</v>
       </c>
       <c r="M78" t="n">
-        <v>78.15000000000001</v>
+        <v>-84.29000000000001</v>
       </c>
     </row>
     <row r="79">
@@ -3981,25 +3981,25 @@
         <v>5</v>
       </c>
       <c r="G79" t="n">
-        <v>5620.831425210465</v>
+        <v>5223.707070049571</v>
       </c>
       <c r="H79" t="n">
-        <v>-307.567542712957</v>
+        <v>-284.8138118922661</v>
       </c>
       <c r="I79" t="n">
-        <v>332.4949242359778</v>
+        <v>203.4449707984895</v>
       </c>
       <c r="J79" t="n">
         <v>0.5</v>
       </c>
       <c r="K79" t="n">
-        <v>362.0354958462345</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L79" t="n">
-        <v>3925.8</v>
+        <v>2605.47</v>
       </c>
       <c r="M79" t="n">
-        <v>-181.45</v>
+        <v>-117.11</v>
       </c>
     </row>
     <row r="80">
@@ -4026,25 +4026,25 @@
         <v>6</v>
       </c>
       <c r="G80" t="n">
-        <v>806.618904117484</v>
+        <v>1300.915807883473</v>
       </c>
       <c r="H80" t="n">
-        <v>14.04905820615261</v>
+        <v>-207.4367289093574</v>
       </c>
       <c r="I80" t="n">
-        <v>201.2551056857135</v>
+        <v>347.075633424912</v>
       </c>
       <c r="J80" t="n">
         <v>0.5</v>
       </c>
       <c r="K80" t="n">
-        <v>238.320939301339</v>
+        <v>323.8143915920092</v>
       </c>
       <c r="L80" t="n">
-        <v>484.51</v>
+        <v>1012.5</v>
       </c>
       <c r="M80" t="n">
-        <v>55.75</v>
+        <v>-134.47</v>
       </c>
     </row>
     <row r="81">
@@ -4071,25 +4071,25 @@
         <v>7</v>
       </c>
       <c r="G81" t="n">
-        <v>1320.316003645021</v>
+        <v>968.7738570388838</v>
       </c>
       <c r="H81" t="n">
-        <v>-359.3403078337209</v>
+        <v>-33.07437837615773</v>
       </c>
       <c r="I81" t="n">
-        <v>150.9190682696963</v>
+        <v>192.9678344014511</v>
       </c>
       <c r="J81" t="n">
         <v>0.5</v>
       </c>
       <c r="K81" t="n">
-        <v>186.9543261531214</v>
+        <v>209.0212909830231</v>
       </c>
       <c r="L81" t="n">
-        <v>603.48</v>
+        <v>540.47</v>
       </c>
       <c r="M81" t="n">
-        <v>-56.08</v>
+        <v>23.48</v>
       </c>
     </row>
     <row r="82">
@@ -4116,25 +4116,25 @@
         <v>8</v>
       </c>
       <c r="G82" t="n">
-        <v>10845.18061696473</v>
+        <v>3713.581089249014</v>
       </c>
       <c r="H82" t="n">
-        <v>-132.2103748407683</v>
+        <v>-304.9725924997871</v>
       </c>
       <c r="I82" t="n">
-        <v>337.5811162484855</v>
+        <v>294.2463315417337</v>
       </c>
       <c r="J82" t="n">
         <v>0.5</v>
       </c>
       <c r="K82" t="n">
-        <v>368.0199590525625</v>
+        <v>302.9006275609877</v>
       </c>
       <c r="L82" t="n">
-        <v>7699.2</v>
+        <v>2603.28</v>
       </c>
       <c r="M82" t="n">
-        <v>-59.77</v>
+        <v>-180.55</v>
       </c>
     </row>
     <row r="83">
@@ -4161,25 +4161,25 @@
         <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>821.0094095015329</v>
+        <v>922.9407721339485</v>
       </c>
       <c r="H83" t="n">
-        <v>-314.4737157130965</v>
+        <v>33.56270100554859</v>
       </c>
       <c r="I83" t="n">
-        <v>230.1167372677171</v>
+        <v>140.6026986083124</v>
       </c>
       <c r="J83" t="n">
         <v>0.5</v>
       </c>
       <c r="K83" t="n">
-        <v>247.317326764409</v>
+        <v>174.8797588600428</v>
       </c>
       <c r="L83" t="n">
-        <v>288.38</v>
+        <v>350.75</v>
       </c>
       <c r="M83" t="n">
-        <v>-60.42</v>
+        <v>97.86</v>
       </c>
     </row>
     <row r="84">
@@ -4206,25 +4206,25 @@
         <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>9424.366600550547</v>
+        <v>10302.93216161453</v>
       </c>
       <c r="H84" t="n">
-        <v>-186.6688346955743</v>
+        <v>-94.90375323989382</v>
       </c>
       <c r="I84" t="n">
-        <v>176.7816210304546</v>
+        <v>204.1965397259627</v>
       </c>
       <c r="J84" t="n">
         <v>0.5</v>
       </c>
       <c r="K84" t="n">
-        <v>219.2233794389425</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L84" t="n">
-        <v>4464.87</v>
+        <v>5413.54</v>
       </c>
       <c r="M84" t="n">
-        <v>-13.99</v>
+        <v>3.28</v>
       </c>
     </row>
     <row r="85">
@@ -4251,25 +4251,25 @@
         <v>2</v>
       </c>
       <c r="G85" t="n">
-        <v>251.9262162017246</v>
+        <v>9479.09009957648</v>
       </c>
       <c r="H85" t="n">
-        <v>-91.6158237965068</v>
+        <v>-235.2627544396135</v>
       </c>
       <c r="I85" t="n">
-        <v>353.2153082206629</v>
+        <v>173.3982232155653</v>
       </c>
       <c r="J85" t="n">
         <v>0.5</v>
       </c>
       <c r="K85" t="n">
-        <v>264.3933435900673</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L85" t="n">
-        <v>-13.27</v>
+        <v>4285.14</v>
       </c>
       <c r="M85" t="n">
-        <v>87.08</v>
+        <v>-44.36</v>
       </c>
     </row>
     <row r="86">
@@ -4296,25 +4296,25 @@
         <v>3</v>
       </c>
       <c r="G86" t="n">
-        <v>1367.609086963569</v>
+        <v>1359.403843636258</v>
       </c>
       <c r="H86" t="n">
-        <v>-10.40511787042215</v>
+        <v>-128.8522447071974</v>
       </c>
       <c r="I86" t="n">
-        <v>225.3103954119474</v>
+        <v>217.1307799291167</v>
       </c>
       <c r="J86" t="n">
         <v>0.5</v>
       </c>
       <c r="K86" t="n">
-        <v>228.9713521405058</v>
+        <v>186.9543261531214</v>
       </c>
       <c r="L86" t="n">
-        <v>881.1799999999999</v>
+        <v>781.51</v>
       </c>
       <c r="M86" t="n">
-        <v>32.43</v>
+        <v>-85.63</v>
       </c>
     </row>
     <row r="87">
@@ -4341,25 +4341,25 @@
         <v>4</v>
       </c>
       <c r="G87" t="n">
-        <v>843.173184300985</v>
+        <v>1067.215863256521</v>
       </c>
       <c r="H87" t="n">
-        <v>-42.35362889704457</v>
+        <v>-116.5051186084018</v>
       </c>
       <c r="I87" t="n">
-        <v>262.2646910600982</v>
+        <v>436.5761056707952</v>
       </c>
       <c r="J87" t="n">
         <v>0.5</v>
       </c>
       <c r="K87" t="n">
-        <v>228.9713521405058</v>
+        <v>407.4575073795997</v>
       </c>
       <c r="L87" t="n">
-        <v>585.86</v>
+        <v>869.33</v>
       </c>
       <c r="M87" t="n">
-        <v>-4.8</v>
+        <v>-81.5</v>
       </c>
     </row>
     <row r="88">
@@ -4386,25 +4386,25 @@
         <v>5</v>
       </c>
       <c r="G88" t="n">
-        <v>4698.991489091691</v>
+        <v>4316.805537472999</v>
       </c>
       <c r="H88" t="n">
-        <v>-231.5252617430352</v>
+        <v>-195.2479000201368</v>
       </c>
       <c r="I88" t="n">
-        <v>336.9590265698472</v>
+        <v>211.7529156177933</v>
       </c>
       <c r="J88" t="n">
         <v>0.5</v>
       </c>
       <c r="K88" t="n">
-        <v>355.9504322854629</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L88" t="n">
-        <v>3310.05</v>
+        <v>2368.39</v>
       </c>
       <c r="M88" t="n">
-        <v>-131.8</v>
+        <v>-58.15</v>
       </c>
     </row>
     <row r="89">
@@ -4431,13 +4431,13 @@
         <v>6</v>
       </c>
       <c r="G89" t="n">
-        <v>847.4753349047522</v>
+        <v>784.9151027896288</v>
       </c>
       <c r="H89" t="n">
-        <v>-20.96975929029902</v>
+        <v>-195.1234692179626</v>
       </c>
       <c r="I89" t="n">
-        <v>222.6392387311265</v>
+        <v>273.4461122101758</v>
       </c>
       <c r="J89" t="n">
         <v>0.5</v>
@@ -4446,10 +4446,10 @@
         <v>209.0212909830231</v>
       </c>
       <c r="L89" t="n">
-        <v>512.3</v>
+        <v>552.41</v>
       </c>
       <c r="M89" t="n">
-        <v>49.23</v>
+        <v>-125.02</v>
       </c>
     </row>
     <row r="90">
@@ -4476,25 +4476,25 @@
         <v>7</v>
       </c>
       <c r="G90" t="n">
-        <v>1390.090753640867</v>
+        <v>1062.193033683856</v>
       </c>
       <c r="H90" t="n">
-        <v>-264.6526271373666</v>
+        <v>13.79825547116479</v>
       </c>
       <c r="I90" t="n">
-        <v>158.1147062953137</v>
+        <v>236.6070604910128</v>
       </c>
       <c r="J90" t="n">
         <v>0.5</v>
       </c>
       <c r="K90" t="n">
-        <v>209.0212909830231</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L90" t="n">
-        <v>612.12</v>
+        <v>707.48</v>
       </c>
       <c r="M90" t="n">
-        <v>-22.75</v>
+        <v>37.67</v>
       </c>
     </row>
     <row r="91">
@@ -4521,25 +4521,25 @@
         <v>8</v>
       </c>
       <c r="G91" t="n">
-        <v>9884.615649716707</v>
+        <v>2929.947548663882</v>
       </c>
       <c r="H91" t="n">
-        <v>-131.0861663068135</v>
+        <v>-232.3181957914322</v>
       </c>
       <c r="I91" t="n">
-        <v>313.6707438378427</v>
+        <v>349.5339280878322</v>
       </c>
       <c r="J91" t="n">
         <v>0.5</v>
       </c>
       <c r="K91" t="n">
-        <v>337.0367045574487</v>
+        <v>355.9504322854629</v>
       </c>
       <c r="L91" t="n">
-        <v>6845.78</v>
+        <v>2123.65</v>
       </c>
       <c r="M91" t="n">
-        <v>-49.65</v>
+        <v>-153.29</v>
       </c>
     </row>
     <row r="92">
@@ -4566,25 +4566,25 @@
         <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>826.4930828588435</v>
+        <v>923.449268779954</v>
       </c>
       <c r="H92" t="n">
-        <v>-243.998280895391</v>
+        <v>-30.00245015128791</v>
       </c>
       <c r="I92" t="n">
-        <v>186.5681578794358</v>
+        <v>133.0242383017033</v>
       </c>
       <c r="J92" t="n">
         <v>0.5</v>
       </c>
       <c r="K92" t="n">
-        <v>132.1966717950337</v>
+        <v>147.8003722664622</v>
       </c>
       <c r="L92" t="n">
-        <v>458.33</v>
+        <v>414.62</v>
       </c>
       <c r="M92" t="n">
-        <v>-120.26</v>
+        <v>102.58</v>
       </c>
     </row>
     <row r="93">
@@ -4611,25 +4611,25 @@
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>8575.481353782689</v>
+        <v>9538.161583812711</v>
       </c>
       <c r="H93" t="n">
-        <v>-184.1518087039896</v>
+        <v>-134.3783285438634</v>
       </c>
       <c r="I93" t="n">
-        <v>178.7833690185174</v>
+        <v>249.9683527606536</v>
       </c>
       <c r="J93" t="n">
         <v>0.5</v>
       </c>
       <c r="K93" t="n">
-        <v>228.9713521405058</v>
+        <v>288.1159665134826</v>
       </c>
       <c r="L93" t="n">
-        <v>3865.53</v>
+        <v>5551.93</v>
       </c>
       <c r="M93" t="n">
-        <v>23.65</v>
+        <v>-20.92</v>
       </c>
     </row>
     <row r="94">
@@ -4656,25 +4656,25 @@
         <v>2</v>
       </c>
       <c r="G94" t="n">
-        <v>-30.04072426406509</v>
+        <v>8631.9082374429</v>
       </c>
       <c r="H94" t="n">
-        <v>-25.77923704665935</v>
+        <v>-230.2874817045138</v>
       </c>
       <c r="I94" t="n">
-        <v>269.8827281243955</v>
+        <v>194.0909016713987</v>
       </c>
       <c r="J94" t="n">
         <v>0.5</v>
       </c>
       <c r="K94" t="n">
-        <v>323.8143915920092</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L94" t="n">
-        <v>-24.9</v>
+        <v>5314.6</v>
       </c>
       <c r="M94" t="n">
-        <v>42.83</v>
+        <v>-93.61</v>
       </c>
     </row>
     <row r="95">
@@ -4701,25 +4701,25 @@
         <v>3</v>
       </c>
       <c r="G95" t="n">
-        <v>1292.018921704342</v>
+        <v>1244.711080688445</v>
       </c>
       <c r="H95" t="n">
-        <v>-62.31087824737482</v>
+        <v>-131.3321067350291</v>
       </c>
       <c r="I95" t="n">
-        <v>233.4158168795942</v>
+        <v>229.0688340889325</v>
       </c>
       <c r="J95" t="n">
         <v>0.5</v>
       </c>
       <c r="K95" t="n">
-        <v>228.9713521405058</v>
+        <v>219.2233794389425</v>
       </c>
       <c r="L95" t="n">
-        <v>837.4299999999999</v>
+        <v>851.88</v>
       </c>
       <c r="M95" t="n">
-        <v>-1.65</v>
+        <v>-54.43</v>
       </c>
     </row>
     <row r="96">
@@ -4746,25 +4746,25 @@
         <v>4</v>
       </c>
       <c r="G96" t="n">
-        <v>1389.740183847462</v>
+        <v>1019.758893899933</v>
       </c>
       <c r="H96" t="n">
-        <v>-65.2318865221127</v>
+        <v>-107.4497988047731</v>
       </c>
       <c r="I96" t="n">
-        <v>332.4624970133045</v>
+        <v>360.8607033132749</v>
       </c>
       <c r="J96" t="n">
         <v>0.5</v>
       </c>
       <c r="K96" t="n">
-        <v>323.8143915920092</v>
+        <v>349.7595177200857</v>
       </c>
       <c r="L96" t="n">
-        <v>1039.1</v>
+        <v>759.17</v>
       </c>
       <c r="M96" t="n">
-        <v>-17.83</v>
+        <v>-50.3</v>
       </c>
     </row>
     <row r="97">
@@ -4791,25 +4791,25 @@
         <v>5</v>
       </c>
       <c r="G97" t="n">
-        <v>3789.688206014015</v>
+        <v>3460.460865829757</v>
       </c>
       <c r="H97" t="n">
-        <v>-153.7511288858043</v>
+        <v>-110.3226041441847</v>
       </c>
       <c r="I97" t="n">
-        <v>280.4378759920298</v>
+        <v>219.8096555602745</v>
       </c>
       <c r="J97" t="n">
         <v>0.5</v>
       </c>
       <c r="K97" t="n">
-        <v>288.1159665134826</v>
+        <v>238.320939301339</v>
       </c>
       <c r="L97" t="n">
-        <v>2590.76</v>
+        <v>1971.82</v>
       </c>
       <c r="M97" t="n">
-        <v>-62.01</v>
+        <v>15.06</v>
       </c>
     </row>
     <row r="98">
@@ -4836,25 +4836,25 @@
         <v>6</v>
       </c>
       <c r="G98" t="n">
-        <v>897.6241205430479</v>
+        <v>437.0261564957461</v>
       </c>
       <c r="H98" t="n">
-        <v>-77.97791948380879</v>
+        <v>-183.3151258207566</v>
       </c>
       <c r="I98" t="n">
-        <v>253.791505850277</v>
+        <v>220.3377926433836</v>
       </c>
       <c r="J98" t="n">
         <v>0.5</v>
       </c>
       <c r="K98" t="n">
-        <v>209.0212909830231</v>
+        <v>161.9071957960046</v>
       </c>
       <c r="L98" t="n">
-        <v>391.67</v>
+        <v>117.2</v>
       </c>
       <c r="M98" t="n">
-        <v>13.52</v>
+        <v>32.56</v>
       </c>
     </row>
     <row r="99">
@@ -4881,25 +4881,25 @@
         <v>7</v>
       </c>
       <c r="G99" t="n">
-        <v>1450.067170507529</v>
+        <v>1170.145811452183</v>
       </c>
       <c r="H99" t="n">
-        <v>-183.3673764041169</v>
+        <v>8.806991004904162</v>
       </c>
       <c r="I99" t="n">
-        <v>166.4951427877066</v>
+        <v>286.2684391407417</v>
       </c>
       <c r="J99" t="n">
         <v>0.5</v>
       </c>
       <c r="K99" t="n">
-        <v>198.2950076925505</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L99" t="n">
-        <v>666.95</v>
+        <v>846.98</v>
       </c>
       <c r="M99" t="n">
-        <v>-15.68</v>
+        <v>44.54</v>
       </c>
     </row>
     <row r="100">
@@ -4926,25 +4926,25 @@
         <v>8</v>
       </c>
       <c r="G100" t="n">
-        <v>8910.642062467716</v>
+        <v>2159.629628539082</v>
       </c>
       <c r="H100" t="n">
-        <v>-126.5533634414246</v>
+        <v>-155.0478468080535</v>
       </c>
       <c r="I100" t="n">
-        <v>252.0964037627788</v>
+        <v>353.5317432120739</v>
       </c>
       <c r="J100" t="n">
         <v>0.5</v>
       </c>
       <c r="K100" t="n">
-        <v>288.1159665134826</v>
+        <v>368.0199590525625</v>
       </c>
       <c r="L100" t="n">
-        <v>5335.98</v>
+        <v>1580.06</v>
       </c>
       <c r="M100" t="n">
-        <v>-26.28</v>
+        <v>-79.31</v>
       </c>
     </row>
   </sheetData>
@@ -5025,7 +5025,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -5041,36 +5041,36 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G2" t="n">
-        <v>1390.090753640867</v>
+        <v>1120.786951322453</v>
       </c>
       <c r="H2" t="n">
-        <v>-264.6526271373666</v>
+        <v>-111.5724788140298</v>
       </c>
       <c r="I2" t="n">
-        <v>158.1147062953137</v>
+        <v>259.7125702096749</v>
       </c>
       <c r="J2" t="n">
         <v>0.5</v>
       </c>
       <c r="K2" t="n">
-        <v>209.0212909830231</v>
+        <v>247.317326764409</v>
       </c>
       <c r="L2" t="n">
-        <v>612.12</v>
+        <v>794.33</v>
       </c>
       <c r="M2" t="n">
-        <v>-22.75</v>
+        <v>-21.13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>97</v>
+        <v>22</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -5086,36 +5086,36 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>1450.067170507529</v>
+        <v>1104.526796348649</v>
       </c>
       <c r="H3" t="n">
-        <v>-183.3673764041169</v>
+        <v>-100.0000175501522</v>
       </c>
       <c r="I3" t="n">
-        <v>166.4951427877066</v>
+        <v>250.340905115194</v>
       </c>
       <c r="J3" t="n">
         <v>0.5</v>
       </c>
       <c r="K3" t="n">
-        <v>198.2950076925505</v>
+        <v>264.3933435900673</v>
       </c>
       <c r="L3" t="n">
-        <v>666.95</v>
+        <v>722.45</v>
       </c>
       <c r="M3" t="n">
-        <v>-15.68</v>
+        <v>-9.039999999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -5131,31 +5131,31 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>1389.740183847462</v>
+        <v>1436.083973909499</v>
       </c>
       <c r="H4" t="n">
-        <v>-65.2318865221127</v>
+        <v>-119.5249169031009</v>
       </c>
       <c r="I4" t="n">
-        <v>332.4624970133045</v>
+        <v>209.5574429532119</v>
       </c>
       <c r="J4" t="n">
         <v>0.5</v>
       </c>
       <c r="K4" t="n">
-        <v>323.8143915920092</v>
+        <v>198.2950076925505</v>
       </c>
       <c r="L4" t="n">
-        <v>1039.1</v>
+        <v>885.9299999999999</v>
       </c>
       <c r="M4" t="n">
-        <v>-17.83</v>
+        <v>-25.22</v>
       </c>
     </row>
   </sheetData>
@@ -5268,31 +5268,31 @@
         <v>-21.42555</v>
       </c>
       <c r="G2" t="n">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="H2" t="n">
-        <v>98</v>
+        <v>26</v>
       </c>
       <c r="I2" t="n">
-        <v>1409</v>
+        <v>1220</v>
       </c>
       <c r="J2" t="n">
-        <v>34</v>
+        <v>186</v>
       </c>
       <c r="K2" t="n">
-        <v>-171</v>
+        <v>-110</v>
       </c>
       <c r="L2" t="n">
-        <v>34</v>
+        <v>186</v>
       </c>
       <c r="M2" t="n">
-        <v>-28.04</v>
+        <v>-16.91</v>
       </c>
       <c r="N2" t="n">
-        <v>48.47473758575618</v>
+        <v>40.47447817116304</v>
       </c>
       <c r="O2" t="n">
-        <v>87.47658776433622</v>
+        <v>80.58678581456877</v>
       </c>
     </row>
   </sheetData>

</xml_diff>